<commit_message>
Update pilot deck and finmodels for shortlist of 9 and approved pilots
Deck (29 slides): new shortlist slide with 9 objects, dual areas
(greenery vs total x2), approved pilots highlighted; pilot cards and
T1-T3 finmodel slides rebuilt around Skver Avenue 5, Headliner
Exclusive alley and the Flora 1+2 cluster.

Workbook v3: dual-area model (greenery from registry, total = greenery
x editable coefficient), cleaning/lighting rates rebased to total area,
object directory with 9-object shortlist and pilot defaults, T4 Sphere
Park sheet, summary recalculated for pilot objects.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014o1yT6nCgffZ5H25q7THst
</commit_message>
<xml_diff>
--- a/docs/research/BIG-Life-finmodels-T1-T4.xlsx
+++ b/docs/research/BIG-Life-finmodels-T1-T4.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нормативы" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т1 Транзитная" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т2 Активная" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т3 Плейхаб" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т3 Сквер" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т4 Sphere Park" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.#"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +57,35 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00008000"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B2A6E"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7A45"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00B03A2E"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
       <sz val="9.5"/>
     </font>
     <font>
@@ -211,11 +238,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -224,23 +251,23 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -250,56 +277,72 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -665,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -692,7 +735,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории) — площадь подтянется сама. Расходная часть считается формулами «площадь × норматив»: ставки правятся на листе «Нормативы» и меняют все модели разом. Жёлтые ячейки с синим шрифтом — редактируемые; остальное — формулы.</t>
+          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая = озеленение × коэффициент (лист «Нормативы», по умолчанию ×2). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Жёлтые ячейки — редактируемые ставки.</t>
         </is>
       </c>
     </row>
@@ -706,17 +749,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Т1 · Транзитная</t>
+          <t>Т1 · Flora 1+2</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Т2 · Активная</t>
+          <t>Т2 · Хедлайнер Экс.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Т3 · Плейхаб</t>
+          <t>Т3 · Авеню 5</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -740,7 +783,7 @@
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>'Т3 Плейхаб'!B3</f>
+        <f>'Т3 Сквер'!B3</f>
         <v/>
       </c>
       <c r="E9" s="7">
@@ -751,7 +794,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Площадь, м²</t>
+          <t>Озеленение, м²</t>
         </is>
       </c>
       <c r="B10" s="8">
@@ -763,7 +806,7 @@
         <v/>
       </c>
       <c r="D10" s="8">
-        <f>'Т3 Плейхаб'!D3</f>
+        <f>'Т3 Сквер'!D3</f>
         <v/>
       </c>
       <c r="E10" s="8">
@@ -774,204 +817,227 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Доходы, млн тг/год (мин)</t>
-        </is>
-      </c>
-      <c r="B11" s="9">
-        <f>'Т1 Транзитная'!C10</f>
-        <v/>
-      </c>
-      <c r="C11" s="9">
-        <f>'Т2 Активная'!C12</f>
-        <v/>
-      </c>
-      <c r="D11" s="9">
-        <f>'Т3 Плейхаб'!C12</f>
-        <v/>
-      </c>
-      <c r="E11" s="9">
-        <f>'Т4 Sphere Park'!C13</f>
+          <t>Общая площадь, м²</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>'Т1 Транзитная'!D4</f>
+        <v/>
+      </c>
+      <c r="C11" s="8">
+        <f>'Т2 Активная'!D4</f>
+        <v/>
+      </c>
+      <c r="D11" s="8">
+        <f>'Т3 Сквер'!D4</f>
+        <v/>
+      </c>
+      <c r="E11" s="8">
+        <f>'Т4 Sphere Park'!D4</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Доходы, млн тг/год (макс)</t>
+          <t>Доходы, млн тг/год (мин)</t>
         </is>
       </c>
       <c r="B12" s="9">
-        <f>'Т1 Транзитная'!D10</f>
+        <f>'Т1 Транзитная'!C11</f>
         <v/>
       </c>
       <c r="C12" s="9">
-        <f>'Т2 Активная'!D12</f>
+        <f>'Т2 Активная'!C13</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>'Т3 Плейхаб'!D12</f>
+        <f>'Т3 Сквер'!C13</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>'Т4 Sphere Park'!D13</f>
+        <f>'Т4 Sphere Park'!C14</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>OPEX, млн тг/год (мин)</t>
+          <t>Доходы, млн тг/год (макс)</t>
         </is>
       </c>
       <c r="B13" s="9">
-        <f>'Т1 Транзитная'!C17</f>
+        <f>'Т1 Транзитная'!D11</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>'Т2 Активная'!C20</f>
+        <f>'Т2 Активная'!D13</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>'Т3 Плейхаб'!C21</f>
+        <f>'Т3 Сквер'!D13</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>'Т4 Sphere Park'!C22</f>
+        <f>'Т4 Sphere Park'!D14</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>OPEX, млн тг/год (макс)</t>
+          <t>OPEX, млн тг/год (мин)</t>
         </is>
       </c>
       <c r="B14" s="9">
-        <f>'Т1 Транзитная'!D17</f>
+        <f>'Т1 Транзитная'!C18</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>'Т2 Активная'!D20</f>
+        <f>'Т2 Активная'!C21</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>'Т3 Плейхаб'!D21</f>
+        <f>'Т3 Сквер'!C22</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>'Т4 Sphere Park'!D22</f>
+        <f>'Т4 Sphere Park'!C23</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Покрытие OPEX, консервативно</t>
-        </is>
-      </c>
-      <c r="B15" s="10">
-        <f>IFERROR('Т1 Транзитная'!C10/'Т1 Транзитная'!D17,0)</f>
-        <v/>
-      </c>
-      <c r="C15" s="10">
-        <f>IFERROR('Т2 Активная'!C12/'Т2 Активная'!D20,0)</f>
-        <v/>
-      </c>
-      <c r="D15" s="10">
-        <f>IFERROR('Т3 Плейхаб'!C12/'Т3 Плейхаб'!D21,0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="10">
-        <f>IFERROR('Т4 Sphere Park'!C13/'Т4 Sphere Park'!D22,0)</f>
+          <t>OPEX, млн тг/год (макс)</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>'Т1 Транзитная'!D18</f>
+        <v/>
+      </c>
+      <c r="C15" s="9">
+        <f>'Т2 Активная'!D21</f>
+        <v/>
+      </c>
+      <c r="D15" s="9">
+        <f>'Т3 Сквер'!D22</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>'Т4 Sphere Park'!D23</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Покрытие OPEX, по середине вилок</t>
+          <t>Покрытие OPEX, консервативно</t>
         </is>
       </c>
       <c r="B16" s="10">
-        <f>IFERROR(AVERAGE('Т1 Транзитная'!C10:D10)/AVERAGE('Т1 Транзитная'!C17:D17),0)</f>
+        <f>IFERROR('Т1 Транзитная'!C11/'Т1 Транзитная'!D18,0)</f>
         <v/>
       </c>
       <c r="C16" s="10">
-        <f>IFERROR(AVERAGE('Т2 Активная'!C12:D12)/AVERAGE('Т2 Активная'!C20:D20),0)</f>
+        <f>IFERROR('Т2 Активная'!C13/'Т2 Активная'!D21,0)</f>
         <v/>
       </c>
       <c r="D16" s="10">
-        <f>IFERROR(AVERAGE('Т3 Плейхаб'!C12:D12)/AVERAGE('Т3 Плейхаб'!C21:D21),0)</f>
+        <f>IFERROR('Т3 Сквер'!C13/'Т3 Сквер'!D22,0)</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>IFERROR(AVERAGE('Т4 Sphere Park'!C13:D13)/AVERAGE('Т4 Sphere Park'!C22:D22),0)</f>
+        <f>IFERROR('Т4 Sphere Park'!C14/'Т4 Sphere Park'!D23,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Покрытие OPEX, оптимистично</t>
+          <t>Покрытие OPEX, по середине вилок</t>
         </is>
       </c>
       <c r="B17" s="10">
-        <f>IFERROR('Т1 Транзитная'!D10/'Т1 Транзитная'!C17,0)</f>
+        <f>IFERROR(AVERAGE('Т1 Транзитная'!C11:D11)/AVERAGE('Т1 Транзитная'!C18:D18),0)</f>
         <v/>
       </c>
       <c r="C17" s="10">
-        <f>IFERROR('Т2 Активная'!D12/'Т2 Активная'!C20,0)</f>
+        <f>IFERROR(AVERAGE('Т2 Активная'!C13:D13)/AVERAGE('Т2 Активная'!C21:D21),0)</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>IFERROR('Т3 Плейхаб'!D12/'Т3 Плейхаб'!C21,0)</f>
+        <f>IFERROR(AVERAGE('Т3 Сквер'!C13:D13)/AVERAGE('Т3 Сквер'!C22:D22),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR('Т4 Sphere Park'!D13/'Т4 Sphere Park'!C22,0)</f>
+        <f>IFERROR(AVERAGE('Т4 Sphere Park'!C14:D14)/AVERAGE('Т4 Sphere Park'!C23:D23),0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
+          <t>Покрытие OPEX, оптимистично</t>
+        </is>
+      </c>
+      <c r="B18" s="10">
+        <f>IFERROR('Т1 Транзитная'!D11/'Т1 Транзитная'!C18,0)</f>
+        <v/>
+      </c>
+      <c r="C18" s="10">
+        <f>IFERROR('Т2 Активная'!D13/'Т2 Активная'!C21,0)</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>IFERROR('Т3 Сквер'!D13/'Т3 Сквер'!C22,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>IFERROR('Т4 Sphere Park'!D14/'Т4 Sphere Park'!C23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>40–70%</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>70–100%</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026. CAPEX Sphere Park (~2,2 млрд тг, BTO) компенсируется бюджетом отдельно и в операционные модели не входит.</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
+    <row r="22"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A20:E21"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A21:E22"/>
     <mergeCell ref="A4:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -984,15 +1050,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1005,7 +1073,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Группы: A — обслуживает BI Green · B — переданы 29.07–03.08.2026 · C — не обслуживаются · D — переданы городу. Тип: предложение для финмодели.</t>
+          <t>Группы: A — обслуживает BI Green · B — переданы 29.07–03.08.2026 · C — не обслуживаются · D — переданы городу. Площадь реестра — зелёные насаждения; общая = озеленение × коэффициент (лист «Нормативы»).</t>
         </is>
       </c>
     </row>
@@ -1032,10 +1100,20 @@
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>Площадь, м²</t>
+          <t>Озеленение, м²</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Общая, м²</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Шорт-лист</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
         <is>
           <t>Статус / примечание</t>
         </is>
@@ -1063,7 +1141,16 @@
       <c r="E4" s="17" t="n">
         <v>2500</v>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="18">
+        <f>E4*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1073,7 +1160,7 @@
       <c r="A5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
@@ -1091,7 +1178,16 @@
       <c r="E5" s="17" t="n">
         <v>1700</v>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="18">
+        <f>E5*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G5" s="21" t="inlineStr">
+        <is>
+          <t>Пилот</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1119,7 +1215,16 @@
       <c r="E6" s="17" t="n">
         <v>1600</v>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="18">
+        <f>E6*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1147,7 +1252,16 @@
       <c r="E7" s="17" t="n">
         <v>6200</v>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="18">
+        <f>E7*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1175,7 +1289,16 @@
       <c r="E8" s="17" t="n">
         <v>800</v>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="18">
+        <f>E8*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1185,7 +1308,7 @@
       <c r="A9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
@@ -1203,7 +1326,16 @@
       <c r="E9" s="17" t="n">
         <v>4000</v>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="18">
+        <f>E9*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G9" s="21" t="inlineStr">
+        <is>
+          <t>Пилот</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1231,7 +1363,16 @@
       <c r="E10" s="17" t="n">
         <v>2300</v>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="18">
+        <f>E10*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1241,7 +1382,7 @@
       <c r="A11" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 1</t>
         </is>
@@ -1259,7 +1400,16 @@
       <c r="E11" s="17" t="n">
         <v>338</v>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="18">
+        <f>E11*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>Пилот</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1269,7 +1419,7 @@
       <c r="A12" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 2</t>
         </is>
@@ -1287,7 +1437,16 @@
       <c r="E12" s="17" t="n">
         <v>338</v>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="18">
+        <f>E12*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>Пилот</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
@@ -1309,15 +1468,24 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>Т3</t>
+          <t>Т2</t>
         </is>
       </c>
       <c r="E13" s="17" t="n">
         <v>2385</v>
       </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>не передан, обслуживает BI Green</t>
+      <c r="F13" s="18">
+        <f>E13*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>не передан, обслуживает BI Green; плейхаб, в шорт-листе как активная</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1511,16 @@
       <c r="E14" s="17" t="n">
         <v>6800</v>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="18">
+        <f>E14*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>передан 29.07.2026</t>
         </is>
@@ -1371,7 +1548,16 @@
       <c r="E15" s="17" t="n">
         <v>2930</v>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="18">
+        <f>E15*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>передан 03.08.2026</t>
         </is>
@@ -1399,7 +1585,16 @@
       <c r="E16" s="17" t="n">
         <v>3650</v>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="18">
+        <f>E16*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>передан 03.08.2026, придомовая</t>
         </is>
@@ -1427,7 +1622,16 @@
       <c r="E17" s="17" t="n">
         <v>1680</v>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="18">
+        <f>E17*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>передан 03.08.2026, есть спортплощадка</t>
         </is>
@@ -1455,7 +1659,16 @@
       <c r="E18" s="17" t="n">
         <v>1680</v>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F18" s="18">
+        <f>E18*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>передан 03.08.2026</t>
         </is>
@@ -1483,7 +1696,16 @@
       <c r="E19" s="17" t="n">
         <v>3500</v>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F19" s="18">
+        <f>E19*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>передан 03.08.2026</t>
         </is>
@@ -1511,7 +1733,16 @@
       <c r="E20" s="17" t="n">
         <v>4000</v>
       </c>
-      <c r="F20" s="16" t="inlineStr">
+      <c r="F20" s="18">
+        <f>E20*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>передан 03.08.2026, аллея-парк</t>
         </is>
@@ -1526,7 +1757,7 @@
           <t>Аллея Nexpo Юнион</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1539,7 +1770,16 @@
       <c r="E21" s="17" t="n">
         <v>2419</v>
       </c>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="F21" s="18">
+        <f>E21*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
         </is>
@@ -1554,7 +1794,7 @@
           <t>Фридом — Зелёный Квартал</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1567,7 +1807,16 @@
       <c r="E22" s="17" t="n">
         <v>3600</v>
       </c>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="F22" s="18">
+        <f>E22*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>парковка, вне типологии; уточнить юраудитом</t>
         </is>
@@ -1582,7 +1831,7 @@
           <t>Де Люкс 4</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1595,7 +1844,16 @@
       <c r="E23" s="17" t="n">
         <v>4200</v>
       </c>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="F23" s="18">
+        <f>E23*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
         </is>
@@ -1610,7 +1868,7 @@
           <t>Насаждения ЖК Айтыс</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1623,7 +1881,16 @@
       <c r="E24" s="17" t="n">
         <v>300</v>
       </c>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="F24" s="18">
+        <f>E24*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается, придомовая</t>
         </is>
@@ -1638,7 +1905,7 @@
           <t>Парк Авеню Эксклюзив</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1651,7 +1918,16 @@
       <c r="E25" s="17" t="n">
         <v>680</v>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F25" s="18">
+        <f>E25*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
         </is>
@@ -1666,7 +1942,7 @@
           <t>Аллея Онли Мун</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1679,7 +1955,16 @@
       <c r="E26" s="17" t="n">
         <v>600</v>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F26" s="18">
+        <f>E26*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
         </is>
@@ -1694,7 +1979,7 @@
           <t>Аллея Сердце Столицы 1, 2</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1707,7 +1992,16 @@
       <c r="E27" s="17" t="n">
         <v>1300</v>
       </c>
-      <c r="F27" s="16" t="inlineStr">
+      <c r="F27" s="18">
+        <f>E27*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается, придомовая</t>
         </is>
@@ -1735,7 +2029,16 @@
       <c r="E28" s="17" t="n">
         <v>1120</v>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F28" s="18">
+        <f>E28*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>передан городу</t>
         </is>
@@ -1763,7 +2066,16 @@
       <c r="E29" s="17" t="n">
         <v>3900</v>
       </c>
-      <c r="F29" s="16" t="inlineStr">
+      <c r="F29" s="18">
+        <f>E29*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
         <is>
           <t>передан городу</t>
         </is>
@@ -1791,7 +2103,16 @@
       <c r="E30" s="17" t="n">
         <v>2900</v>
       </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F30" s="18">
+        <f>E30*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G30" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
         <is>
           <t>передан городу</t>
         </is>
@@ -1819,7 +2140,16 @@
       <c r="E31" s="17" t="n">
         <v>17000</v>
       </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="F31" s="18">
+        <f>E31*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
         <is>
           <t>передан городу, кандидат на ГЧП</t>
         </is>
@@ -1847,7 +2177,16 @@
       <c r="E32" s="17" t="n">
         <v>3100</v>
       </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F32" s="18">
+        <f>E32*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
         <is>
           <t>передан городу</t>
         </is>
@@ -1875,7 +2214,16 @@
       <c r="E33" s="17" t="n">
         <v>5500</v>
       </c>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F33" s="18">
+        <f>E33*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
         <is>
           <t>передан городу</t>
         </is>
@@ -1903,7 +2251,16 @@
       <c r="E34" s="17" t="n">
         <v>1100</v>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F34" s="18">
+        <f>E34*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="inlineStr">
         <is>
           <t>передан городу</t>
         </is>
@@ -1931,16 +2288,61 @@
       <c r="E35" s="17" t="n">
         <v>70000</v>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F35" s="24" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
         <is>
           <t>проект ГЧП (BTO): парк 7 га + озеро 2 га у школы BINOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="20" t="inlineStr">
+        <is>
+          <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Т1</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="n">
+        <v>676</v>
+      </c>
+      <c r="F36" s="18">
+        <f>E36*Нормативы!$C$17</f>
+        <v/>
+      </c>
+      <c r="G36" s="21" t="inlineStr">
+        <is>
+          <t>Пилот</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>пилот Т1: два объекта под одной командой</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1952,7 +2354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1982,52 +2384,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Т1 мин</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>Т1 макс</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>Т2 мин</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="25" t="inlineStr">
         <is>
           <t>Т2 макс</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="25" t="inlineStr">
         <is>
           <t>Т3 мин</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="25" t="inlineStr">
         <is>
           <t>Т3 макс</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="25" t="inlineStr">
         <is>
           <t>Т4 мин</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="25" t="inlineStr">
         <is>
           <t>Т4 макс</t>
         </is>
@@ -2039,34 +2441,34 @@
           <t>Уборка и снегоуборка</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>тг/м² в месяц</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>120</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>175</v>
-      </c>
-      <c r="E5" s="21" t="n">
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>тг/м² общей пл. в месяц</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="n">
         <v>60</v>
       </c>
-      <c r="F5" s="21" t="n">
-        <v>110</v>
-      </c>
-      <c r="G5" s="21" t="n">
-        <v>120</v>
-      </c>
-      <c r="H5" s="21" t="n">
-        <v>200</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>40</v>
-      </c>
-      <c r="J5" s="21" t="n">
-        <v>80</v>
+      <c r="D5" s="27" t="n">
+        <v>90</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>55</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>60</v>
+      </c>
+      <c r="H5" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="J5" s="27" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -2075,33 +2477,33 @@
           <t>Озеленение и полив (апр–окт)</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>тг/м² в месяц</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="n">
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>тг/м² озеленения в месяц</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="n">
         <v>90</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="27" t="n">
         <v>160</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="27" t="n">
         <v>70</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="27" t="n">
         <v>55</v>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="27" t="n">
         <v>90</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="27" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2111,34 +2513,34 @@
           <t>Свет, электро, digital</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>тг/м² в год</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="n">
-        <v>310</v>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>500</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>130</v>
-      </c>
-      <c r="F7" s="21" t="n">
-        <v>225</v>
-      </c>
-      <c r="G7" s="21" t="n">
-        <v>380</v>
-      </c>
-      <c r="H7" s="21" t="n">
-        <v>630</v>
-      </c>
-      <c r="I7" s="21" t="n">
-        <v>100</v>
-      </c>
-      <c r="J7" s="21" t="n">
-        <v>200</v>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>тг/м² общей пл. в год</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>155</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>250</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>65</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>115</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>190</v>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>315</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>80</v>
+      </c>
+      <c r="J7" s="27" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="8">
@@ -2147,33 +2549,33 @@
           <t>Доля ставки координатора</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>доля ставки</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="28" t="n">
         <v>0.2</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="28" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="28" t="n">
         <v>0.33</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="28" t="n">
         <v>0.33</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="28" t="n">
         <v>0.6</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="28" t="n">
         <v>0.6</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="I8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2183,33 +2585,33 @@
           <t>Число событий в год</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="21" t="n">
+      <c r="F9" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="G9" s="21" t="n">
+      <c r="G9" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="H9" s="21" t="n">
+      <c r="H9" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="I9" s="21" t="n">
+      <c r="I9" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="J9" s="27" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2219,33 +2621,33 @@
           <t>Зимний пакет (каток, горка, свет)</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>млн тг/год</t>
         </is>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="21" t="n">
+      <c r="F10" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="29" t="n">
         <v>2.5</v>
       </c>
-      <c r="H10" s="23" t="n">
+      <c r="H10" s="29" t="n">
         <v>4.5</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="27" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2255,38 +2657,38 @@
           <t>Персонал парка (только Т4)</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>млн тг/год</t>
         </is>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="21" t="n">
+      <c r="G11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="21" t="n">
+      <c r="H11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="21" t="n">
+      <c r="I11" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="21" t="n">
+      <c r="J11" s="27" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>ОБЩИЕ НОРМАТИВЫ (мин / макс)</t>
         </is>
@@ -2298,23 +2700,23 @@
           <t>Ставка координатора кластера</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>тыс тг/мес</t>
         </is>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="27" t="n">
         <v>420</v>
       </c>
-      <c r="E14" s="25" t="n"/>
-      <c r="F14" s="25" t="n"/>
-      <c r="G14" s="25" t="n"/>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
-      <c r="J14" s="25" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2322,23 +2724,23 @@
           <t>Цена события с продвижением</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>тыс тг</t>
         </is>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="27" t="n">
         <v>95</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="27" t="n">
         <v>130</v>
       </c>
-      <c r="E15" s="25" t="n"/>
-      <c r="F15" s="25" t="n"/>
-      <c r="G15" s="25" t="n"/>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
-      <c r="J15" s="25" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="31" t="n"/>
+      <c r="I15" s="31" t="n"/>
+      <c r="J15" s="31" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -2346,23 +2748,47 @@
           <t>Ремфонд, доля от прочих статей OPEX</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>доля</t>
         </is>
       </c>
-      <c r="C16" s="26" t="n">
+      <c r="C16" s="32" t="n">
         <v>0.05</v>
       </c>
-      <c r="D16" s="26" t="n">
+      <c r="D16" s="32" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="E16" s="25" t="n"/>
-      <c r="F16" s="25" t="n"/>
-      <c r="G16" s="25" t="n"/>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
-      <c r="J16" s="25" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
+      <c r="H16" s="31" t="n"/>
+      <c r="I16" s="31" t="n"/>
+      <c r="J16" s="31" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Коэффициент: общая площадь / озеленение</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="31" t="n"/>
+      <c r="J17" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2380,7 +2806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2390,390 +2816,401 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>Финмодель Т1 · Транзитная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="35" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="29" t="inlineStr">
-        <is>
-          <t>Аура Аллея</t>
-        </is>
-      </c>
-      <c r="C3" s="30" t="inlineStr">
-        <is>
-          <t>Площадь, м²:</t>
-        </is>
-      </c>
-      <c r="D3" s="31">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$35,MATCH($B$3,Объекты!$B$4:$B$35,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
+        <is>
+          <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>Озеленение, м²:</t>
+        </is>
+      </c>
+      <c r="D3" s="38">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Общая площадь, м²:</t>
+        </is>
+      </c>
+      <c r="D4" s="38">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Статья</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Как считаем / привязка</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Мин, млн тг/год</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Макс, млн тг/год</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n"/>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="25" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Вендинг, 1 автомат</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>аренда точки 25–45 тыс тг/мес</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Спонсорство «Усынови клумбу»</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>3–5 спонсоров по 80–150 тыс тг/год</t>
+          <t>Вендинг, 1 автомат</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>аренда точки 25–45 тыс тг/мес</t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>Спонсорство «Усынови клумбу»</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>3–5 спонсоров по 80–150 тыс тг/год</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>Реклама на навигации</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>при подходящем юрстатусе земли</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C10" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D10" s="33" t="n">
         <v>0.4</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="34" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B10" s="35" t="n"/>
-      <c r="C10" s="36">
-        <f>SUM(C7:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="36">
-        <f>SUM(D7:D9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="B11" s="41" t="n"/>
+      <c r="C11" s="42">
+        <f>SUM(C8:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="42">
+        <f>SUM(D8:D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B11" s="25" t="n"/>
-      <c r="C11" s="25" t="n"/>
-      <c r="D11" s="25" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Уборка и снегоуборка</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 12 мес</t>
-        </is>
-      </c>
-      <c r="C12" s="37">
-        <f>$D$3*Нормативы!C5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D12" s="37">
-        <f>$D$3*Нормативы!D5*12/1000000</f>
-        <v/>
-      </c>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="31" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Озеленение и полив</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 7 мес (апр–окт)</t>
-        </is>
-      </c>
-      <c r="C13" s="37">
-        <f>$D$3*Нормативы!C6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D13" s="37">
-        <f>$D$3*Нормативы!D6*7/1000000</f>
+          <t>Уборка и снегоуборка</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × норматив × 12 мес</t>
+        </is>
+      </c>
+      <c r="C13" s="43">
+        <f>$D$4*Нормативы!C5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D13" s="43">
+        <f>$D$4*Нормативы!D5*12/1000000</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Свет, электро, digital</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>площадь × годовой норматив</t>
-        </is>
-      </c>
-      <c r="C14" s="37">
-        <f>$D$3*Нормативы!C7/1000000</f>
-        <v/>
-      </c>
-      <c r="D14" s="37">
-        <f>$D$3*Нормативы!D7/1000000</f>
+          <t>Озеленение и полив</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>озеленение × норматив × 7 мес (апр–окт)</t>
+        </is>
+      </c>
+      <c r="C14" s="43">
+        <f>$D$3*Нормативы!C6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D14" s="43">
+        <f>$D$3*Нормативы!D6*7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Координатор кластера</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>ставка × доля × 12 мес</t>
-        </is>
-      </c>
-      <c r="C15" s="37">
-        <f>Нормативы!$C$14*Нормативы!C8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D15" s="37">
-        <f>Нормативы!$D$14*Нормативы!D8*12/1000</f>
+          <t>Свет, электро, digital</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × годовой норматив</t>
+        </is>
+      </c>
+      <c r="C15" s="43">
+        <f>$D$4*Нормативы!C7/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="43">
+        <f>$D$4*Нормативы!D7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>Координатор кластера</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>ставка × доля × 12 мес</t>
+        </is>
+      </c>
+      <c r="C16" s="43">
+        <f>Нормативы!$C$14*Нормативы!C8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D16" s="43">
+        <f>Нормативы!$D$14*Нормативы!D8*12/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>доля от прочих статей OPEX</t>
         </is>
       </c>
-      <c r="C16" s="37">
-        <f>Нормативы!$C$16*SUM(C12:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="37">
-        <f>Нормативы!$D$16*SUM(D12:D15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="C17" s="43">
+        <f>Нормативы!$C$16*SUM(C13:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="43">
+        <f>Нормативы!$D$16*SUM(D13:D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="44" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B17" s="35" t="n"/>
-      <c r="C17" s="39">
-        <f>SUM(C12:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="39">
-        <f>SUM(D12:D16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="B18" s="41" t="n"/>
+      <c r="C18" s="45">
+        <f>SUM(C13:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="45">
+        <f>SUM(D13:D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B19" s="25" t="n"/>
-      <c r="C19" s="25" t="n"/>
-      <c r="D19" s="25" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Консервативный сценарий</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>низ доходов / верх расходов</t>
-        </is>
-      </c>
-      <c r="C20" s="40">
-        <f>IFERROR(C10/D17,0)</f>
-        <v/>
-      </c>
-      <c r="D20" s="25" t="n"/>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="31" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>По середине вилок</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>средние значения обеих вилок</t>
-        </is>
-      </c>
-      <c r="C21" s="40">
-        <f>IFERROR(AVERAGE(C10:D10)/AVERAGE(C17:D17),0)</f>
-        <v/>
-      </c>
-      <c r="D21" s="25" t="n"/>
+          <t>Консервативный сценарий</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>низ доходов / верх расходов</t>
+        </is>
+      </c>
+      <c r="C21" s="46">
+        <f>IFERROR(C11/D18,0)</f>
+        <v/>
+      </c>
+      <c r="D21" s="31" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>По середине вилок</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>средние значения обеих вилок</t>
+        </is>
+      </c>
+      <c r="C22" s="46">
+        <f>IFERROR(AVERAGE(C11:D11)/AVERAGE(C18:D18),0)</f>
+        <v/>
+      </c>
+      <c r="D22" s="31" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C22" s="40">
-        <f>IFERROR(D10/C17,0)</f>
-        <v/>
-      </c>
-      <c r="D22" s="25" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="41" t="inlineStr">
+      <c r="C23" s="46">
+        <f>IFERROR(D11/C18,0)</f>
+        <v/>
+      </c>
+      <c r="D23" s="31" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="47" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B23" s="25" t="n"/>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="48" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
       </c>
-      <c r="D23" s="25" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="D24" s="31" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="39" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B25" s="25" t="n"/>
-      <c r="C25" s="25" t="n"/>
-      <c r="D25" s="25" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="43" t="inlineStr">
+      <c r="B26" s="31" t="n"/>
+      <c r="C26" s="31" t="n"/>
+      <c r="D26" s="31" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="inlineStr">
         <is>
           <t>• Кластер: общий координатор и бригада, не своя</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="43" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
         <is>
           <t>• Спонсоры продлеваются на второй год</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="43" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
         <is>
           <t>• Юрстатус пропускает рекламу на стелах</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
+    <row r="32"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A30:D31"/>
     <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A31:D32"/>
     <mergeCell ref="A28:D28"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$35</formula1>
+      <formula1>=Объекты!$B$4:$B$36</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2781,468 +3218,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="27" t="inlineStr">
-        <is>
-          <t>Финмодель Т2 · Активная аллея</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="28" t="inlineStr">
-        <is>
-          <t>Объект (выберите из списка):</t>
-        </is>
-      </c>
-      <c r="B3" s="29" t="inlineStr">
-        <is>
-          <t>Аллея Nexpo Классик</t>
-        </is>
-      </c>
-      <c r="C3" s="30" t="inlineStr">
-        <is>
-          <t>Площадь, м²:</t>
-        </is>
-      </c>
-      <c r="D3" s="31">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$35,MATCH($B$3,Объекты!$B$4:$B$35,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Как считаем / привязка</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Мин, млн тг/год</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Макс, млн тг/год</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
-        <is>
-          <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="n"/>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="25" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>НТО-якорь: кофе-павильон</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Ярмарка выходного дня</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Секции и кикшеринг</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>слоты тренерам + rev-share операторов</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Digital-экран и реклама</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>при подходящем юрстатусе земли</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D10" s="33" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Спонсорство объектов</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>воркаут, клумбы, скамейки</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D11" s="33" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t>Доходы, итого</t>
-        </is>
-      </c>
-      <c r="B12" s="35" t="n"/>
-      <c r="C12" s="36">
-        <f>SUM(C7:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="36">
-        <f>SUM(D7:D11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="32" t="inlineStr">
-        <is>
-          <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n"/>
-      <c r="C13" s="25" t="n"/>
-      <c r="D13" s="25" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Уборка и снегоуборка</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 12 мес</t>
-        </is>
-      </c>
-      <c r="C14" s="37">
-        <f>$D$3*Нормативы!E5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D14" s="37">
-        <f>$D$3*Нормативы!F5*12/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Озеленение и полив</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 7 мес (апр–окт)</t>
-        </is>
-      </c>
-      <c r="C15" s="37">
-        <f>$D$3*Нормативы!E6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="37">
-        <f>$D$3*Нормативы!F6*7/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Свет, электро, digital</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>площадь × годовой норматив</t>
-        </is>
-      </c>
-      <c r="C16" s="37">
-        <f>$D$3*Нормативы!E7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="37">
-        <f>$D$3*Нормативы!F7/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Программа и маркетинг</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>число событий × цена события</t>
-        </is>
-      </c>
-      <c r="C17" s="37">
-        <f>Нормативы!E9*Нормативы!$C$15/1000</f>
-        <v/>
-      </c>
-      <c r="D17" s="37">
-        <f>Нормативы!F9*Нормативы!$D$15/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Координатор кластера</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>ставка × доля × 12 мес</t>
-        </is>
-      </c>
-      <c r="C18" s="37">
-        <f>Нормативы!$C$14*Нормативы!E8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D18" s="37">
-        <f>Нормативы!$D$14*Нормативы!F8*12/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Ремфонд</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>доля от прочих статей OPEX</t>
-        </is>
-      </c>
-      <c r="C19" s="37">
-        <f>Нормативы!$C$16*SUM(C14:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="37">
-        <f>Нормативы!$D$16*SUM(D14:D18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="38" t="inlineStr">
-        <is>
-          <t>OPEX, итого</t>
-        </is>
-      </c>
-      <c r="B20" s="35" t="n"/>
-      <c r="C20" s="39">
-        <f>SUM(C14:C19)</f>
-        <v/>
-      </c>
-      <c r="D20" s="39">
-        <f>SUM(D14:D19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="32" t="inlineStr">
-        <is>
-          <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
-        </is>
-      </c>
-      <c r="B22" s="25" t="n"/>
-      <c r="C22" s="25" t="n"/>
-      <c r="D22" s="25" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Консервативный сценарий</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>низ доходов / верх расходов</t>
-        </is>
-      </c>
-      <c r="C23" s="40">
-        <f>IFERROR(C12/D20,0)</f>
-        <v/>
-      </c>
-      <c r="D23" s="25" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>По середине вилок</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="inlineStr">
-        <is>
-          <t>средние значения обеих вилок</t>
-        </is>
-      </c>
-      <c r="C24" s="40">
-        <f>IFERROR(AVERAGE(C12:D12)/AVERAGE(C20:D20),0)</f>
-        <v/>
-      </c>
-      <c r="D24" s="25" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Оптимистичный сценарий</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>верх доходов / низ расходов</t>
-        </is>
-      </c>
-      <c r="C25" s="40">
-        <f>IFERROR(D12/C20,0)</f>
-        <v/>
-      </c>
-      <c r="D25" s="25" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="41" t="inlineStr">
-        <is>
-          <t>Целевой коридор пилота</t>
-        </is>
-      </c>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="42" t="inlineStr">
-        <is>
-          <t>40–70%</t>
-        </is>
-      </c>
-      <c r="D26" s="25" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="32" t="inlineStr">
-        <is>
-          <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
-        </is>
-      </c>
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="25" t="n"/>
-      <c r="D28" s="25" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="43" t="inlineStr">
-        <is>
-          <t>• Якорь-павильон заполнен с мая по сентябрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="43" t="inlineStr">
-        <is>
-          <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="43" t="inlineStr">
-        <is>
-          <t>• Вечерние слоты секций выкуплены</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A33:D34"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A13:D13"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$35</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3258,258 +3233,249 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
-        <is>
-          <t>Финмодель Т3 · Плейхаб</t>
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Финмодель Т2 · Активная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="35" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="29" t="inlineStr">
-        <is>
-          <t>Плейхаб Аква 1</t>
-        </is>
-      </c>
-      <c r="C3" s="30" t="inlineStr">
-        <is>
-          <t>Площадь, м²:</t>
-        </is>
-      </c>
-      <c r="D3" s="31">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$35,MATCH($B$3,Объекты!$B$4:$B$35,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
+        <is>
+          <t>Аллея Хедлайнер Эксклюзив</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>Озеленение, м²:</t>
+        </is>
+      </c>
+      <c r="D3" s="38">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Общая площадь, м²:</t>
+        </is>
+      </c>
+      <c r="D4" s="38">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Статья</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Как считаем / привязка</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Мин, млн тг/год</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Макс, млн тг/год</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n"/>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="25" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Две НТО-точки</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>кофе и выпечка: аренда + % оборота</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>4.8</v>
-      </c>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Каток: прокат и билеты</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>120–160 дней зимнего сезона</t>
+          <t>НТО-якорь: кофе-павильон</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>5.5</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Событийная аренда</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>10–18 частных и корпоративных событий</t>
+          <t>Ярмарка выходного дня</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Ярмарки, маркеты, секции</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>круглогодичный календарь</t>
+          <t>Секции и кикшеринг</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>слоты тренерам + rev-share операторов</t>
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Спонсор года и реклама</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>один якорный партнёр + экран</t>
+          <t>Digital-экран и реклама</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>при подходящем юрстатусе земли</t>
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="34" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Спонсорство объектов</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>воркаут, клумбы, скамейки</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B12" s="35" t="n"/>
-      <c r="C12" s="36">
-        <f>SUM(C7:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="36">
-        <f>SUM(D7:D11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="B13" s="41" t="n"/>
+      <c r="C13" s="42">
+        <f>SUM(C8:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="42">
+        <f>SUM(D8:D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B13" s="25" t="n"/>
-      <c r="C13" s="25" t="n"/>
-      <c r="D13" s="25" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Уборка и снегоуборка</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 12 мес</t>
-        </is>
-      </c>
-      <c r="C14" s="37">
-        <f>$D$3*Нормативы!G5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D14" s="37">
-        <f>$D$3*Нормативы!H5*12/1000000</f>
-        <v/>
-      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Озеленение и полив</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 7 мес (апр–окт)</t>
-        </is>
-      </c>
-      <c r="C15" s="37">
-        <f>$D$3*Нормативы!G6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="37">
-        <f>$D$3*Нормативы!H6*7/1000000</f>
+          <t>Уборка и снегоуборка</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × норматив × 12 мес</t>
+        </is>
+      </c>
+      <c r="C15" s="43">
+        <f>$D$4*Нормативы!E5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="43">
+        <f>$D$4*Нормативы!F5*12/1000000</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Свет, электро, digital</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>площадь × годовой норматив</t>
-        </is>
-      </c>
-      <c r="C16" s="37">
-        <f>$D$3*Нормативы!G7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="37">
-        <f>$D$3*Нормативы!H7/1000000</f>
+          <t>Озеленение и полив</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>озеленение × норматив × 7 мес (апр–окт)</t>
+        </is>
+      </c>
+      <c r="C16" s="43">
+        <f>$D$3*Нормативы!E6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="43">
+        <f>$D$3*Нормативы!F6*7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Зимний пакет</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>норматив, млн тг/год</t>
-        </is>
-      </c>
-      <c r="C17" s="37">
-        <f>Нормативы!G10</f>
-        <v/>
-      </c>
-      <c r="D17" s="37">
-        <f>Нормативы!H10</f>
+          <t>Свет, электро, digital</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × годовой норматив</t>
+        </is>
+      </c>
+      <c r="C17" s="43">
+        <f>$D$4*Нормативы!E7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="43">
+        <f>$D$4*Нормативы!F7/1000000</f>
         <v/>
       </c>
     </row>
@@ -3519,17 +3485,17 @@
           <t>Программа и маркетинг</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C18" s="37">
-        <f>Нормативы!G9*Нормативы!$C$15/1000</f>
-        <v/>
-      </c>
-      <c r="D18" s="37">
-        <f>Нормативы!H9*Нормативы!$D$15/1000</f>
+      <c r="C18" s="43">
+        <f>Нормативы!E9*Нормативы!$C$15/1000</f>
+        <v/>
+      </c>
+      <c r="D18" s="43">
+        <f>Нормативы!F9*Нормативы!$D$15/1000</f>
         <v/>
       </c>
     </row>
@@ -3539,17 +3505,17 @@
           <t>Координатор кластера</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C19" s="37">
-        <f>Нормативы!$C$14*Нормативы!G8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D19" s="37">
-        <f>Нормативы!$D$14*Нормативы!H8*12/1000</f>
+      <c r="C19" s="43">
+        <f>Нормативы!$C$14*Нормативы!E8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="43">
+        <f>Нормативы!$D$14*Нормативы!F8*12/1000</f>
         <v/>
       </c>
     </row>
@@ -3559,45 +3525,45 @@
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>доля от прочих статей OPEX</t>
         </is>
       </c>
-      <c r="C20" s="37">
-        <f>Нормативы!$C$16*SUM(C14:C19)</f>
-        <v/>
-      </c>
-      <c r="D20" s="37">
-        <f>Нормативы!$D$16*SUM(D14:D19)</f>
+      <c r="C20" s="43">
+        <f>Нормативы!$C$16*SUM(C15:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="43">
+        <f>Нормативы!$D$16*SUM(D15:D19)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="38" t="inlineStr">
+      <c r="A21" s="44" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B21" s="35" t="n"/>
-      <c r="C21" s="39">
-        <f>SUM(C14:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="39">
-        <f>SUM(D14:D20)</f>
+      <c r="B21" s="41" t="n"/>
+      <c r="C21" s="45">
+        <f>SUM(C15:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="45">
+        <f>SUM(D15:D20)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B23" s="25" t="n"/>
-      <c r="C23" s="25" t="n"/>
-      <c r="D23" s="25" t="n"/>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="31" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -3605,16 +3571,16 @@
           <t>Консервативный сценарий</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C24" s="40">
-        <f>IFERROR(C12/D21,0)</f>
-        <v/>
-      </c>
-      <c r="D24" s="25" t="n"/>
+      <c r="C24" s="46">
+        <f>IFERROR(C13/D21,0)</f>
+        <v/>
+      </c>
+      <c r="D24" s="31" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -3622,16 +3588,16 @@
           <t>По середине вилок</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C25" s="40">
-        <f>IFERROR(AVERAGE(C12:D12)/AVERAGE(C21:D21),0)</f>
-        <v/>
-      </c>
-      <c r="D25" s="25" t="n"/>
+      <c r="C25" s="46">
+        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
+        <v/>
+      </c>
+      <c r="D25" s="31" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -3639,59 +3605,59 @@
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C26" s="40">
-        <f>IFERROR(D12/C21,0)</f>
-        <v/>
-      </c>
-      <c r="D26" s="25" t="n"/>
+      <c r="C26" s="46">
+        <f>IFERROR(D13/C21,0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="41" t="inlineStr">
+      <c r="A27" s="47" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="42" t="inlineStr">
-        <is>
-          <t>70–100%</t>
-        </is>
-      </c>
-      <c r="D27" s="25" t="n"/>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="48" t="inlineStr">
+        <is>
+          <t>40–70%</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="32" t="inlineStr">
+      <c r="A29" s="39" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
+      <c r="B29" s="31" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="31" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="43" t="inlineStr">
-        <is>
-          <t>• Каток отработал первую зиму без простоев</t>
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>• Якорь-павильон заполнен с мая по сентябрь</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="43" t="inlineStr">
-        <is>
-          <t>• Заявок на события больше, чем слотов</t>
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="43" t="inlineStr">
-        <is>
-          <t>• Спонсор года подписан до старта сезона</t>
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>• Вечерние слоты секций выкуплены</t>
         </is>
       </c>
     </row>
@@ -3708,16 +3674,509 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A6:D6"/>
     <mergeCell ref="A34:D35"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$35</formula1>
+      <formula1>=Объекты!$B$4:$B$36</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Финмодель Т3 · Сквер / плейхаб</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>Объект (выберите из списка):</t>
+        </is>
+      </c>
+      <c r="B3" s="36" t="inlineStr">
+        <is>
+          <t>Сквер Авеню 5</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>Озеленение, м²:</t>
+        </is>
+      </c>
+      <c r="D3" s="38">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Общая площадь, м²:</t>
+        </is>
+      </c>
+      <c r="D4" s="38">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Как считаем / привязка</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Мин, млн тг/год</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Макс, млн тг/год</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Две НТО-точки</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>кофе и выпечка: аренда + % оборота</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Каток: прокат и билеты</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>компактный контур, 120–160 дней</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Событийная аренда</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>10–18 частных и корпоративных событий</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="33" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Ярмарки, маркеты, секции</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>круглогодичный календарь</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Спонсор года и реклама</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>один якорный партнёр + экран</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Доходы, итого</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="n"/>
+      <c r="C13" s="42">
+        <f>SUM(C8:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="42">
+        <f>SUM(D8:D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Уборка и снегоуборка</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × норматив × 12 мес</t>
+        </is>
+      </c>
+      <c r="C15" s="43">
+        <f>$D$4*Нормативы!G5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="43">
+        <f>$D$4*Нормативы!H5*12/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Озеленение и полив</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>озеленение × норматив × 7 мес (апр–окт)</t>
+        </is>
+      </c>
+      <c r="C16" s="43">
+        <f>$D$3*Нормативы!G6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="43">
+        <f>$D$3*Нормативы!H6*7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Свет, электро, digital</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × годовой норматив</t>
+        </is>
+      </c>
+      <c r="C17" s="43">
+        <f>$D$4*Нормативы!G7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="43">
+        <f>$D$4*Нормативы!H7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Зимний пакет</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>норматив, млн тг/год</t>
+        </is>
+      </c>
+      <c r="C18" s="43">
+        <f>Нормативы!G10</f>
+        <v/>
+      </c>
+      <c r="D18" s="43">
+        <f>Нормативы!H10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Программа и маркетинг</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>число событий × цена события</t>
+        </is>
+      </c>
+      <c r="C19" s="43">
+        <f>Нормативы!G9*Нормативы!$C$15/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="43">
+        <f>Нормативы!H9*Нормативы!$D$15/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Координатор кластера</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>ставка × доля × 12 мес</t>
+        </is>
+      </c>
+      <c r="C20" s="43">
+        <f>Нормативы!$C$14*Нормативы!G8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D20" s="43">
+        <f>Нормативы!$D$14*Нормативы!H8*12/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Ремфонд</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>доля от прочих статей OPEX</t>
+        </is>
+      </c>
+      <c r="C21" s="43">
+        <f>Нормативы!$C$16*SUM(C15:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="43">
+        <f>Нормативы!$D$16*SUM(D15:D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>OPEX, итого</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="n"/>
+      <c r="C22" s="45">
+        <f>SUM(C15:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="45">
+        <f>SUM(D15:D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="31" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Консервативный сценарий</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>низ доходов / верх расходов</t>
+        </is>
+      </c>
+      <c r="C25" s="46">
+        <f>IFERROR(C13/D22,0)</f>
+        <v/>
+      </c>
+      <c r="D25" s="31" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>По середине вилок</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>средние значения обеих вилок</t>
+        </is>
+      </c>
+      <c r="C26" s="46">
+        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C22:D22),0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Оптимистичный сценарий</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>верх доходов / низ расходов</t>
+        </is>
+      </c>
+      <c r="C27" s="46">
+        <f>IFERROR(D13/C22,0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="31" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="47" t="inlineStr">
+        <is>
+          <t>Целевой коридор пилота</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="n"/>
+      <c r="C28" s="48" t="inlineStr">
+        <is>
+          <t>70–100%</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="n"/>
+      <c r="C30" s="31" t="n"/>
+      <c r="D30" s="31" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>• Каток отработал первую зиму без простоев</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>• Заявок на события больше, чем слотов</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>• Спонсор года подписан до старта сезона</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A35:D36"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=Объекты!$B$4:$B$36</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3730,7 +4189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3740,492 +4199,503 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>Финмодель Т4 · Парк по ГЧП (BTO)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="35" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="29" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>Sphere Park</t>
         </is>
       </c>
-      <c r="C3" s="30" t="inlineStr">
-        <is>
-          <t>Площадь, м²:</t>
-        </is>
-      </c>
-      <c r="D3" s="31">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$35,MATCH($B$3,Объекты!$B$4:$B$35,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>Озеленение, м²:</t>
+        </is>
+      </c>
+      <c r="D3" s="38">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Общая площадь, м²:</t>
+        </is>
+      </c>
+      <c r="D4" s="38">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Статья</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Как считаем / привязка</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Мин, млн тг/год</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Макс, млн тг/год</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n"/>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="25" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Компенсация эксплуатации (акимат)</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>структура BTO: ~0,33 млрд тг за 5 лет</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>55</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>70</v>
-      </c>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>НТО-точки, 3–5 шт</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>кофе, стритфуд, прокат</t>
+          <t>Компенсация эксплуатации (акимат)</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>структура BTO: ~0,33 млрд тг за 5 лет</t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>6</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Каток и зимний прокат</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>большой контур, 120–160 дней</t>
+          <t>НТО-точки, 3–5 шт</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>кофе, стритфуд, прокат</t>
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Событийная аренда и фестивали</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>городской масштаб</t>
+          <t>Каток и зимний прокат</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>большой контур, 120–160 дней</t>
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Ярмарки и маркеты</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>круглогодично</t>
+          <t>Событийная аренда и фестивали</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>городской масштаб</t>
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Спонсоры и реклама</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>якорные партнёры</t>
+          <t>Ярмарки и маркеты</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>круглогодично</t>
         </is>
       </c>
       <c r="C12" s="33" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="33" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Спонсоры и реклама</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>якорные партнёры</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="33" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="34" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="36">
-        <f>SUM(C7:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="36">
-        <f>SUM(D7:D12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="B14" s="41" t="n"/>
+      <c r="C14" s="42">
+        <f>SUM(C8:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="42">
+        <f>SUM(D8:D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="25" t="n"/>
-      <c r="D14" s="25" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Уборка и снегоуборка</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 12 мес</t>
-        </is>
-      </c>
-      <c r="C15" s="37">
-        <f>$D$3*Нормативы!I5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="37">
-        <f>$D$3*Нормативы!J5*12/1000000</f>
-        <v/>
-      </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Озеленение и полив</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>площадь × норматив × 7 мес (апр–окт)</t>
-        </is>
-      </c>
-      <c r="C16" s="37">
-        <f>$D$3*Нормативы!I6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="37">
-        <f>$D$3*Нормативы!J6*7/1000000</f>
+          <t>Уборка и снегоуборка</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × норматив × 12 мес</t>
+        </is>
+      </c>
+      <c r="C16" s="43">
+        <f>$D$4*Нормативы!I5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="43">
+        <f>$D$4*Нормативы!J5*12/1000000</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Свет, электро, digital</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>площадь × годовой норматив</t>
-        </is>
-      </c>
-      <c r="C17" s="37">
-        <f>$D$3*Нормативы!I7/1000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="37">
-        <f>$D$3*Нормативы!J7/1000000</f>
+          <t>Озеленение и полив</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>озеленение × норматив × 7 мес (апр–окт)</t>
+        </is>
+      </c>
+      <c r="C17" s="43">
+        <f>$D$3*Нормативы!I6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="43">
+        <f>$D$3*Нормативы!J6*7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Зимний пакет</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>норматив, млн тг/год</t>
-        </is>
-      </c>
-      <c r="C18" s="37">
-        <f>Нормативы!I10</f>
-        <v/>
-      </c>
-      <c r="D18" s="37">
-        <f>Нормативы!J10</f>
+          <t>Свет, электро, digital</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × годовой норматив</t>
+        </is>
+      </c>
+      <c r="C18" s="43">
+        <f>$D$4*Нормативы!I7/1000000</f>
+        <v/>
+      </c>
+      <c r="D18" s="43">
+        <f>$D$4*Нормативы!J7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Программа и маркетинг</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>число событий × цена события</t>
-        </is>
-      </c>
-      <c r="C19" s="37">
-        <f>Нормативы!I9*Нормативы!$C$15/1000</f>
-        <v/>
-      </c>
-      <c r="D19" s="37">
-        <f>Нормативы!J9*Нормативы!$D$15/1000</f>
+          <t>Зимний пакет</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>норматив, млн тг/год</t>
+        </is>
+      </c>
+      <c r="C19" s="43">
+        <f>Нормативы!I10</f>
+        <v/>
+      </c>
+      <c r="D19" s="43">
+        <f>Нормативы!J10</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Персонал парка</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>норматив, млн тг/год</t>
-        </is>
-      </c>
-      <c r="C20" s="37">
-        <f>Нормативы!I11</f>
-        <v/>
-      </c>
-      <c r="D20" s="37">
-        <f>Нормативы!J11</f>
+          <t>Программа и маркетинг</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>число событий × цена события</t>
+        </is>
+      </c>
+      <c r="C20" s="43">
+        <f>Нормативы!I9*Нормативы!$C$15/1000</f>
+        <v/>
+      </c>
+      <c r="D20" s="43">
+        <f>Нормативы!J9*Нормативы!$D$15/1000</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>Персонал парка</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>норматив, млн тг/год</t>
+        </is>
+      </c>
+      <c r="C21" s="43">
+        <f>Нормативы!I11</f>
+        <v/>
+      </c>
+      <c r="D21" s="43">
+        <f>Нормативы!J11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>доля от прочих статей OPEX</t>
         </is>
       </c>
-      <c r="C21" s="37">
-        <f>Нормативы!$C$16*SUM(C15:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="37">
-        <f>Нормативы!$D$16*SUM(D15:D20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="38" t="inlineStr">
+      <c r="C22" s="43">
+        <f>Нормативы!$C$16*SUM(C16:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="43">
+        <f>Нормативы!$D$16*SUM(D16:D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="44" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B22" s="35" t="n"/>
-      <c r="C22" s="39">
-        <f>SUM(C15:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="39">
-        <f>SUM(D15:D21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="B23" s="41" t="n"/>
+      <c r="C23" s="45">
+        <f>SUM(C16:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="45">
+        <f>SUM(D16:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="39" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B24" s="25" t="n"/>
-      <c r="C24" s="25" t="n"/>
-      <c r="D24" s="25" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Консервативный сценарий</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>низ доходов / верх расходов</t>
-        </is>
-      </c>
-      <c r="C25" s="40">
-        <f>IFERROR(C13/D22,0)</f>
-        <v/>
-      </c>
-      <c r="D25" s="25" t="n"/>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="31" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>По середине вилок</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>средние значения обеих вилок</t>
-        </is>
-      </c>
-      <c r="C26" s="40">
-        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C22:D22),0)</f>
-        <v/>
-      </c>
-      <c r="D26" s="25" t="n"/>
+          <t>Консервативный сценарий</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>низ доходов / верх расходов</t>
+        </is>
+      </c>
+      <c r="C26" s="46">
+        <f>IFERROR(C14/D23,0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
+          <t>По середине вилок</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>средние значения обеих вилок</t>
+        </is>
+      </c>
+      <c r="C27" s="46">
+        <f>IFERROR(AVERAGE(C14:D14)/AVERAGE(C23:D23),0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="31" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B28" s="26" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C27" s="40">
-        <f>IFERROR(D13/C22,0)</f>
-        <v/>
-      </c>
-      <c r="D27" s="25" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="41" t="inlineStr">
+      <c r="C28" s="46">
+        <f>IFERROR(D14/C23,0)</f>
+        <v/>
+      </c>
+      <c r="D28" s="31" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="B29" s="31" t="n"/>
+      <c r="C29" s="48" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
       </c>
-      <c r="D28" s="25" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="32" t="inlineStr">
+      <c r="D29" s="31" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="39" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="43" t="inlineStr">
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="31" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
         <is>
           <t>• ГЧП-договор подписан, компенсация в бюджете МИО</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="43" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
         <is>
           <t>• Каток и события дотягивают покрытие до 100%+</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="43" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
         <is>
           <t>• Стандарт содержания выше городского бенчмарка</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="43" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
         <is>
           <t>• CAPEX ~2,2 млрд тг компенсируется бюджетом МИО отдельно (2026–2031) — в операционную модель не входит</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
         </is>
       </c>
     </row>
-    <row r="37"/>
+    <row r="38"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A6:D6"/>
     <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A36:D37"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A25:D25"/>
     <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A37:D38"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$35</formula1>
+      <formula1>=Объекты!$B$4:$B$36</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Detail deck and finmodels with developer asset certificates
Deck (30 slides): new balance-sheet assets slide (~504M KZT across 8
shortlist objects), pilot cards updated with asset facts (Flora 1+2
72.1M incl. 40 lights, Avenue 5 greenery-only 2.1M, Headliner
certificate pending), T1-T3 repair-fund lines and totals recalculated.

Workbook v4: new Assets sheet from 8 developer certificates with
category breakdown, activation CAPEX norm per type, repair fund
reworked to 1-1.5%/yr of (assets + activation CAPEX), asset row in
model sheets and summary.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014o1yT6nCgffZ5H25q7THst
</commit_message>
<xml_diff>
--- a/docs/research/BIG-Life-finmodels-T1-T4.xlsx
+++ b/docs/research/BIG-Life-finmodels-T1-T4.xlsx
@@ -10,10 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нормативы" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т1 Транзитная" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т2 Активная" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т3 Сквер" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т4 Sphere Park" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Активы" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т1 Транзитная" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т2 Активная" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т3 Сквер" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т4 Sphere Park" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +23,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.#"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +110,28 @@
       <b val="1"/>
       <color rgb="001B2A6E"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="008A93A6"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B2A6E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -238,10 +262,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -252,22 +276,22 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -307,39 +331,71 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -708,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -735,310 +791,334 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая = озеленение × коэффициент (лист «Нормативы», по умолчанию ×2). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Жёлтые ячейки — редактируемые ставки.</t>
+          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая = озеленение × коэффициент (лист «Нормативы», по умолчанию ×2). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Жёлтые ячейки — редактируемые ставки.</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6"/>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="7"/>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Т1 · Flora 1+2</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Т2 · Хедлайнер Экс.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Т3 · Авеню 5</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Т4 · Sphere Park</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Выбранный объект</t>
-        </is>
-      </c>
-      <c r="B9" s="7">
-        <f>'Т1 Транзитная'!B3</f>
-        <v/>
-      </c>
-      <c r="C9" s="7">
-        <f>'Т2 Активная'!B3</f>
-        <v/>
-      </c>
-      <c r="D9" s="7">
-        <f>'Т3 Сквер'!B3</f>
-        <v/>
-      </c>
-      <c r="E9" s="7">
-        <f>'Т4 Sphere Park'!B3</f>
-        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Озеленение, м²</t>
-        </is>
-      </c>
-      <c r="B10" s="8">
-        <f>'Т1 Транзитная'!D3</f>
-        <v/>
-      </c>
-      <c r="C10" s="8">
-        <f>'Т2 Активная'!D3</f>
-        <v/>
-      </c>
-      <c r="D10" s="8">
-        <f>'Т3 Сквер'!D3</f>
-        <v/>
-      </c>
-      <c r="E10" s="8">
-        <f>'Т4 Sphere Park'!D3</f>
+          <t>Выбранный объект</t>
+        </is>
+      </c>
+      <c r="B10" s="7">
+        <f>'Т1 Транзитная'!B3</f>
+        <v/>
+      </c>
+      <c r="C10" s="7">
+        <f>'Т2 Активная'!B3</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>'Т3 Сквер'!B3</f>
+        <v/>
+      </c>
+      <c r="E10" s="7">
+        <f>'Т4 Sphere Park'!B3</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Общая площадь, м²</t>
+          <t>Озеленение, м²</t>
         </is>
       </c>
       <c r="B11" s="8">
-        <f>'Т1 Транзитная'!D4</f>
+        <f>'Т1 Транзитная'!D3</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>'Т2 Активная'!D4</f>
+        <f>'Т2 Активная'!D3</f>
         <v/>
       </c>
       <c r="D11" s="8">
-        <f>'Т3 Сквер'!D4</f>
+        <f>'Т3 Сквер'!D3</f>
         <v/>
       </c>
       <c r="E11" s="8">
-        <f>'Т4 Sphere Park'!D4</f>
+        <f>'Т4 Sphere Park'!D3</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Доходы, млн тг/год (мин)</t>
-        </is>
-      </c>
-      <c r="B12" s="9">
-        <f>'Т1 Транзитная'!C11</f>
-        <v/>
-      </c>
-      <c r="C12" s="9">
-        <f>'Т2 Активная'!C13</f>
-        <v/>
-      </c>
-      <c r="D12" s="9">
-        <f>'Т3 Сквер'!C13</f>
-        <v/>
-      </c>
-      <c r="E12" s="9">
-        <f>'Т4 Sphere Park'!C14</f>
+          <t>Общая площадь, м²</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>'Т1 Транзитная'!D4</f>
+        <v/>
+      </c>
+      <c r="C12" s="8">
+        <f>'Т2 Активная'!D4</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>'Т3 Сквер'!D4</f>
+        <v/>
+      </c>
+      <c r="E12" s="8">
+        <f>'Т4 Sphere Park'!D4</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Доходы, млн тг/год (макс)</t>
+          <t>Активы на балансе, млн тг</t>
         </is>
       </c>
       <c r="B13" s="9">
-        <f>'Т1 Транзитная'!D11</f>
+        <f>'Т1 Транзитная'!B4</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>'Т2 Активная'!D13</f>
+        <f>'Т2 Активная'!B4</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>'Т3 Сквер'!D13</f>
+        <f>'Т3 Сквер'!B4</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>'Т4 Sphere Park'!D14</f>
+        <f>'Т4 Sphere Park'!B4</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>OPEX, млн тг/год (мин)</t>
+          <t>Доходы, млн тг/год (мин)</t>
         </is>
       </c>
       <c r="B14" s="9">
-        <f>'Т1 Транзитная'!C18</f>
+        <f>'Т1 Транзитная'!C11</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>'Т2 Активная'!C21</f>
+        <f>'Т2 Активная'!C13</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>'Т3 Сквер'!C22</f>
+        <f>'Т3 Сквер'!C13</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>'Т4 Sphere Park'!C23</f>
+        <f>'Т4 Sphere Park'!C14</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>OPEX, млн тг/год (макс)</t>
+          <t>Доходы, млн тг/год (макс)</t>
         </is>
       </c>
       <c r="B15" s="9">
-        <f>'Т1 Транзитная'!D18</f>
+        <f>'Т1 Транзитная'!D11</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>'Т2 Активная'!D21</f>
+        <f>'Т2 Активная'!D13</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>'Т3 Сквер'!D22</f>
+        <f>'Т3 Сквер'!D13</f>
         <v/>
       </c>
       <c r="E15" s="9">
-        <f>'Т4 Sphere Park'!D23</f>
+        <f>'Т4 Sphere Park'!D14</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Покрытие OPEX, консервативно</t>
-        </is>
-      </c>
-      <c r="B16" s="10">
-        <f>IFERROR('Т1 Транзитная'!C11/'Т1 Транзитная'!D18,0)</f>
-        <v/>
-      </c>
-      <c r="C16" s="10">
-        <f>IFERROR('Т2 Активная'!C13/'Т2 Активная'!D21,0)</f>
-        <v/>
-      </c>
-      <c r="D16" s="10">
-        <f>IFERROR('Т3 Сквер'!C13/'Т3 Сквер'!D22,0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="10">
-        <f>IFERROR('Т4 Sphere Park'!C14/'Т4 Sphere Park'!D23,0)</f>
+          <t>OPEX, млн тг/год (мин)</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
+        <f>'Т1 Транзитная'!C18</f>
+        <v/>
+      </c>
+      <c r="C16" s="9">
+        <f>'Т2 Активная'!C21</f>
+        <v/>
+      </c>
+      <c r="D16" s="9">
+        <f>'Т3 Сквер'!C22</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>'Т4 Sphere Park'!C23</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Покрытие OPEX, по середине вилок</t>
-        </is>
-      </c>
-      <c r="B17" s="10">
-        <f>IFERROR(AVERAGE('Т1 Транзитная'!C11:D11)/AVERAGE('Т1 Транзитная'!C18:D18),0)</f>
-        <v/>
-      </c>
-      <c r="C17" s="10">
-        <f>IFERROR(AVERAGE('Т2 Активная'!C13:D13)/AVERAGE('Т2 Активная'!C21:D21),0)</f>
-        <v/>
-      </c>
-      <c r="D17" s="10">
-        <f>IFERROR(AVERAGE('Т3 Сквер'!C13:D13)/AVERAGE('Т3 Сквер'!C22:D22),0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="10">
-        <f>IFERROR(AVERAGE('Т4 Sphere Park'!C14:D14)/AVERAGE('Т4 Sphere Park'!C23:D23),0)</f>
+          <t>OPEX, млн тг/год (макс)</t>
+        </is>
+      </c>
+      <c r="B17" s="9">
+        <f>'Т1 Транзитная'!D18</f>
+        <v/>
+      </c>
+      <c r="C17" s="9">
+        <f>'Т2 Активная'!D21</f>
+        <v/>
+      </c>
+      <c r="D17" s="9">
+        <f>'Т3 Сквер'!D22</f>
+        <v/>
+      </c>
+      <c r="E17" s="9">
+        <f>'Т4 Sphere Park'!D23</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Покрытие OPEX, оптимистично</t>
+          <t>Покрытие OPEX, консервативно</t>
         </is>
       </c>
       <c r="B18" s="10">
-        <f>IFERROR('Т1 Транзитная'!D11/'Т1 Транзитная'!C18,0)</f>
+        <f>IFERROR('Т1 Транзитная'!C11/'Т1 Транзитная'!D18,0)</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>IFERROR('Т2 Активная'!D13/'Т2 Активная'!C21,0)</f>
+        <f>IFERROR('Т2 Активная'!C13/'Т2 Активная'!D21,0)</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>IFERROR('Т3 Сквер'!D13/'Т3 Сквер'!C22,0)</f>
+        <f>IFERROR('Т3 Сквер'!C13/'Т3 Сквер'!D22,0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR('Т4 Sphere Park'!D14/'Т4 Sphere Park'!C23,0)</f>
+        <f>IFERROR('Т4 Sphere Park'!C14/'Т4 Sphere Park'!D23,0)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
+          <t>Покрытие OPEX, по середине вилок</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>IFERROR(AVERAGE('Т1 Транзитная'!C11:D11)/AVERAGE('Т1 Транзитная'!C18:D18),0)</f>
+        <v/>
+      </c>
+      <c r="C19" s="10">
+        <f>IFERROR(AVERAGE('Т2 Активная'!C13:D13)/AVERAGE('Т2 Активная'!C21:D21),0)</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>IFERROR(AVERAGE('Т3 Сквер'!C13:D13)/AVERAGE('Т3 Сквер'!C22:D22),0)</f>
+        <v/>
+      </c>
+      <c r="E19" s="10">
+        <f>IFERROR(AVERAGE('Т4 Sphere Park'!C14:D14)/AVERAGE('Т4 Sphere Park'!C23:D23),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Покрытие OPEX, оптимистично</t>
+        </is>
+      </c>
+      <c r="B20" s="10">
+        <f>IFERROR('Т1 Транзитная'!D11/'Т1 Транзитная'!C18,0)</f>
+        <v/>
+      </c>
+      <c r="C20" s="10">
+        <f>IFERROR('Т2 Активная'!D13/'Т2 Активная'!C21,0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="10">
+        <f>IFERROR('Т3 Сквер'!D13/'Т3 Сквер'!C22,0)</f>
+        <v/>
+      </c>
+      <c r="E20" s="10">
+        <f>IFERROR('Т4 Sphere Park'!D14/'Т4 Sphere Park'!C23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>40–70%</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>70–100%</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026. CAPEX Sphere Park (~2,2 млрд тг, BTO) компенсируется бюджетом отдельно и в операционные модели не входит.</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
+    <row r="24"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A23:E24"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A21:E22"/>
-    <mergeCell ref="A4:E6"/>
+    <mergeCell ref="A4:E7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1142,7 +1222,7 @@
         <v>2500</v>
       </c>
       <c r="F4" s="18">
-        <f>E4*Нормативы!$C$17</f>
+        <f>E4*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G4" s="19" t="inlineStr">
@@ -1179,7 +1259,7 @@
         <v>1700</v>
       </c>
       <c r="F5" s="18">
-        <f>E5*Нормативы!$C$17</f>
+        <f>E5*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G5" s="21" t="inlineStr">
@@ -1216,7 +1296,7 @@
         <v>1600</v>
       </c>
       <c r="F6" s="18">
-        <f>E6*Нормативы!$C$17</f>
+        <f>E6*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G6" s="19" t="inlineStr">
@@ -1253,7 +1333,7 @@
         <v>6200</v>
       </c>
       <c r="F7" s="18">
-        <f>E7*Нормативы!$C$17</f>
+        <f>E7*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G7" s="22" t="inlineStr">
@@ -1290,7 +1370,7 @@
         <v>800</v>
       </c>
       <c r="F8" s="18">
-        <f>E8*Нормативы!$C$17</f>
+        <f>E8*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G8" s="22" t="inlineStr">
@@ -1327,7 +1407,7 @@
         <v>4000</v>
       </c>
       <c r="F9" s="18">
-        <f>E9*Нормативы!$C$17</f>
+        <f>E9*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G9" s="21" t="inlineStr">
@@ -1364,7 +1444,7 @@
         <v>2300</v>
       </c>
       <c r="F10" s="18">
-        <f>E10*Нормативы!$C$17</f>
+        <f>E10*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G10" s="22" t="inlineStr">
@@ -1401,7 +1481,7 @@
         <v>338</v>
       </c>
       <c r="F11" s="18">
-        <f>E11*Нормативы!$C$17</f>
+        <f>E11*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G11" s="21" t="inlineStr">
@@ -1438,7 +1518,7 @@
         <v>338</v>
       </c>
       <c r="F12" s="18">
-        <f>E12*Нормативы!$C$17</f>
+        <f>E12*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G12" s="21" t="inlineStr">
@@ -1475,7 +1555,7 @@
         <v>2385</v>
       </c>
       <c r="F13" s="18">
-        <f>E13*Нормативы!$C$17</f>
+        <f>E13*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G13" s="22" t="inlineStr">
@@ -1512,7 +1592,7 @@
         <v>6800</v>
       </c>
       <c r="F14" s="18">
-        <f>E14*Нормативы!$C$17</f>
+        <f>E14*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G14" s="19" t="inlineStr">
@@ -1549,7 +1629,7 @@
         <v>2930</v>
       </c>
       <c r="F15" s="18">
-        <f>E15*Нормативы!$C$17</f>
+        <f>E15*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G15" s="19" t="inlineStr">
@@ -1586,7 +1666,7 @@
         <v>3650</v>
       </c>
       <c r="F16" s="18">
-        <f>E16*Нормативы!$C$17</f>
+        <f>E16*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G16" s="19" t="inlineStr">
@@ -1623,7 +1703,7 @@
         <v>1680</v>
       </c>
       <c r="F17" s="18">
-        <f>E17*Нормативы!$C$17</f>
+        <f>E17*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G17" s="19" t="inlineStr">
@@ -1660,7 +1740,7 @@
         <v>1680</v>
       </c>
       <c r="F18" s="18">
-        <f>E18*Нормативы!$C$17</f>
+        <f>E18*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G18" s="19" t="inlineStr">
@@ -1697,7 +1777,7 @@
         <v>3500</v>
       </c>
       <c r="F19" s="18">
-        <f>E19*Нормативы!$C$17</f>
+        <f>E19*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G19" s="19" t="inlineStr">
@@ -1734,7 +1814,7 @@
         <v>4000</v>
       </c>
       <c r="F20" s="18">
-        <f>E20*Нормативы!$C$17</f>
+        <f>E20*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G20" s="19" t="inlineStr">
@@ -1771,7 +1851,7 @@
         <v>2419</v>
       </c>
       <c r="F21" s="18">
-        <f>E21*Нормативы!$C$17</f>
+        <f>E21*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G21" s="22" t="inlineStr">
@@ -1808,7 +1888,7 @@
         <v>3600</v>
       </c>
       <c r="F22" s="18">
-        <f>E22*Нормативы!$C$17</f>
+        <f>E22*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G22" s="19" t="inlineStr">
@@ -1845,7 +1925,7 @@
         <v>4200</v>
       </c>
       <c r="F23" s="18">
-        <f>E23*Нормативы!$C$17</f>
+        <f>E23*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G23" s="19" t="inlineStr">
@@ -1882,7 +1962,7 @@
         <v>300</v>
       </c>
       <c r="F24" s="18">
-        <f>E24*Нормативы!$C$17</f>
+        <f>E24*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G24" s="19" t="inlineStr">
@@ -1919,7 +1999,7 @@
         <v>680</v>
       </c>
       <c r="F25" s="18">
-        <f>E25*Нормативы!$C$17</f>
+        <f>E25*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G25" s="19" t="inlineStr">
@@ -1956,7 +2036,7 @@
         <v>600</v>
       </c>
       <c r="F26" s="18">
-        <f>E26*Нормативы!$C$17</f>
+        <f>E26*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G26" s="19" t="inlineStr">
@@ -1993,7 +2073,7 @@
         <v>1300</v>
       </c>
       <c r="F27" s="18">
-        <f>E27*Нормативы!$C$17</f>
+        <f>E27*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G27" s="19" t="inlineStr">
@@ -2030,7 +2110,7 @@
         <v>1120</v>
       </c>
       <c r="F28" s="18">
-        <f>E28*Нормативы!$C$17</f>
+        <f>E28*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G28" s="19" t="inlineStr">
@@ -2067,7 +2147,7 @@
         <v>3900</v>
       </c>
       <c r="F29" s="18">
-        <f>E29*Нормативы!$C$17</f>
+        <f>E29*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G29" s="19" t="inlineStr">
@@ -2104,7 +2184,7 @@
         <v>2900</v>
       </c>
       <c r="F30" s="18">
-        <f>E30*Нормативы!$C$17</f>
+        <f>E30*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G30" s="19" t="inlineStr">
@@ -2141,7 +2221,7 @@
         <v>17000</v>
       </c>
       <c r="F31" s="18">
-        <f>E31*Нормативы!$C$17</f>
+        <f>E31*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G31" s="19" t="inlineStr">
@@ -2178,7 +2258,7 @@
         <v>3100</v>
       </c>
       <c r="F32" s="18">
-        <f>E32*Нормативы!$C$17</f>
+        <f>E32*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G32" s="19" t="inlineStr">
@@ -2215,7 +2295,7 @@
         <v>5500</v>
       </c>
       <c r="F33" s="18">
-        <f>E33*Нормативы!$C$17</f>
+        <f>E33*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G33" s="19" t="inlineStr">
@@ -2252,7 +2332,7 @@
         <v>1100</v>
       </c>
       <c r="F34" s="18">
-        <f>E34*Нормативы!$C$17</f>
+        <f>E34*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G34" s="19" t="inlineStr">
@@ -2325,7 +2405,7 @@
         <v>676</v>
       </c>
       <c r="F36" s="18">
-        <f>E36*Нормативы!$C$17</f>
+        <f>E36*Нормативы!$C$18</f>
         <v/>
       </c>
       <c r="G36" s="21" t="inlineStr">
@@ -2354,7 +2434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -2687,53 +2767,65 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>CAPEX активации (разово, план)</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>млн тг, единовременно</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="27" t="n">
+        <v>40</v>
+      </c>
+      <c r="G12" s="27" t="n">
+        <v>40</v>
+      </c>
+      <c r="H12" s="27" t="n">
+        <v>120</v>
+      </c>
+      <c r="I12" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>ОБЩИЕ НОРМАТИВЫ (мин / макс)</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Ставка координатора кластера</t>
-        </is>
-      </c>
-      <c r="B14" s="26" t="inlineStr">
-        <is>
-          <t>тыс тг/мес</t>
-        </is>
-      </c>
-      <c r="C14" s="27" t="n">
-        <v>300</v>
-      </c>
-      <c r="D14" s="27" t="n">
-        <v>420</v>
-      </c>
-      <c r="E14" s="31" t="n"/>
-      <c r="F14" s="31" t="n"/>
-      <c r="G14" s="31" t="n"/>
-      <c r="H14" s="31" t="n"/>
-      <c r="I14" s="31" t="n"/>
-      <c r="J14" s="31" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Цена события с продвижением</t>
+          <t>Ставка координатора кластера</t>
         </is>
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>тыс тг</t>
+          <t>тыс тг/мес</t>
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>95</v>
+        <v>300</v>
       </c>
       <c r="D15" s="27" t="n">
-        <v>130</v>
+        <v>420</v>
       </c>
       <c r="E15" s="31" t="n"/>
       <c r="F15" s="31" t="n"/>
@@ -2745,19 +2837,19 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Ремфонд, доля от прочих статей OPEX</t>
+          <t>Цена события с продвижением</t>
         </is>
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>доля</t>
-        </is>
-      </c>
-      <c r="C16" s="32" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D16" s="32" t="n">
-        <v>0.07000000000000001</v>
+          <t>тыс тг</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="n">
+        <v>95</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>130</v>
       </c>
       <c r="E16" s="31" t="n"/>
       <c r="F16" s="31" t="n"/>
@@ -2769,19 +2861,19 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Коэффициент: общая площадь / озеленение</t>
+          <t>Ремфонд, % в год от активов и вложений</t>
         </is>
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>×</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="33" t="n">
-        <v>2</v>
+          <t>% в год</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D17" s="32" t="n">
+        <v>0.015</v>
       </c>
       <c r="E17" s="31" t="n"/>
       <c r="F17" s="31" t="n"/>
@@ -2790,10 +2882,34 @@
       <c r="I17" s="31" t="n"/>
       <c r="J17" s="31" t="n"/>
     </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Коэффициент: общая площадь / озеленение</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="31" t="n"/>
+      <c r="G18" s="31" t="n"/>
+      <c r="H18" s="31" t="n"/>
+      <c r="I18" s="31" t="n"/>
+      <c r="J18" s="31" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A14:J14"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2801,6 +2917,512 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Активы на балансе · справки застройщиков, август 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Балансовая стоимость по справкам ТОО-застройщиков, млн тг. Ремфонд в моделях = ставка (лист «Нормативы») × (активы объекта + плановый CAPEX активации).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>Объект</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>Покрытия</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Озеленение</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>МАФы</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>Свет</t>
+        </is>
+      </c>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>Полив</t>
+        </is>
+      </c>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Земля</t>
+        </is>
+      </c>
+      <c r="H3" s="35" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="I3" s="34" t="inlineStr">
+        <is>
+          <t>Что на балансе (по справке)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Сквер Авеню 5</t>
+        </is>
+      </c>
+      <c r="B4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="36" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="D4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="37">
+        <f>SUM(B4:G4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="38" t="inlineStr">
+        <is>
+          <t>только озеленение: 458 растений (вяз-изгородь 408 шт, 18 сосен, 11 елей). Света, МАФов и покрытий на балансе нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Аллея ЖК Flora 1</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C5" s="36" t="n">
+        <v>32.11</v>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="F5" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="37">
+        <f>SUM(B5:G5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="38" t="inlineStr">
+        <is>
+          <t>брусчатка 279 м², 1 647 кустарников + 515 многолетников + 49 деревьев, 10 скамеек, 20 светильников, гирлянда 300 м</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Аллея ЖК Flora 2</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>20.68</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="F6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="37">
+        <f>SUM(B6:G6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="38" t="inlineStr">
+        <is>
+          <t>брусчатка 226 м², 1 087 кустарников + 34 дерева, 8 скамеек, 20 светильников, гирлянда 480 м</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Аллея Хедлайнер Эксклюзив</t>
+        </is>
+      </c>
+      <c r="B7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="37">
+        <f>SUM(B7:G7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="38" t="inlineStr">
+        <is>
+          <t>СПРАВКА ЗАПРОШЕНА у застройщика — внести после нулевого спринта (жёлтые ячейки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Аура Аллея</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="F8" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="37">
+        <f>SUM(B8:G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="38" t="inlineStr">
+        <is>
+          <t>брусчатка 2 000 м², 2 226 кустарников + 42 дерева, 11 скамеек, 14 светильников 3,5 м, гирлянда 250 м</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Аллея Nexpo Классик</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>53.75</v>
+      </c>
+      <c r="E9" s="36" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F9" s="36" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="G9" s="36" t="n">
+        <v>57.09</v>
+      </c>
+      <c r="H9" s="37">
+        <f>SUM(B9:G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="38" t="inlineStr">
+        <is>
+          <t>детское ядро: две горки (26,2 и 14,5 млн), карусель, батут, качели, тренажёр; автополив Hunter/Grundfos; земля 0,37 га</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Аллея Гранд Туран Комфорт</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>43.81</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>46.89</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>29.55</v>
+      </c>
+      <c r="E10" s="36" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="F10" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="37">
+        <f>SUM(B10:G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="38" t="inlineStr">
+        <is>
+          <t>спецификация: покрытия ~5 200 м², 10 игровых комплексов, 27 скамеек, 21 урна, 23 опоры света (материалы, без НДС)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Плейхаб Аква 1</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>23</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F11" s="36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G11" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="37">
+        <f>SUM(B11:G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="38" t="inlineStr">
+        <is>
+          <t>спортядро: огороженное поле 312 м² искусственной травы (борт 5 м), баскетбол, воркаут-серия, 4 вида качелей, канатный лаз</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Аллея Nexpo Юнион</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>16.52</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>52.11</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="F12" s="36" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G12" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="37">
+        <f>SUM(B12:G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="38" t="inlineStr">
+        <is>
+          <t>игровой комплекс 42 млн (тартан, скалодром, тоннели), воркаут, теннисный стол, 54 светильника, автополив</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Фридом — Зелёный Квартал</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="37">
+        <f>SUM(B13:G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="38" t="inlineStr">
+        <is>
+          <t>справка без стоимостей: 47 деревьев (сосна, осина, клён) — вне шорт-листа</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>Итого шорт-лист (9 объектов)</t>
+        </is>
+      </c>
+      <c r="B15" s="41">
+        <f>SUM(B4:B12)</f>
+        <v/>
+      </c>
+      <c r="C15" s="41">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+      <c r="D15" s="41">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E15" s="41">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F15" s="41">
+        <f>SUM(F4:F12)</f>
+        <v/>
+      </c>
+      <c r="G15" s="41">
+        <f>SUM(G4:G12)</f>
+        <v/>
+      </c>
+      <c r="H15" s="41">
+        <f>SUM(H4:H12)</f>
+        <v/>
+      </c>
+      <c r="I15" s="42" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
+        </is>
+      </c>
+      <c r="B16" s="43">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C16" s="43">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D16" s="43">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E16" s="43">
+        <f>E5+E6</f>
+        <v/>
+      </c>
+      <c r="F16" s="43">
+        <f>F5+F6</f>
+        <v/>
+      </c>
+      <c r="G16" s="43">
+        <f>G5+G6</f>
+        <v/>
+      </c>
+      <c r="H16" s="44">
+        <f>SUM(B16:G16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="45" t="inlineStr">
+        <is>
+          <t>строка для выпадающего списка Т1: сумма двух Flora</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2816,40 +3438,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>Финмодель Т1 · Транзитная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
+      <c r="C3" s="49" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="38">
+      <c r="D3" s="50">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="37" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Активы на балансе, млн тг:</t>
+        </is>
+      </c>
+      <c r="B4" s="51">
+        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="38">
+      <c r="D4" s="50">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -2877,7 +3508,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="52" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -2941,23 +3572,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="40" t="inlineStr">
+      <c r="A11" s="53" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B11" s="41" t="n"/>
-      <c r="C11" s="42">
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="54">
         <f>SUM(C8:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="42">
+      <c r="D11" s="54">
         <f>SUM(D8:D10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="inlineStr">
+      <c r="A12" s="52" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -2977,11 +3608,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C13" s="43">
+      <c r="C13" s="55">
         <f>$D$4*Нормативы!C5*12/1000000</f>
         <v/>
       </c>
-      <c r="D13" s="43">
+      <c r="D13" s="55">
         <f>$D$4*Нормативы!D5*12/1000000</f>
         <v/>
       </c>
@@ -2997,11 +3628,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="55">
         <f>$D$3*Нормативы!C6*7/1000000</f>
         <v/>
       </c>
-      <c r="D14" s="43">
+      <c r="D14" s="55">
         <f>$D$3*Нормативы!D6*7/1000000</f>
         <v/>
       </c>
@@ -3017,11 +3648,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="55">
         <f>$D$4*Нормативы!C7/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="43">
+      <c r="D15" s="55">
         <f>$D$4*Нормативы!D7/1000000</f>
         <v/>
       </c>
@@ -3037,12 +3668,12 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="43">
-        <f>Нормативы!$C$14*Нормативы!C8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D16" s="43">
-        <f>Нормативы!$D$14*Нормативы!D8*12/1000</f>
+      <c r="C16" s="55">
+        <f>Нормативы!$C$15*Нормативы!C8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D16" s="55">
+        <f>Нормативы!$D$15*Нормативы!D8*12/1000</f>
         <v/>
       </c>
     </row>
@@ -3054,36 +3685,36 @@
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>доля от прочих статей OPEX</t>
-        </is>
-      </c>
-      <c r="C17" s="43">
-        <f>Нормативы!$C$16*SUM(C13:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="43">
-        <f>Нормативы!$D$16*SUM(D13:D16)</f>
+          <t>% в год от активов на балансе + CAPEX активации</t>
+        </is>
+      </c>
+      <c r="C17" s="55">
+        <f>Нормативы!$C$17*($B$4+Нормативы!C12)</f>
+        <v/>
+      </c>
+      <c r="D17" s="55">
+        <f>Нормативы!$D$17*($B$4+Нормативы!D12)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="44" t="inlineStr">
+      <c r="A18" s="56" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B18" s="41" t="n"/>
-      <c r="C18" s="45">
+      <c r="B18" s="42" t="n"/>
+      <c r="C18" s="57">
         <f>SUM(C13:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="45">
+      <c r="D18" s="57">
         <f>SUM(D13:D17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="39" t="inlineStr">
+      <c r="A20" s="52" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -3103,7 +3734,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C21" s="46">
+      <c r="C21" s="58">
         <f>IFERROR(C11/D18,0)</f>
         <v/>
       </c>
@@ -3120,7 +3751,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C22" s="46">
+      <c r="C22" s="58">
         <f>IFERROR(AVERAGE(C11:D11)/AVERAGE(C18:D18),0)</f>
         <v/>
       </c>
@@ -3137,20 +3768,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C23" s="46">
+      <c r="C23" s="58">
         <f>IFERROR(D11/C18,0)</f>
         <v/>
       </c>
       <c r="D23" s="31" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="47" t="inlineStr">
+      <c r="A24" s="59" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B24" s="31" t="n"/>
-      <c r="C24" s="48" t="inlineStr">
+      <c r="C24" s="60" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
@@ -3158,7 +3789,7 @@
       <c r="D24" s="31" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="39" t="inlineStr">
+      <c r="A26" s="52" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -3168,21 +3799,21 @@
       <c r="D26" s="31" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="49" t="inlineStr">
+      <c r="A27" s="61" t="inlineStr">
         <is>
           <t>• Кластер: общий координатор и бригада, не своя</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="49" t="inlineStr">
+      <c r="A28" s="61" t="inlineStr">
         <is>
           <t>• Спонсоры продлеваются на второй год</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="49" t="inlineStr">
+      <c r="A29" s="61" t="inlineStr">
         <is>
           <t>• Юрстатус пропускает рекламу на стелах</t>
         </is>
@@ -3207,479 +3838,6 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A31:D32"/>
     <mergeCell ref="A28:D28"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$36</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="34" t="inlineStr">
-        <is>
-          <t>Финмодель Т2 · Активная аллея</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="35" t="inlineStr">
-        <is>
-          <t>Объект (выберите из списка):</t>
-        </is>
-      </c>
-      <c r="B3" s="36" t="inlineStr">
-        <is>
-          <t>Аллея Хедлайнер Эксклюзив</t>
-        </is>
-      </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>Озеленение, м²:</t>
-        </is>
-      </c>
-      <c r="D3" s="38">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" s="37" t="inlineStr">
-        <is>
-          <t>Общая площадь, м²:</t>
-        </is>
-      </c>
-      <c r="D4" s="38">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Как считаем / привязка</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Мин, млн тг/год</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Макс, млн тг/год</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="39" t="inlineStr">
-        <is>
-          <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
-        </is>
-      </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>НТО-якорь: кофе-павильон</t>
-        </is>
-      </c>
-      <c r="B8" s="26" t="inlineStr">
-        <is>
-          <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Ярмарка выходного дня</t>
-        </is>
-      </c>
-      <c r="B9" s="26" t="inlineStr">
-        <is>
-          <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Секции и кикшеринг</t>
-        </is>
-      </c>
-      <c r="B10" s="26" t="inlineStr">
-        <is>
-          <t>слоты тренерам + rev-share операторов</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D10" s="33" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Digital-экран и реклама</t>
-        </is>
-      </c>
-      <c r="B11" s="26" t="inlineStr">
-        <is>
-          <t>при подходящем юрстатусе земли</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D11" s="33" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Спонсорство объектов</t>
-        </is>
-      </c>
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>воркаут, клумбы, скамейки</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>Доходы, итого</t>
-        </is>
-      </c>
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="42">
-        <f>SUM(C8:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="42">
-        <f>SUM(D8:D12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="39" t="inlineStr">
-        <is>
-          <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
-        </is>
-      </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Уборка и снегоуборка</t>
-        </is>
-      </c>
-      <c r="B15" s="26" t="inlineStr">
-        <is>
-          <t>общая площадь × норматив × 12 мес</t>
-        </is>
-      </c>
-      <c r="C15" s="43">
-        <f>$D$4*Нормативы!E5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="43">
-        <f>$D$4*Нормативы!F5*12/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Озеленение и полив</t>
-        </is>
-      </c>
-      <c r="B16" s="26" t="inlineStr">
-        <is>
-          <t>озеленение × норматив × 7 мес (апр–окт)</t>
-        </is>
-      </c>
-      <c r="C16" s="43">
-        <f>$D$3*Нормативы!E6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="43">
-        <f>$D$3*Нормативы!F6*7/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Свет, электро, digital</t>
-        </is>
-      </c>
-      <c r="B17" s="26" t="inlineStr">
-        <is>
-          <t>общая площадь × годовой норматив</t>
-        </is>
-      </c>
-      <c r="C17" s="43">
-        <f>$D$4*Нормативы!E7/1000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="43">
-        <f>$D$4*Нормативы!F7/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Программа и маркетинг</t>
-        </is>
-      </c>
-      <c r="B18" s="26" t="inlineStr">
-        <is>
-          <t>число событий × цена события</t>
-        </is>
-      </c>
-      <c r="C18" s="43">
-        <f>Нормативы!E9*Нормативы!$C$15/1000</f>
-        <v/>
-      </c>
-      <c r="D18" s="43">
-        <f>Нормативы!F9*Нормативы!$D$15/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Координатор кластера</t>
-        </is>
-      </c>
-      <c r="B19" s="26" t="inlineStr">
-        <is>
-          <t>ставка × доля × 12 мес</t>
-        </is>
-      </c>
-      <c r="C19" s="43">
-        <f>Нормативы!$C$14*Нормативы!E8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D19" s="43">
-        <f>Нормативы!$D$14*Нормативы!F8*12/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Ремфонд</t>
-        </is>
-      </c>
-      <c r="B20" s="26" t="inlineStr">
-        <is>
-          <t>доля от прочих статей OPEX</t>
-        </is>
-      </c>
-      <c r="C20" s="43">
-        <f>Нормативы!$C$16*SUM(C15:C19)</f>
-        <v/>
-      </c>
-      <c r="D20" s="43">
-        <f>Нормативы!$D$16*SUM(D15:D19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="44" t="inlineStr">
-        <is>
-          <t>OPEX, итого</t>
-        </is>
-      </c>
-      <c r="B21" s="41" t="n"/>
-      <c r="C21" s="45">
-        <f>SUM(C15:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="45">
-        <f>SUM(D15:D20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="39" t="inlineStr">
-        <is>
-          <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
-        </is>
-      </c>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="31" t="n"/>
-      <c r="D23" s="31" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Консервативный сценарий</t>
-        </is>
-      </c>
-      <c r="B24" s="26" t="inlineStr">
-        <is>
-          <t>низ доходов / верх расходов</t>
-        </is>
-      </c>
-      <c r="C24" s="46">
-        <f>IFERROR(C13/D21,0)</f>
-        <v/>
-      </c>
-      <c r="D24" s="31" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>По середине вилок</t>
-        </is>
-      </c>
-      <c r="B25" s="26" t="inlineStr">
-        <is>
-          <t>средние значения обеих вилок</t>
-        </is>
-      </c>
-      <c r="C25" s="46">
-        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
-        <v/>
-      </c>
-      <c r="D25" s="31" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Оптимистичный сценарий</t>
-        </is>
-      </c>
-      <c r="B26" s="26" t="inlineStr">
-        <is>
-          <t>верх доходов / низ расходов</t>
-        </is>
-      </c>
-      <c r="C26" s="46">
-        <f>IFERROR(D13/C21,0)</f>
-        <v/>
-      </c>
-      <c r="D26" s="31" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="47" t="inlineStr">
-        <is>
-          <t>Целевой коридор пилота</t>
-        </is>
-      </c>
-      <c r="B27" s="31" t="n"/>
-      <c r="C27" s="48" t="inlineStr">
-        <is>
-          <t>40–70%</t>
-        </is>
-      </c>
-      <c r="D27" s="31" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="39" t="inlineStr">
-        <is>
-          <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
-        </is>
-      </c>
-      <c r="B29" s="31" t="n"/>
-      <c r="C29" s="31" t="n"/>
-      <c r="D29" s="31" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="49" t="inlineStr">
-        <is>
-          <t>• Якорь-павильон заполнен с мая по сентябрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="49" t="inlineStr">
-        <is>
-          <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="49" t="inlineStr">
-        <is>
-          <t>• Вечерние слоты секций выкуплены</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
-        <is>
-          <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A34:D35"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -3706,40 +3864,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
-        <is>
-          <t>Финмодель Т3 · Сквер / плейхаб</t>
+      <c r="A1" s="46" t="inlineStr">
+        <is>
+          <t>Финмодель Т2 · Активная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
-        <is>
-          <t>Сквер Авеню 5</t>
-        </is>
-      </c>
-      <c r="C3" s="37" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>Аллея Хедлайнер Эксклюзив</t>
+        </is>
+      </c>
+      <c r="C3" s="49" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="38">
+      <c r="D3" s="50">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="37" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Активы на балансе, млн тг:</t>
+        </is>
+      </c>
+      <c r="B4" s="51">
+        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="38">
+      <c r="D4" s="50">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -3767,7 +3934,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="52" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -3779,111 +3946,111 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Две НТО-точки</t>
+          <t>НТО-якорь: кофе-павильон</t>
         </is>
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>кофе и выпечка: аренда + % оборота</t>
+          <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Каток: прокат и билеты</t>
+          <t>Ярмарка выходного дня</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>компактный контур, 120–160 дней</t>
+          <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>3.5</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Событийная аренда</t>
+          <t>Секции и кикшеринг</t>
         </is>
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>10–18 частных и корпоративных событий</t>
+          <t>слоты тренерам + rev-share операторов</t>
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Ярмарки, маркеты, секции</t>
+          <t>Digital-экран и реклама</t>
         </is>
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>круглогодичный календарь</t>
+          <t>при подходящем юрстатусе земли</t>
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Спонсор года и реклама</t>
+          <t>Спонсорство объектов</t>
         </is>
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>один якорный партнёр + экран</t>
+          <t>воркаут, клумбы, скамейки</t>
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="40" t="inlineStr">
+      <c r="A13" s="53" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="42">
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="54">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="42">
+      <c r="D13" s="54">
         <f>SUM(D8:D12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="39" t="inlineStr">
+      <c r="A14" s="52" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -3903,12 +4070,12 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C15" s="43">
-        <f>$D$4*Нормативы!G5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="43">
-        <f>$D$4*Нормативы!H5*12/1000000</f>
+      <c r="C15" s="55">
+        <f>$D$4*Нормативы!E5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="55">
+        <f>$D$4*Нормативы!F5*12/1000000</f>
         <v/>
       </c>
     </row>
@@ -3923,12 +4090,12 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C16" s="43">
-        <f>$D$3*Нормативы!G6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="43">
-        <f>$D$3*Нормативы!H6*7/1000000</f>
+      <c r="C16" s="55">
+        <f>$D$3*Нормативы!E6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="55">
+        <f>$D$3*Нормативы!F6*7/1000000</f>
         <v/>
       </c>
     </row>
@@ -3943,58 +4110,548 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C17" s="43">
-        <f>$D$4*Нормативы!G7/1000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="43">
-        <f>$D$4*Нормативы!H7/1000000</f>
+      <c r="C17" s="55">
+        <f>$D$4*Нормативы!E7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="55">
+        <f>$D$4*Нормативы!F7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Зимний пакет</t>
+          <t>Программа и маркетинг</t>
         </is>
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>норматив, млн тг/год</t>
-        </is>
-      </c>
-      <c r="C18" s="43">
-        <f>Нормативы!G10</f>
-        <v/>
-      </c>
-      <c r="D18" s="43">
-        <f>Нормативы!H10</f>
+          <t>число событий × цена события</t>
+        </is>
+      </c>
+      <c r="C18" s="55">
+        <f>Нормативы!E9*Нормативы!$C$16/1000</f>
+        <v/>
+      </c>
+      <c r="D18" s="55">
+        <f>Нормативы!F9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Программа и маркетинг</t>
+          <t>Координатор кластера</t>
         </is>
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>число событий × цена события</t>
-        </is>
-      </c>
-      <c r="C19" s="43">
-        <f>Нормативы!G9*Нормативы!$C$15/1000</f>
-        <v/>
-      </c>
-      <c r="D19" s="43">
-        <f>Нормативы!H9*Нормативы!$D$15/1000</f>
+          <t>ставка × доля × 12 мес</t>
+        </is>
+      </c>
+      <c r="C19" s="55">
+        <f>Нормативы!$C$15*Нормативы!E8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="55">
+        <f>Нормативы!$D$15*Нормативы!F8*12/1000</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>Ремфонд</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>% в год от активов на балансе + CAPEX активации</t>
+        </is>
+      </c>
+      <c r="C20" s="55">
+        <f>Нормативы!$C$17*($B$4+Нормативы!E12)</f>
+        <v/>
+      </c>
+      <c r="D20" s="55">
+        <f>Нормативы!$D$17*($B$4+Нормативы!F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="56" t="inlineStr">
+        <is>
+          <t>OPEX, итого</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="n"/>
+      <c r="C21" s="57">
+        <f>SUM(C15:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="57">
+        <f>SUM(D15:D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="52" t="inlineStr">
+        <is>
+          <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="31" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Консервативный сценарий</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>низ доходов / верх расходов</t>
+        </is>
+      </c>
+      <c r="C24" s="58">
+        <f>IFERROR(C13/D21,0)</f>
+        <v/>
+      </c>
+      <c r="D24" s="31" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>По середине вилок</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>средние значения обеих вилок</t>
+        </is>
+      </c>
+      <c r="C25" s="58">
+        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
+        <v/>
+      </c>
+      <c r="D25" s="31" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Оптимистичный сценарий</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>верх доходов / низ расходов</t>
+        </is>
+      </c>
+      <c r="C26" s="58">
+        <f>IFERROR(D13/C21,0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="59" t="inlineStr">
+        <is>
+          <t>Целевой коридор пилота</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="60" t="inlineStr">
+        <is>
+          <t>40–70%</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="52" t="inlineStr">
+        <is>
+          <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="31" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="61" t="inlineStr">
+        <is>
+          <t>• Справка по активам Хедлайнера получена, суммы внесены в лист «Активы»</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="61" t="inlineStr">
+        <is>
+          <t>• Якорь-павильон заполнен с мая по сентябрь</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="61" t="inlineStr">
+        <is>
+          <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="61" t="inlineStr">
+        <is>
+          <t>• Вечерние слоты секций выкуплены</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A35:D36"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=Объекты!$B$4:$B$36</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="46" t="inlineStr">
+        <is>
+          <t>Финмодель Т3 · Сквер / плейхаб</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>Объект (выберите из списка):</t>
+        </is>
+      </c>
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>Сквер Авеню 5</t>
+        </is>
+      </c>
+      <c r="C3" s="49" t="inlineStr">
+        <is>
+          <t>Озеленение, м²:</t>
+        </is>
+      </c>
+      <c r="D3" s="50">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Активы на балансе, млн тг:</t>
+        </is>
+      </c>
+      <c r="B4" s="51">
+        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>Общая площадь, м²:</t>
+        </is>
+      </c>
+      <c r="D4" s="50">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Как считаем / привязка</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Мин, млн тг/год</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Макс, млн тг/год</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="52" t="inlineStr">
+        <is>
+          <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Две НТО-точки</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>кофе и выпечка: аренда + % оборота</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Каток: прокат и билеты</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>компактный контур, 120–160 дней</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Событийная аренда</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>10–18 частных и корпоративных событий</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="33" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Ярмарки, маркеты, секции</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>круглогодичный календарь</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Спонсор года и реклама</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>один якорный партнёр + экран</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="53" t="inlineStr">
+        <is>
+          <t>Доходы, итого</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="54">
+        <f>SUM(C8:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="54">
+        <f>SUM(D8:D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Уборка и снегоуборка</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × норматив × 12 мес</t>
+        </is>
+      </c>
+      <c r="C15" s="55">
+        <f>$D$4*Нормативы!G5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="55">
+        <f>$D$4*Нормативы!H5*12/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Озеленение и полив</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>озеленение × норматив × 7 мес (апр–окт)</t>
+        </is>
+      </c>
+      <c r="C16" s="55">
+        <f>$D$3*Нормативы!G6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="55">
+        <f>$D$3*Нормативы!H6*7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Свет, электро, digital</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>общая площадь × годовой норматив</t>
+        </is>
+      </c>
+      <c r="C17" s="55">
+        <f>$D$4*Нормативы!G7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="55">
+        <f>$D$4*Нормативы!H7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Зимний пакет</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>норматив, млн тг/год</t>
+        </is>
+      </c>
+      <c r="C18" s="55">
+        <f>Нормативы!G10</f>
+        <v/>
+      </c>
+      <c r="D18" s="55">
+        <f>Нормативы!H10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Программа и маркетинг</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>число событий × цена события</t>
+        </is>
+      </c>
+      <c r="C19" s="55">
+        <f>Нормативы!G9*Нормативы!$C$16/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="55">
+        <f>Нормативы!H9*Нормативы!$D$16/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t>Координатор кластера</t>
         </is>
       </c>
@@ -4003,12 +4660,12 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C20" s="43">
-        <f>Нормативы!$C$14*Нормативы!G8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D20" s="43">
-        <f>Нормативы!$D$14*Нормативы!H8*12/1000</f>
+      <c r="C20" s="55">
+        <f>Нормативы!$C$15*Нормативы!G8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D20" s="55">
+        <f>Нормативы!$D$15*Нормативы!H8*12/1000</f>
         <v/>
       </c>
     </row>
@@ -4020,36 +4677,36 @@
       </c>
       <c r="B21" s="26" t="inlineStr">
         <is>
-          <t>доля от прочих статей OPEX</t>
-        </is>
-      </c>
-      <c r="C21" s="43">
-        <f>Нормативы!$C$16*SUM(C15:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="43">
-        <f>Нормативы!$D$16*SUM(D15:D20)</f>
+          <t>% в год от активов на балансе + CAPEX активации</t>
+        </is>
+      </c>
+      <c r="C21" s="55">
+        <f>Нормативы!$C$17*($B$4+Нормативы!G12)</f>
+        <v/>
+      </c>
+      <c r="D21" s="55">
+        <f>Нормативы!$D$17*($B$4+Нормативы!H12)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B22" s="41" t="n"/>
-      <c r="C22" s="45">
+      <c r="B22" s="42" t="n"/>
+      <c r="C22" s="57">
         <f>SUM(C15:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="45">
+      <c r="D22" s="57">
         <f>SUM(D15:D21)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="39" t="inlineStr">
+      <c r="A24" s="52" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -4069,7 +4726,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C25" s="46">
+      <c r="C25" s="58">
         <f>IFERROR(C13/D22,0)</f>
         <v/>
       </c>
@@ -4086,7 +4743,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="58">
         <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C22:D22),0)</f>
         <v/>
       </c>
@@ -4103,20 +4760,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C27" s="46">
+      <c r="C27" s="58">
         <f>IFERROR(D13/C22,0)</f>
         <v/>
       </c>
       <c r="D27" s="31" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="47" t="inlineStr">
+      <c r="A28" s="59" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B28" s="31" t="n"/>
-      <c r="C28" s="48" t="inlineStr">
+      <c r="C28" s="60" t="inlineStr">
         <is>
           <t>70–100%</t>
         </is>
@@ -4124,7 +4781,7 @@
       <c r="D28" s="31" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="39" t="inlineStr">
+      <c r="A30" s="52" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -4134,21 +4791,21 @@
       <c r="D30" s="31" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="49" t="inlineStr">
+      <c r="A31" s="61" t="inlineStr">
         <is>
           <t>• Каток отработал первую зиму без простоев</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="49" t="inlineStr">
+      <c r="A32" s="61" t="inlineStr">
         <is>
           <t>• Заявок на события больше, чем слотов</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="49" t="inlineStr">
+      <c r="A33" s="61" t="inlineStr">
         <is>
           <t>• Спонсор года подписан до старта сезона</t>
         </is>
@@ -4183,13 +4840,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4199,40 +4856,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>Финмодель Т4 · Парк по ГЧП (BTO)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
         <is>
           <t>Sphere Park</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
+      <c r="C3" s="49" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="38">
+      <c r="D3" s="50">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="37" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Активы на балансе, млн тг:</t>
+        </is>
+      </c>
+      <c r="B4" s="51">
+        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="38">
+      <c r="D4" s="50">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -4260,7 +4926,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="52" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -4378,23 +5044,23 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="40" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B14" s="41" t="n"/>
-      <c r="C14" s="42">
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="54">
         <f>SUM(C8:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="42">
+      <c r="D14" s="54">
         <f>SUM(D8:D13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="39" t="inlineStr">
+      <c r="A15" s="52" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -4414,11 +5080,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="43">
+      <c r="C16" s="55">
         <f>$D$4*Нормативы!I5*12/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="43">
+      <c r="D16" s="55">
         <f>$D$4*Нормативы!J5*12/1000000</f>
         <v/>
       </c>
@@ -4434,11 +5100,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C17" s="43">
+      <c r="C17" s="55">
         <f>$D$3*Нормативы!I6*7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="43">
+      <c r="D17" s="55">
         <f>$D$3*Нормативы!J6*7/1000000</f>
         <v/>
       </c>
@@ -4454,11 +5120,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C18" s="43">
+      <c r="C18" s="55">
         <f>$D$4*Нормативы!I7/1000000</f>
         <v/>
       </c>
-      <c r="D18" s="43">
+      <c r="D18" s="55">
         <f>$D$4*Нормативы!J7/1000000</f>
         <v/>
       </c>
@@ -4474,11 +5140,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C19" s="43">
+      <c r="C19" s="55">
         <f>Нормативы!I10</f>
         <v/>
       </c>
-      <c r="D19" s="43">
+      <c r="D19" s="55">
         <f>Нормативы!J10</f>
         <v/>
       </c>
@@ -4494,12 +5160,12 @@
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C20" s="43">
-        <f>Нормативы!I9*Нормативы!$C$15/1000</f>
-        <v/>
-      </c>
-      <c r="D20" s="43">
-        <f>Нормативы!J9*Нормативы!$D$15/1000</f>
+      <c r="C20" s="55">
+        <f>Нормативы!I9*Нормативы!$C$16/1000</f>
+        <v/>
+      </c>
+      <c r="D20" s="55">
+        <f>Нормативы!J9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
     </row>
@@ -4514,11 +5180,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C21" s="43">
+      <c r="C21" s="55">
         <f>Нормативы!I11</f>
         <v/>
       </c>
-      <c r="D21" s="43">
+      <c r="D21" s="55">
         <f>Нормативы!J11</f>
         <v/>
       </c>
@@ -4531,36 +5197,36 @@
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>доля от прочих статей OPEX</t>
-        </is>
-      </c>
-      <c r="C22" s="43">
-        <f>Нормативы!$C$16*SUM(C16:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="43">
-        <f>Нормативы!$D$16*SUM(D16:D21)</f>
+          <t>% в год от активов на балансе + CAPEX активации</t>
+        </is>
+      </c>
+      <c r="C22" s="55">
+        <f>Нормативы!$C$17*($B$4+Нормативы!I12)</f>
+        <v/>
+      </c>
+      <c r="D22" s="55">
+        <f>Нормативы!$D$17*($B$4+Нормативы!J12)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="44" t="inlineStr">
+      <c r="A23" s="56" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B23" s="41" t="n"/>
-      <c r="C23" s="45">
+      <c r="B23" s="42" t="n"/>
+      <c r="C23" s="57">
         <f>SUM(C16:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="45">
+      <c r="D23" s="57">
         <f>SUM(D16:D22)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="39" t="inlineStr">
+      <c r="A25" s="52" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -4580,7 +5246,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="58">
         <f>IFERROR(C14/D23,0)</f>
         <v/>
       </c>
@@ -4597,7 +5263,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C27" s="46">
+      <c r="C27" s="58">
         <f>IFERROR(AVERAGE(C14:D14)/AVERAGE(C23:D23),0)</f>
         <v/>
       </c>
@@ -4614,20 +5280,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C28" s="46">
+      <c r="C28" s="58">
         <f>IFERROR(D14/C23,0)</f>
         <v/>
       </c>
       <c r="D28" s="31" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="47" t="inlineStr">
+      <c r="A29" s="59" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B29" s="31" t="n"/>
-      <c r="C29" s="48" t="inlineStr">
+      <c r="C29" s="60" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
@@ -4635,7 +5301,7 @@
       <c r="D29" s="31" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="39" t="inlineStr">
+      <c r="A31" s="52" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -4645,53 +5311,61 @@
       <c r="D31" s="31" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="49" t="inlineStr">
+      <c r="A32" s="61" t="inlineStr">
+        <is>
+          <t>• Ремфонд и капремонт сидят в компенсации эксплуатации (BTO), в OPEX не дублируются</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="61" t="inlineStr">
         <is>
           <t>• ГЧП-договор подписан, компенсация в бюджете МИО</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="49" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="61" t="inlineStr">
         <is>
           <t>• Каток и события дотягивают покрытие до 100%+</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="49" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="61" t="inlineStr">
         <is>
           <t>• Стандарт содержания выше городского бенчмарка</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="49" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="61" t="inlineStr">
         <is>
           <t>• CAPEX ~2,2 млрд тг компенсируется бюджетом МИО отдельно (2026–2031) — в операционную модель не входит</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
         </is>
       </c>
     </row>
-    <row r="38"/>
+    <row r="39"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A38:D39"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A37:D38"/>
     <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
Add area columns to assets slide and Assets sheet
Assets slide now shows greenery/total area per shortlist object next to
balance-sheet value; Assets sheet pulls both areas from the object
registry via INDEX/MATCH so they follow the editable coefficient.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014o1yT6nCgffZ5H25q7THst
</commit_message>
<xml_diff>
--- a/docs/research/BIG-Life-finmodels-T1-T4.xlsx
+++ b/docs/research/BIG-Life-finmodels-T1-T4.xlsx
@@ -262,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -356,6 +356,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="166" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -2922,18 +2925,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="72" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9.5" customWidth="1" min="6" max="6"/>
+    <col width="8.5" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9.5" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2958,40 +2963,50 @@
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
+          <t>Озеленение, м²</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Общая, м²</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
           <t>Покрытия</t>
         </is>
       </c>
-      <c r="C3" s="35" t="inlineStr">
-        <is>
-          <t>Озеленение</t>
-        </is>
-      </c>
-      <c r="D3" s="35" t="inlineStr">
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>Насаждения</t>
+        </is>
+      </c>
+      <c r="F3" s="35" t="inlineStr">
         <is>
           <t>МАФы</t>
         </is>
       </c>
-      <c r="E3" s="35" t="inlineStr">
+      <c r="G3" s="35" t="inlineStr">
         <is>
           <t>Свет</t>
         </is>
       </c>
-      <c r="F3" s="35" t="inlineStr">
+      <c r="H3" s="35" t="inlineStr">
         <is>
           <t>Полив</t>
         </is>
       </c>
-      <c r="G3" s="35" t="inlineStr">
+      <c r="I3" s="35" t="inlineStr">
         <is>
           <t>Земля</t>
         </is>
       </c>
-      <c r="H3" s="35" t="inlineStr">
+      <c r="J3" s="35" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="I3" s="34" t="inlineStr">
+      <c r="K3" s="34" t="inlineStr">
         <is>
           <t>Что на балансе (по справке)</t>
         </is>
@@ -3003,17 +3018,19 @@
           <t>Сквер Авеню 5</t>
         </is>
       </c>
-      <c r="B4" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="36" t="n">
-        <v>2.09</v>
+      <c r="B4" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A4,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C4" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A4,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
       </c>
       <c r="D4" s="36" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="36" t="n">
-        <v>0</v>
+        <v>2.09</v>
       </c>
       <c r="F4" s="36" t="n">
         <v>0</v>
@@ -3021,11 +3038,17 @@
       <c r="G4" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="37">
-        <f>SUM(B4:G4)</f>
-        <v/>
-      </c>
-      <c r="I4" s="38" t="inlineStr">
+      <c r="H4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="37">
+        <f>SUM(D4:I4)</f>
+        <v/>
+      </c>
+      <c r="K4" s="38" t="inlineStr">
         <is>
           <t>только озеленение: 458 растений (вяз-изгородь 408 шт, 18 сосен, 11 елей). Света, МАФов и покрытий на балансе нет</t>
         </is>
@@ -3037,29 +3060,37 @@
           <t>Аллея ЖК Flora 1</t>
         </is>
       </c>
-      <c r="B5" s="36" t="n">
+      <c r="B5" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A5,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C5" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A5,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="C5" s="36" t="n">
+      <c r="E5" s="36" t="n">
         <v>32.11</v>
       </c>
-      <c r="D5" s="36" t="n">
+      <c r="F5" s="36" t="n">
         <v>2.23</v>
       </c>
-      <c r="E5" s="36" t="n">
+      <c r="G5" s="36" t="n">
         <v>5.23</v>
       </c>
-      <c r="F5" s="36" t="n">
+      <c r="H5" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="36" t="n">
+      <c r="I5" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="37">
-        <f>SUM(B5:G5)</f>
-        <v/>
-      </c>
-      <c r="I5" s="38" t="inlineStr">
+      <c r="J5" s="37">
+        <f>SUM(D5:I5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="38" t="inlineStr">
         <is>
           <t>брусчатка 279 м², 1 647 кустарников + 515 многолетников + 49 деревьев, 10 скамеек, 20 светильников, гирлянда 300 м</t>
         </is>
@@ -3071,29 +3102,37 @@
           <t>Аллея ЖК Flora 2</t>
         </is>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A6,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C6" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A6,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D6" s="36" t="n">
         <v>2.07</v>
       </c>
-      <c r="C6" s="36" t="n">
+      <c r="E6" s="36" t="n">
         <v>20.68</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="F6" s="36" t="n">
         <v>1.47</v>
       </c>
-      <c r="E6" s="36" t="n">
+      <c r="G6" s="36" t="n">
         <v>5.85</v>
       </c>
-      <c r="F6" s="36" t="n">
+      <c r="H6" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="36" t="n">
+      <c r="I6" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="37">
-        <f>SUM(B6:G6)</f>
-        <v/>
-      </c>
-      <c r="I6" s="38" t="inlineStr">
+      <c r="J6" s="37">
+        <f>SUM(D6:I6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="38" t="inlineStr">
         <is>
           <t>брусчатка 226 м², 1 087 кустарников + 34 дерева, 8 скамеек, 20 светильников, гирлянда 480 м</t>
         </is>
@@ -3105,11 +3144,13 @@
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
       </c>
-      <c r="B7" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="39" t="n">
-        <v>0</v>
+      <c r="B7" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A7,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C7" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A7,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
       </c>
       <c r="D7" s="39" t="n">
         <v>0</v>
@@ -3123,11 +3164,17 @@
       <c r="G7" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="37">
-        <f>SUM(B7:G7)</f>
-        <v/>
-      </c>
-      <c r="I7" s="38" t="inlineStr">
+      <c r="H7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="37">
+        <f>SUM(D7:I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="38" t="inlineStr">
         <is>
           <t>СПРАВКА ЗАПРОШЕНА у застройщика — внести после нулевого спринта (жёлтые ячейки)</t>
         </is>
@@ -3139,29 +3186,37 @@
           <t>Аура Аллея</t>
         </is>
       </c>
-      <c r="B8" s="36" t="n">
+      <c r="B8" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A8,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A8,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="36" t="n">
         <v>14.97</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="E8" s="36" t="n">
         <v>38.65</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="F8" s="36" t="n">
         <v>2.38</v>
       </c>
-      <c r="E8" s="36" t="n">
+      <c r="G8" s="36" t="n">
         <v>4.26</v>
       </c>
-      <c r="F8" s="36" t="n">
+      <c r="H8" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="36" t="n">
+      <c r="I8" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="37">
-        <f>SUM(B8:G8)</f>
-        <v/>
-      </c>
-      <c r="I8" s="38" t="inlineStr">
+      <c r="J8" s="37">
+        <f>SUM(D8:I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="38" t="inlineStr">
         <is>
           <t>брусчатка 2 000 м², 2 226 кустарников + 42 дерева, 11 скамеек, 14 светильников 3,5 м, гирлянда 250 м</t>
         </is>
@@ -3173,29 +3228,37 @@
           <t>Аллея Nexpo Классик</t>
         </is>
       </c>
-      <c r="B9" s="36" t="n">
+      <c r="B9" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A9,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A9,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D9" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="E9" s="36" t="n">
         <v>21.89</v>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="F9" s="36" t="n">
         <v>53.75</v>
       </c>
-      <c r="E9" s="36" t="n">
+      <c r="G9" s="36" t="n">
         <v>1.3</v>
       </c>
-      <c r="F9" s="36" t="n">
+      <c r="H9" s="36" t="n">
         <v>1.34</v>
       </c>
-      <c r="G9" s="36" t="n">
+      <c r="I9" s="36" t="n">
         <v>57.09</v>
       </c>
-      <c r="H9" s="37">
-        <f>SUM(B9:G9)</f>
-        <v/>
-      </c>
-      <c r="I9" s="38" t="inlineStr">
+      <c r="J9" s="37">
+        <f>SUM(D9:I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="38" t="inlineStr">
         <is>
           <t>детское ядро: две горки (26,2 и 14,5 млн), карусель, батут, качели, тренажёр; автополив Hunter/Grundfos; земля 0,37 га</t>
         </is>
@@ -3207,29 +3270,37 @@
           <t>Аллея Гранд Туран Комфорт</t>
         </is>
       </c>
-      <c r="B10" s="36" t="n">
+      <c r="B10" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A10,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A10,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="36" t="n">
         <v>43.81</v>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="E10" s="36" t="n">
         <v>46.89</v>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="F10" s="36" t="n">
         <v>29.55</v>
       </c>
-      <c r="E10" s="36" t="n">
+      <c r="G10" s="36" t="n">
         <v>8.81</v>
       </c>
-      <c r="F10" s="36" t="n">
+      <c r="H10" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="36" t="n">
+      <c r="I10" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="37">
-        <f>SUM(B10:G10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="38" t="inlineStr">
+      <c r="J10" s="37">
+        <f>SUM(D10:I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="38" t="inlineStr">
         <is>
           <t>спецификация: покрытия ~5 200 м², 10 игровых комплексов, 27 скамеек, 21 урна, 23 опоры света (материалы, без НДС)</t>
         </is>
@@ -3241,29 +3312,37 @@
           <t>Плейхаб Аква 1</t>
         </is>
       </c>
-      <c r="B11" s="36" t="n">
+      <c r="B11" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A11,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A11,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="36" t="n">
+      <c r="E11" s="36" t="n">
         <v>6.83</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="F11" s="36" t="n">
         <v>23</v>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="G11" s="36" t="n">
         <v>1.26</v>
       </c>
-      <c r="F11" s="36" t="n">
+      <c r="H11" s="36" t="n">
         <v>0.7</v>
       </c>
-      <c r="G11" s="36" t="n">
+      <c r="I11" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="37">
-        <f>SUM(B11:G11)</f>
-        <v/>
-      </c>
-      <c r="I11" s="38" t="inlineStr">
+      <c r="J11" s="37">
+        <f>SUM(D11:I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="38" t="inlineStr">
         <is>
           <t>спортядро: огороженное поле 312 м² искусственной травы (борт 5 м), баскетбол, воркаут-серия, 4 вида качелей, канатный лаз</t>
         </is>
@@ -3275,29 +3354,37 @@
           <t>Аллея Nexpo Юнион</t>
         </is>
       </c>
-      <c r="B12" s="36" t="n">
+      <c r="B12" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A12,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A12,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="36" t="n">
+      <c r="E12" s="36" t="n">
         <v>16.52</v>
       </c>
-      <c r="D12" s="36" t="n">
+      <c r="F12" s="36" t="n">
         <v>52.11</v>
       </c>
-      <c r="E12" s="36" t="n">
+      <c r="G12" s="36" t="n">
         <v>4.08</v>
       </c>
-      <c r="F12" s="36" t="n">
+      <c r="H12" s="36" t="n">
         <v>0.72</v>
       </c>
-      <c r="G12" s="36" t="n">
+      <c r="I12" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="37">
-        <f>SUM(B12:G12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="38" t="inlineStr">
+      <c r="J12" s="37">
+        <f>SUM(D12:I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="38" t="inlineStr">
         <is>
           <t>игровой комплекс 42 млн (тартан, скалодром, тоннели), воркаут, теннисный стол, 54 светильника, автополив</t>
         </is>
@@ -3309,11 +3396,13 @@
           <t>Фридом — Зелёный Квартал</t>
         </is>
       </c>
-      <c r="B13" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>0</v>
+      <c r="B13" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A13,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A13,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
       </c>
       <c r="D13" s="36" t="n">
         <v>0</v>
@@ -3327,11 +3416,17 @@
       <c r="G13" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="37">
-        <f>SUM(B13:G13)</f>
-        <v/>
-      </c>
-      <c r="I13" s="38" t="inlineStr">
+      <c r="H13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="37">
+        <f>SUM(D13:I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="38" t="inlineStr">
         <is>
           <t>справка без стоимостей: 47 деревьев (сосна, осина, клён) — вне шорт-листа</t>
         </is>
@@ -3351,27 +3446,35 @@
         <f>SUM(C4:C12)</f>
         <v/>
       </c>
-      <c r="D15" s="41">
+      <c r="D15" s="42">
         <f>SUM(D4:D12)</f>
         <v/>
       </c>
-      <c r="E15" s="41">
+      <c r="E15" s="42">
         <f>SUM(E4:E12)</f>
         <v/>
       </c>
-      <c r="F15" s="41">
+      <c r="F15" s="42">
         <f>SUM(F4:F12)</f>
         <v/>
       </c>
-      <c r="G15" s="41">
+      <c r="G15" s="42">
         <f>SUM(G4:G12)</f>
         <v/>
       </c>
-      <c r="H15" s="41">
+      <c r="H15" s="42">
         <f>SUM(H4:H12)</f>
         <v/>
       </c>
-      <c r="I15" s="42" t="n"/>
+      <c r="I15" s="42">
+        <f>SUM(I4:I12)</f>
+        <v/>
+      </c>
+      <c r="J15" s="42">
+        <f>SUM(J4:J12)</f>
+        <v/>
+      </c>
+      <c r="K15" s="43" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
@@ -3379,35 +3482,43 @@
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
       </c>
-      <c r="B16" s="43">
-        <f>B5+B6</f>
-        <v/>
-      </c>
-      <c r="C16" s="43">
-        <f>C5+C6</f>
-        <v/>
-      </c>
-      <c r="D16" s="43">
+      <c r="B16" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A16,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A16,Объекты!$B$4:$B$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="44">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E16" s="43">
+      <c r="E16" s="44">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F16" s="43">
+      <c r="F16" s="44">
         <f>F5+F6</f>
         <v/>
       </c>
-      <c r="G16" s="43">
+      <c r="G16" s="44">
         <f>G5+G6</f>
         <v/>
       </c>
       <c r="H16" s="44">
-        <f>SUM(B16:G16)</f>
-        <v/>
-      </c>
-      <c r="I16" s="45" t="inlineStr">
+        <f>H5+H6</f>
+        <v/>
+      </c>
+      <c r="I16" s="44">
+        <f>I5+I6</f>
+        <v/>
+      </c>
+      <c r="J16" s="45">
+        <f>SUM(D16:I16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="46" t="inlineStr">
         <is>
           <t>строка для выпадающего списка Т1: сумма двух Flora</t>
         </is>
@@ -3415,8 +3526,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3438,49 +3549,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Финмодель Т1 · Транзитная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="48" t="inlineStr">
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
       </c>
-      <c r="C3" s="49" t="inlineStr">
+      <c r="C3" s="50" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="51">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="51">
-        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="49" t="inlineStr">
+      <c r="B4" s="52">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="51">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -3508,7 +3619,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="52" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -3572,23 +3683,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="53" t="inlineStr">
+      <c r="A11" s="54" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B11" s="42" t="n"/>
-      <c r="C11" s="54">
+      <c r="B11" s="43" t="n"/>
+      <c r="C11" s="55">
         <f>SUM(C8:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="54">
+      <c r="D11" s="55">
         <f>SUM(D8:D10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="52" t="inlineStr">
+      <c r="A12" s="53" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -3608,11 +3719,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C13" s="55">
+      <c r="C13" s="56">
         <f>$D$4*Нормативы!C5*12/1000000</f>
         <v/>
       </c>
-      <c r="D13" s="55">
+      <c r="D13" s="56">
         <f>$D$4*Нормативы!D5*12/1000000</f>
         <v/>
       </c>
@@ -3628,11 +3739,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C14" s="55">
+      <c r="C14" s="56">
         <f>$D$3*Нормативы!C6*7/1000000</f>
         <v/>
       </c>
-      <c r="D14" s="55">
+      <c r="D14" s="56">
         <f>$D$3*Нормативы!D6*7/1000000</f>
         <v/>
       </c>
@@ -3648,11 +3759,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C15" s="55">
+      <c r="C15" s="56">
         <f>$D$4*Нормативы!C7/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="55">
+      <c r="D15" s="56">
         <f>$D$4*Нормативы!D7/1000000</f>
         <v/>
       </c>
@@ -3668,11 +3779,11 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="56">
         <f>Нормативы!$C$15*Нормативы!C8*12/1000</f>
         <v/>
       </c>
-      <c r="D16" s="55">
+      <c r="D16" s="56">
         <f>Нормативы!$D$15*Нормативы!D8*12/1000</f>
         <v/>
       </c>
@@ -3688,33 +3799,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C17" s="55">
+      <c r="C17" s="56">
         <f>Нормативы!$C$17*($B$4+Нормативы!C12)</f>
         <v/>
       </c>
-      <c r="D17" s="55">
+      <c r="D17" s="56">
         <f>Нормативы!$D$17*($B$4+Нормативы!D12)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="56" t="inlineStr">
+      <c r="A18" s="57" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B18" s="42" t="n"/>
-      <c r="C18" s="57">
+      <c r="B18" s="43" t="n"/>
+      <c r="C18" s="58">
         <f>SUM(C13:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="57">
+      <c r="D18" s="58">
         <f>SUM(D13:D17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="52" t="inlineStr">
+      <c r="A20" s="53" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -3734,7 +3845,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C21" s="58">
+      <c r="C21" s="59">
         <f>IFERROR(C11/D18,0)</f>
         <v/>
       </c>
@@ -3751,7 +3862,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C22" s="58">
+      <c r="C22" s="59">
         <f>IFERROR(AVERAGE(C11:D11)/AVERAGE(C18:D18),0)</f>
         <v/>
       </c>
@@ -3768,20 +3879,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C23" s="58">
+      <c r="C23" s="59">
         <f>IFERROR(D11/C18,0)</f>
         <v/>
       </c>
       <c r="D23" s="31" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="59" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B24" s="31" t="n"/>
-      <c r="C24" s="60" t="inlineStr">
+      <c r="C24" s="61" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
@@ -3789,7 +3900,7 @@
       <c r="D24" s="31" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="52" t="inlineStr">
+      <c r="A26" s="53" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -3799,21 +3910,21 @@
       <c r="D26" s="31" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="61" t="inlineStr">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>• Кластер: общий координатор и бригада, не своя</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="61" t="inlineStr">
+      <c r="A28" s="62" t="inlineStr">
         <is>
           <t>• Спонсоры продлеваются на второй год</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="61" t="inlineStr">
+      <c r="A29" s="62" t="inlineStr">
         <is>
           <t>• Юрстатус пропускает рекламу на стелах</t>
         </is>
@@ -3864,49 +3975,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Финмодель Т2 · Активная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="48" t="inlineStr">
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
       </c>
-      <c r="C3" s="49" t="inlineStr">
+      <c r="C3" s="50" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="51">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="51">
-        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="49" t="inlineStr">
+      <c r="B4" s="52">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="51">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -3934,7 +4045,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="52" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -4034,23 +4145,23 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="53" t="inlineStr">
+      <c r="A13" s="54" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B13" s="42" t="n"/>
-      <c r="C13" s="54">
+      <c r="B13" s="43" t="n"/>
+      <c r="C13" s="55">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="54">
+      <c r="D13" s="55">
         <f>SUM(D8:D12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="52" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -4070,11 +4181,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C15" s="55">
+      <c r="C15" s="56">
         <f>$D$4*Нормативы!E5*12/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="55">
+      <c r="D15" s="56">
         <f>$D$4*Нормативы!F5*12/1000000</f>
         <v/>
       </c>
@@ -4090,11 +4201,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="56">
         <f>$D$3*Нормативы!E6*7/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="55">
+      <c r="D16" s="56">
         <f>$D$3*Нормативы!F6*7/1000000</f>
         <v/>
       </c>
@@ -4110,11 +4221,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C17" s="55">
+      <c r="C17" s="56">
         <f>$D$4*Нормативы!E7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="55">
+      <c r="D17" s="56">
         <f>$D$4*Нормативы!F7/1000000</f>
         <v/>
       </c>
@@ -4130,11 +4241,11 @@
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C18" s="55">
+      <c r="C18" s="56">
         <f>Нормативы!E9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D18" s="55">
+      <c r="D18" s="56">
         <f>Нормативы!F9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -4150,11 +4261,11 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C19" s="55">
+      <c r="C19" s="56">
         <f>Нормативы!$C$15*Нормативы!E8*12/1000</f>
         <v/>
       </c>
-      <c r="D19" s="55">
+      <c r="D19" s="56">
         <f>Нормативы!$D$15*Нормативы!F8*12/1000</f>
         <v/>
       </c>
@@ -4170,33 +4281,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C20" s="55">
+      <c r="C20" s="56">
         <f>Нормативы!$C$17*($B$4+Нормативы!E12)</f>
         <v/>
       </c>
-      <c r="D20" s="55">
+      <c r="D20" s="56">
         <f>Нормативы!$D$17*($B$4+Нормативы!F12)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="56" t="inlineStr">
+      <c r="A21" s="57" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B21" s="42" t="n"/>
-      <c r="C21" s="57">
+      <c r="B21" s="43" t="n"/>
+      <c r="C21" s="58">
         <f>SUM(C15:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="57">
+      <c r="D21" s="58">
         <f>SUM(D15:D20)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="52" t="inlineStr">
+      <c r="A23" s="53" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -4216,7 +4327,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C24" s="58">
+      <c r="C24" s="59">
         <f>IFERROR(C13/D21,0)</f>
         <v/>
       </c>
@@ -4233,7 +4344,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C25" s="58">
+      <c r="C25" s="59">
         <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
         <v/>
       </c>
@@ -4250,20 +4361,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C26" s="58">
+      <c r="C26" s="59">
         <f>IFERROR(D13/C21,0)</f>
         <v/>
       </c>
       <c r="D26" s="31" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B27" s="31" t="n"/>
-      <c r="C27" s="60" t="inlineStr">
+      <c r="C27" s="61" t="inlineStr">
         <is>
           <t>40–70%</t>
         </is>
@@ -4271,7 +4382,7 @@
       <c r="D27" s="31" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="52" t="inlineStr">
+      <c r="A29" s="53" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -4281,28 +4392,28 @@
       <c r="D29" s="31" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="61" t="inlineStr">
+      <c r="A30" s="62" t="inlineStr">
         <is>
           <t>• Справка по активам Хедлайнера получена, суммы внесены в лист «Активы»</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="61" t="inlineStr">
+      <c r="A31" s="62" t="inlineStr">
         <is>
           <t>• Якорь-павильон заполнен с мая по сентябрь</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="61" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr">
         <is>
           <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="61" t="inlineStr">
+      <c r="A33" s="62" t="inlineStr">
         <is>
           <t>• Вечерние слоты секций выкуплены</t>
         </is>
@@ -4354,49 +4465,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Финмодель Т3 · Сквер / плейхаб</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="48" t="inlineStr">
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
       </c>
-      <c r="C3" s="49" t="inlineStr">
+      <c r="C3" s="50" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="51">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="51">
-        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="49" t="inlineStr">
+      <c r="B4" s="52">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="51">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -4424,7 +4535,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="52" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -4524,23 +4635,23 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="53" t="inlineStr">
+      <c r="A13" s="54" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B13" s="42" t="n"/>
-      <c r="C13" s="54">
+      <c r="B13" s="43" t="n"/>
+      <c r="C13" s="55">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="54">
+      <c r="D13" s="55">
         <f>SUM(D8:D12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="52" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -4560,11 +4671,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C15" s="55">
+      <c r="C15" s="56">
         <f>$D$4*Нормативы!G5*12/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="55">
+      <c r="D15" s="56">
         <f>$D$4*Нормативы!H5*12/1000000</f>
         <v/>
       </c>
@@ -4580,11 +4691,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="56">
         <f>$D$3*Нормативы!G6*7/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="55">
+      <c r="D16" s="56">
         <f>$D$3*Нормативы!H6*7/1000000</f>
         <v/>
       </c>
@@ -4600,11 +4711,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C17" s="55">
+      <c r="C17" s="56">
         <f>$D$4*Нормативы!G7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="55">
+      <c r="D17" s="56">
         <f>$D$4*Нормативы!H7/1000000</f>
         <v/>
       </c>
@@ -4620,11 +4731,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C18" s="55">
+      <c r="C18" s="56">
         <f>Нормативы!G10</f>
         <v/>
       </c>
-      <c r="D18" s="55">
+      <c r="D18" s="56">
         <f>Нормативы!H10</f>
         <v/>
       </c>
@@ -4640,11 +4751,11 @@
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C19" s="55">
+      <c r="C19" s="56">
         <f>Нормативы!G9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D19" s="55">
+      <c r="D19" s="56">
         <f>Нормативы!H9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -4660,11 +4771,11 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C20" s="55">
+      <c r="C20" s="56">
         <f>Нормативы!$C$15*Нормативы!G8*12/1000</f>
         <v/>
       </c>
-      <c r="D20" s="55">
+      <c r="D20" s="56">
         <f>Нормативы!$D$15*Нормативы!H8*12/1000</f>
         <v/>
       </c>
@@ -4680,33 +4791,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C21" s="55">
+      <c r="C21" s="56">
         <f>Нормативы!$C$17*($B$4+Нормативы!G12)</f>
         <v/>
       </c>
-      <c r="D21" s="55">
+      <c r="D21" s="56">
         <f>Нормативы!$D$17*($B$4+Нормативы!H12)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="56" t="inlineStr">
+      <c r="A22" s="57" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B22" s="42" t="n"/>
-      <c r="C22" s="57">
+      <c r="B22" s="43" t="n"/>
+      <c r="C22" s="58">
         <f>SUM(C15:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="57">
+      <c r="D22" s="58">
         <f>SUM(D15:D21)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="52" t="inlineStr">
+      <c r="A24" s="53" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -4726,7 +4837,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C25" s="58">
+      <c r="C25" s="59">
         <f>IFERROR(C13/D22,0)</f>
         <v/>
       </c>
@@ -4743,7 +4854,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C26" s="58">
+      <c r="C26" s="59">
         <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C22:D22),0)</f>
         <v/>
       </c>
@@ -4760,20 +4871,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C27" s="58">
+      <c r="C27" s="59">
         <f>IFERROR(D13/C22,0)</f>
         <v/>
       </c>
       <c r="D27" s="31" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B28" s="31" t="n"/>
-      <c r="C28" s="60" t="inlineStr">
+      <c r="C28" s="61" t="inlineStr">
         <is>
           <t>70–100%</t>
         </is>
@@ -4781,7 +4892,7 @@
       <c r="D28" s="31" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="52" t="inlineStr">
+      <c r="A30" s="53" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -4791,21 +4902,21 @@
       <c r="D30" s="31" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="61" t="inlineStr">
+      <c r="A31" s="62" t="inlineStr">
         <is>
           <t>• Каток отработал первую зиму без простоев</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="61" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr">
         <is>
           <t>• Заявок на события больше, чем слотов</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="61" t="inlineStr">
+      <c r="A33" s="62" t="inlineStr">
         <is>
           <t>• Спонсор года подписан до старта сезона</t>
         </is>
@@ -4856,49 +4967,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Финмодель Т4 · Парк по ГЧП (BTO)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="48" t="inlineStr">
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>Sphere Park</t>
         </is>
       </c>
-      <c r="C3" s="49" t="inlineStr">
+      <c r="C3" s="50" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="51">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="51">
-        <f>IFERROR(INDEX(Активы!$H$4:$H$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="49" t="inlineStr">
+      <c r="B4" s="52">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="51">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -4926,7 +5037,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="52" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -5044,23 +5155,23 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="54" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B14" s="42" t="n"/>
-      <c r="C14" s="54">
+      <c r="B14" s="43" t="n"/>
+      <c r="C14" s="55">
         <f>SUM(C8:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="54">
+      <c r="D14" s="55">
         <f>SUM(D8:D13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="52" t="inlineStr">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -5080,11 +5191,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="56">
         <f>$D$4*Нормативы!I5*12/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="55">
+      <c r="D16" s="56">
         <f>$D$4*Нормативы!J5*12/1000000</f>
         <v/>
       </c>
@@ -5100,11 +5211,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C17" s="55">
+      <c r="C17" s="56">
         <f>$D$3*Нормативы!I6*7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="55">
+      <c r="D17" s="56">
         <f>$D$3*Нормативы!J6*7/1000000</f>
         <v/>
       </c>
@@ -5120,11 +5231,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C18" s="55">
+      <c r="C18" s="56">
         <f>$D$4*Нормативы!I7/1000000</f>
         <v/>
       </c>
-      <c r="D18" s="55">
+      <c r="D18" s="56">
         <f>$D$4*Нормативы!J7/1000000</f>
         <v/>
       </c>
@@ -5140,11 +5251,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C19" s="55">
+      <c r="C19" s="56">
         <f>Нормативы!I10</f>
         <v/>
       </c>
-      <c r="D19" s="55">
+      <c r="D19" s="56">
         <f>Нормативы!J10</f>
         <v/>
       </c>
@@ -5160,11 +5271,11 @@
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C20" s="55">
+      <c r="C20" s="56">
         <f>Нормативы!I9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D20" s="55">
+      <c r="D20" s="56">
         <f>Нормативы!J9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -5180,11 +5291,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C21" s="55">
+      <c r="C21" s="56">
         <f>Нормативы!I11</f>
         <v/>
       </c>
-      <c r="D21" s="55">
+      <c r="D21" s="56">
         <f>Нормативы!J11</f>
         <v/>
       </c>
@@ -5200,33 +5311,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C22" s="55">
+      <c r="C22" s="56">
         <f>Нормативы!$C$17*($B$4+Нормативы!I12)</f>
         <v/>
       </c>
-      <c r="D22" s="55">
+      <c r="D22" s="56">
         <f>Нормативы!$D$17*($B$4+Нормативы!J12)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="56" t="inlineStr">
+      <c r="A23" s="57" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B23" s="42" t="n"/>
-      <c r="C23" s="57">
+      <c r="B23" s="43" t="n"/>
+      <c r="C23" s="58">
         <f>SUM(C16:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="57">
+      <c r="D23" s="58">
         <f>SUM(D16:D22)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="52" t="inlineStr">
+      <c r="A25" s="53" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -5246,7 +5357,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C26" s="58">
+      <c r="C26" s="59">
         <f>IFERROR(C14/D23,0)</f>
         <v/>
       </c>
@@ -5263,7 +5374,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C27" s="58">
+      <c r="C27" s="59">
         <f>IFERROR(AVERAGE(C14:D14)/AVERAGE(C23:D23),0)</f>
         <v/>
       </c>
@@ -5280,20 +5391,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C28" s="58">
+      <c r="C28" s="59">
         <f>IFERROR(D14/C23,0)</f>
         <v/>
       </c>
       <c r="D28" s="31" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="59" t="inlineStr">
+      <c r="A29" s="60" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B29" s="31" t="n"/>
-      <c r="C29" s="60" t="inlineStr">
+      <c r="C29" s="61" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
@@ -5301,7 +5412,7 @@
       <c r="D29" s="31" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="52" t="inlineStr">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -5311,35 +5422,35 @@
       <c r="D31" s="31" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="61" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr">
         <is>
           <t>• Ремфонд и капремонт сидят в компенсации эксплуатации (BTO), в OPEX не дублируются</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="61" t="inlineStr">
+      <c r="A33" s="62" t="inlineStr">
         <is>
           <t>• ГЧП-договор подписан, компенсация в бюджете МИО</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="61" t="inlineStr">
+      <c r="A34" s="62" t="inlineStr">
         <is>
           <t>• Каток и события дотягивают покрытие до 100%+</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="61" t="inlineStr">
+      <c r="A35" s="62" t="inlineStr">
         <is>
           <t>• Стандарт содержания выше городского бенчмарка</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="61" t="inlineStr">
+      <c r="A36" s="62" t="inlineStr">
         <is>
           <t>• CAPEX ~2,2 млрд тг компенсируется бюджетом МИО отдельно (2026–2031) — в операционную модель не входит</t>
         </is>

</xml_diff>

<commit_message>
Use surveyed areas, add BI Service units and satellite slide
Deck (31 slides): shortlist and assets slides now use Google Earth
surveyed total areas (36,258 sqm vs the x2 assumption), new management
unit column, recalculated T1-T3 economics (T2 coverage midpoint rises
to ~84%, T1 drops to ~18%), new slide with satellite crops of the
three pilots.

Workbook v5: surveyed totals in the object registry (Nexpo Union as an
editable estimate pending survey), management unit column, asset
density column (thousand KZT per sqm) in the Assets sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014o1yT6nCgffZ5H25q7THst
</commit_message>
<xml_diff>
--- a/docs/research/BIG-Life-finmodels-T1-T4.xlsx
+++ b/docs/research/BIG-Life-finmodels-T1-T4.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00008000"/>
       <sz val="9.5"/>
     </font>
@@ -81,13 +86,18 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00B03A2E"/>
+      <color rgb="008A93A6"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
+      <color rgb="000000FF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B03A2E"/>
       <sz val="9.5"/>
     </font>
     <font>
@@ -115,11 +125,6 @@
       <name val="Arial"/>
       <color rgb="008A93A6"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -262,11 +267,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -275,23 +280,23 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -301,107 +306,113 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -794,7 +805,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая = озеленение × коэффициент (лист «Нормативы», по умолчанию ×2). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Жёлтые ячейки — редактируемые ставки.</t>
+          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая — фактический обмер Google Earth для группы A (для незамеренных: озеленение × коэффициент). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Жёлтые ячейки — редактируемые ставки.</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1144,6 +1155,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1156,7 +1168,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Группы: A — обслуживает BI Green · B — переданы 29.07–03.08.2026 · C — не обслуживаются · D — переданы городу. Площадь реестра — зелёные насаждения; общая = озеленение × коэффициент (лист «Нормативы»).</t>
+          <t>Группы: A — обслуживает BI Green · B — переданы 29.07–03.08.2026 · C — не обслуживаются · D — переданы городу. Озеленение — из реестра; общая площадь группы A — обмер Google Earth (18.08.2026), Nexpo Юнион — оценка по аналогу (жёлтая ячейка, уточнить замером), прочие — озеленение × коэффициент. «Упр.» — Управление BI Service.</t>
         </is>
       </c>
     </row>
@@ -1199,6 +1211,11 @@
       <c r="H3" s="15" t="inlineStr">
         <is>
           <t>Статус / примечание</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Упр.</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1255,15 @@
           <t>не передан, обслуживает BI Green</t>
         </is>
       </c>
+      <c r="I4" s="20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
@@ -1261,11 +1281,10 @@
       <c r="E5" s="17" t="n">
         <v>1700</v>
       </c>
-      <c r="F5" s="18">
-        <f>E5*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G5" s="21" t="inlineStr">
+      <c r="F5" s="17" t="n">
+        <v>3114</v>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1274,6 +1293,9 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1298,9 +1320,8 @@
       <c r="E6" s="17" t="n">
         <v>1600</v>
       </c>
-      <c r="F6" s="18">
-        <f>E6*Нормативы!$C$18</f>
-        <v/>
+      <c r="F6" s="17" t="n">
+        <v>4804</v>
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
@@ -1311,6 +1332,9 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1335,11 +1359,10 @@
       <c r="E7" s="17" t="n">
         <v>6200</v>
       </c>
-      <c r="F7" s="18">
-        <f>E7*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G7" s="22" t="inlineStr">
+      <c r="F7" s="17" t="n">
+        <v>10805</v>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1348,6 +1371,9 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1372,11 +1398,10 @@
       <c r="E8" s="17" t="n">
         <v>800</v>
       </c>
-      <c r="F8" s="18">
-        <f>E8*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G8" s="22" t="inlineStr">
+      <c r="F8" s="17" t="n">
+        <v>1415</v>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1385,13 +1410,16 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
@@ -1409,11 +1437,10 @@
       <c r="E9" s="17" t="n">
         <v>4000</v>
       </c>
-      <c r="F9" s="18">
-        <f>E9*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G9" s="21" t="inlineStr">
+      <c r="F9" s="17" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1422,6 +1449,9 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1446,11 +1476,10 @@
       <c r="E10" s="17" t="n">
         <v>2300</v>
       </c>
-      <c r="F10" s="18">
-        <f>E10*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G10" s="22" t="inlineStr">
+      <c r="F10" s="17" t="n">
+        <v>7059</v>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1459,13 +1488,16 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 1</t>
         </is>
@@ -1483,11 +1515,10 @@
       <c r="E11" s="17" t="n">
         <v>338</v>
       </c>
-      <c r="F11" s="18">
-        <f>E11*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="F11" s="17" t="n">
+        <v>1512</v>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1496,13 +1527,16 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I11" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 2</t>
         </is>
@@ -1520,11 +1554,10 @@
       <c r="E12" s="17" t="n">
         <v>338</v>
       </c>
-      <c r="F12" s="18">
-        <f>E12*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="F12" s="17" t="n">
+        <v>1210</v>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1533,6 +1566,9 @@
         <is>
           <t>не передан, обслуживает BI Green</t>
         </is>
+      </c>
+      <c r="I12" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1557,11 +1593,10 @@
       <c r="E13" s="17" t="n">
         <v>2385</v>
       </c>
-      <c r="F13" s="18">
-        <f>E13*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G13" s="22" t="inlineStr">
+      <c r="F13" s="17" t="n">
+        <v>2843</v>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1570,6 +1605,9 @@
         <is>
           <t>не передан, обслуживает BI Green; плейхаб, в шорт-листе как активная</t>
         </is>
+      </c>
+      <c r="I13" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1608,6 +1646,11 @@
           <t>передан 29.07.2026</t>
         </is>
       </c>
+      <c r="I14" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n">
@@ -1645,6 +1688,11 @@
           <t>передан 03.08.2026</t>
         </is>
       </c>
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="n">
@@ -1682,6 +1730,11 @@
           <t>передан 03.08.2026, придомовая</t>
         </is>
       </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="n">
@@ -1719,6 +1772,11 @@
           <t>передан 03.08.2026, есть спортплощадка</t>
         </is>
       </c>
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="n">
@@ -1756,6 +1814,11 @@
           <t>передан 03.08.2026</t>
         </is>
       </c>
+      <c r="I18" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="n">
@@ -1793,6 +1856,11 @@
           <t>передан 03.08.2026</t>
         </is>
       </c>
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="n">
@@ -1830,6 +1898,11 @@
           <t>передан 03.08.2026, аллея-парк</t>
         </is>
       </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="n">
@@ -1840,7 +1913,7 @@
           <t>Аллея Nexpo Юнион</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1853,11 +1926,10 @@
       <c r="E21" s="17" t="n">
         <v>2419</v>
       </c>
-      <c r="F21" s="18">
-        <f>E21*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G21" s="22" t="inlineStr">
+      <c r="F21" s="26" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1865,6 +1937,11 @@
       <c r="H21" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1954,7 @@
           <t>Фридом — Зелёный Квартал</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1902,6 +1979,11 @@
       <c r="H22" s="16" t="inlineStr">
         <is>
           <t>парковка, вне типологии; уточнить юраудитом</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1996,7 @@
           <t>Де Люкс 4</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1939,6 +2021,11 @@
       <c r="H23" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1951,7 +2038,7 @@
           <t>Насаждения ЖК Айтыс</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1976,6 +2063,11 @@
       <c r="H24" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается, придомовая</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1988,7 +2080,7 @@
           <t>Парк Авеню Эксклюзив</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2013,6 +2105,11 @@
       <c r="H25" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2122,7 @@
           <t>Аллея Онли Мун</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2050,6 +2147,11 @@
       <c r="H26" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается</t>
+        </is>
+      </c>
+      <c r="I26" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2164,7 @@
           <t>Аллея Сердце Столицы 1, 2</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C27" s="25" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2087,6 +2189,11 @@
       <c r="H27" s="16" t="inlineStr">
         <is>
           <t>не передан, не обслуживается, придомовая</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2126,6 +2233,11 @@
           <t>передан городу</t>
         </is>
       </c>
+      <c r="I28" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="n">
@@ -2163,6 +2275,11 @@
           <t>передан городу</t>
         </is>
       </c>
+      <c r="I29" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="n">
@@ -2200,6 +2317,11 @@
           <t>передан городу</t>
         </is>
       </c>
+      <c r="I30" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="n">
@@ -2237,6 +2359,11 @@
           <t>передан городу, кандидат на ГЧП</t>
         </is>
       </c>
+      <c r="I31" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="n">
@@ -2274,6 +2401,11 @@
           <t>передан городу</t>
         </is>
       </c>
+      <c r="I32" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="n">
@@ -2311,6 +2443,11 @@
           <t>передан городу</t>
         </is>
       </c>
+      <c r="I33" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="n">
@@ -2348,6 +2485,11 @@
           <t>передан городу</t>
         </is>
       </c>
+      <c r="I34" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16" t="n">
@@ -2371,7 +2513,7 @@
       <c r="E35" s="17" t="n">
         <v>70000</v>
       </c>
-      <c r="F35" s="24" t="n">
+      <c r="F35" s="17" t="n">
         <v>90000</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
@@ -2382,6 +2524,11 @@
       <c r="H35" s="16" t="inlineStr">
         <is>
           <t>проект ГЧП (BTO): парк 7 га + озеро 2 га у школы BINOM</t>
+        </is>
+      </c>
+      <c r="I35" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2536,7 @@
       <c r="A36" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
@@ -2408,10 +2555,10 @@
         <v>676</v>
       </c>
       <c r="F36" s="18">
-        <f>E36*Нормативы!$C$18</f>
-        <v/>
-      </c>
-      <c r="G36" s="21" t="inlineStr">
+        <f>F11+F12</f>
+        <v/>
+      </c>
+      <c r="G36" s="22" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -2420,12 +2567,15 @@
         <is>
           <t>пилот Т1: два объекта под одной командой</t>
         </is>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2467,52 +2617,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>Т1 мин</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>Т1 макс</t>
         </is>
       </c>
-      <c r="E4" s="25" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
         <is>
           <t>Т2 мин</t>
         </is>
       </c>
-      <c r="F4" s="25" t="inlineStr">
+      <c r="F4" s="27" t="inlineStr">
         <is>
           <t>Т2 макс</t>
         </is>
       </c>
-      <c r="G4" s="25" t="inlineStr">
+      <c r="G4" s="27" t="inlineStr">
         <is>
           <t>Т3 мин</t>
         </is>
       </c>
-      <c r="H4" s="25" t="inlineStr">
+      <c r="H4" s="27" t="inlineStr">
         <is>
           <t>Т3 макс</t>
         </is>
       </c>
-      <c r="I4" s="25" t="inlineStr">
+      <c r="I4" s="27" t="inlineStr">
         <is>
           <t>Т4 мин</t>
         </is>
       </c>
-      <c r="J4" s="25" t="inlineStr">
+      <c r="J4" s="27" t="inlineStr">
         <is>
           <t>Т4 макс</t>
         </is>
@@ -2524,33 +2674,33 @@
           <t>Уборка и снегоуборка</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>тг/м² общей пл. в месяц</t>
         </is>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="29" t="n">
         <v>60</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="29" t="n">
         <v>90</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="29" t="n">
         <v>55</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="29" t="n">
         <v>60</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="29" t="n">
         <v>100</v>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="J5" s="27" t="n">
+      <c r="J5" s="29" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2560,33 +2710,33 @@
           <t>Озеленение и полив (апр–окт)</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>тг/м² озеленения в месяц</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="29" t="n">
         <v>90</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="29" t="n">
         <v>160</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="29" t="n">
         <v>70</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="29" t="n">
         <v>55</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="29" t="n">
         <v>90</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="29" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2596,33 +2746,33 @@
           <t>Свет, электро, digital</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>тг/м² общей пл. в год</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="29" t="n">
         <v>155</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="29" t="n">
         <v>250</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="29" t="n">
         <v>65</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="29" t="n">
         <v>115</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="29" t="n">
         <v>190</v>
       </c>
-      <c r="H7" s="27" t="n">
+      <c r="H7" s="29" t="n">
         <v>315</v>
       </c>
-      <c r="I7" s="27" t="n">
+      <c r="I7" s="29" t="n">
         <v>80</v>
       </c>
-      <c r="J7" s="27" t="n">
+      <c r="J7" s="29" t="n">
         <v>150</v>
       </c>
     </row>
@@ -2632,33 +2782,33 @@
           <t>Доля ставки координатора</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>доля ставки</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="30" t="n">
         <v>0.2</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="30" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="30" t="n">
         <v>0.33</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="30" t="n">
         <v>0.33</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="30" t="n">
         <v>0.6</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="30" t="n">
         <v>0.6</v>
       </c>
-      <c r="I8" s="28" t="n">
+      <c r="I8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="28" t="n">
+      <c r="J8" s="30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2668,33 +2818,33 @@
           <t>Число событий в год</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="29" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2704,33 +2854,33 @@
           <t>Зимний пакет (каток, горка, свет)</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>млн тг/год</t>
         </is>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="29" t="n">
+      <c r="G10" s="31" t="n">
         <v>2.5</v>
       </c>
-      <c r="H10" s="29" t="n">
+      <c r="H10" s="31" t="n">
         <v>4.5</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="29" t="n">
         <v>6</v>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="29" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2740,33 +2890,33 @@
           <t>Персонал парка (только Т4)</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>млн тг/год</t>
         </is>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="27" t="n">
+      <c r="H11" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="27" t="n">
+      <c r="I11" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="27" t="n">
+      <c r="J11" s="29" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2776,38 +2926,38 @@
           <t>CAPEX активации (разово, план)</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>млн тг, единовременно</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="29" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="H12" s="27" t="n">
+      <c r="H12" s="29" t="n">
         <v>120</v>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="27" t="n">
+      <c r="J12" s="29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>ОБЩИЕ НОРМАТИВЫ (мин / макс)</t>
         </is>
@@ -2819,23 +2969,23 @@
           <t>Ставка координатора кластера</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>тыс тг/мес</t>
         </is>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="29" t="n">
         <v>300</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="29" t="n">
         <v>420</v>
       </c>
-      <c r="E15" s="31" t="n"/>
-      <c r="F15" s="31" t="n"/>
-      <c r="G15" s="31" t="n"/>
-      <c r="H15" s="31" t="n"/>
-      <c r="I15" s="31" t="n"/>
-      <c r="J15" s="31" t="n"/>
+      <c r="E15" s="33" t="n"/>
+      <c r="F15" s="33" t="n"/>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="33" t="n"/>
+      <c r="I15" s="33" t="n"/>
+      <c r="J15" s="33" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -2843,23 +2993,23 @@
           <t>Цена события с продвижением</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>тыс тг</t>
         </is>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="29" t="n">
         <v>95</v>
       </c>
-      <c r="D16" s="27" t="n">
+      <c r="D16" s="29" t="n">
         <v>130</v>
       </c>
-      <c r="E16" s="31" t="n"/>
-      <c r="F16" s="31" t="n"/>
-      <c r="G16" s="31" t="n"/>
-      <c r="H16" s="31" t="n"/>
-      <c r="I16" s="31" t="n"/>
-      <c r="J16" s="31" t="n"/>
+      <c r="E16" s="33" t="n"/>
+      <c r="F16" s="33" t="n"/>
+      <c r="G16" s="33" t="n"/>
+      <c r="H16" s="33" t="n"/>
+      <c r="I16" s="33" t="n"/>
+      <c r="J16" s="33" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2867,23 +3017,23 @@
           <t>Ремфонд, % в год от активов и вложений</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>% в год</t>
         </is>
       </c>
-      <c r="C17" s="32" t="n">
+      <c r="C17" s="34" t="n">
         <v>0.01</v>
       </c>
-      <c r="D17" s="32" t="n">
+      <c r="D17" s="34" t="n">
         <v>0.015</v>
       </c>
-      <c r="E17" s="31" t="n"/>
-      <c r="F17" s="31" t="n"/>
-      <c r="G17" s="31" t="n"/>
-      <c r="H17" s="31" t="n"/>
-      <c r="I17" s="31" t="n"/>
-      <c r="J17" s="31" t="n"/>
+      <c r="E17" s="33" t="n"/>
+      <c r="F17" s="33" t="n"/>
+      <c r="G17" s="33" t="n"/>
+      <c r="H17" s="33" t="n"/>
+      <c r="I17" s="33" t="n"/>
+      <c r="J17" s="33" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -2891,23 +3041,23 @@
           <t>Коэффициент: общая площадь / озеленение</t>
         </is>
       </c>
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>×</t>
         </is>
       </c>
-      <c r="C18" s="33" t="n">
+      <c r="C18" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="33" t="n">
+      <c r="D18" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="31" t="n"/>
-      <c r="F18" s="31" t="n"/>
-      <c r="G18" s="31" t="n"/>
-      <c r="H18" s="31" t="n"/>
-      <c r="I18" s="31" t="n"/>
-      <c r="J18" s="31" t="n"/>
+      <c r="E18" s="33" t="n"/>
+      <c r="F18" s="33" t="n"/>
+      <c r="G18" s="33" t="n"/>
+      <c r="H18" s="33" t="n"/>
+      <c r="I18" s="33" t="n"/>
+      <c r="J18" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2925,7 +3075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2938,7 +3088,8 @@
     <col width="8.5" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9.5" customWidth="1" min="10" max="10"/>
-    <col width="58" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="56" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2956,64 +3107,69 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="34" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B3" s="35" t="inlineStr">
+      <c r="B3" s="37" t="inlineStr">
         <is>
           <t>Озеленение, м²</t>
         </is>
       </c>
-      <c r="C3" s="35" t="inlineStr">
+      <c r="C3" s="37" t="inlineStr">
         <is>
           <t>Общая, м²</t>
         </is>
       </c>
-      <c r="D3" s="35" t="inlineStr">
+      <c r="D3" s="37" t="inlineStr">
         <is>
           <t>Покрытия</t>
         </is>
       </c>
-      <c r="E3" s="35" t="inlineStr">
+      <c r="E3" s="37" t="inlineStr">
         <is>
           <t>Насаждения</t>
         </is>
       </c>
-      <c r="F3" s="35" t="inlineStr">
+      <c r="F3" s="37" t="inlineStr">
         <is>
           <t>МАФы</t>
         </is>
       </c>
-      <c r="G3" s="35" t="inlineStr">
+      <c r="G3" s="37" t="inlineStr">
         <is>
           <t>Свет</t>
         </is>
       </c>
-      <c r="H3" s="35" t="inlineStr">
+      <c r="H3" s="37" t="inlineStr">
         <is>
           <t>Полив</t>
         </is>
       </c>
-      <c r="I3" s="35" t="inlineStr">
+      <c r="I3" s="37" t="inlineStr">
         <is>
           <t>Земля</t>
         </is>
       </c>
-      <c r="J3" s="35" t="inlineStr">
+      <c r="J3" s="37" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="K3" s="34" t="inlineStr">
+      <c r="K3" s="37" t="inlineStr">
+        <is>
+          <t>тыс тг/м²</t>
+        </is>
+      </c>
+      <c r="L3" s="36" t="inlineStr">
         <is>
           <t>Что на балансе (по справке)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
@@ -3026,36 +3182,40 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A4,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D4" s="36" t="n">
+      <c r="D4" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="36" t="n">
+      <c r="E4" s="38" t="n">
         <v>2.09</v>
       </c>
-      <c r="F4" s="36" t="n">
+      <c r="F4" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="36" t="n">
+      <c r="G4" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="36" t="n">
+      <c r="H4" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="36" t="n">
+      <c r="I4" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="37">
+      <c r="J4" s="39">
         <f>SUM(D4:I4)</f>
         <v/>
       </c>
-      <c r="K4" s="38" t="inlineStr">
+      <c r="K4" s="40">
+        <f>IFERROR(J4/C4*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="41" t="inlineStr">
         <is>
           <t>только озеленение: 458 растений (вяз-изгородь 408 шт, 18 сосен, 11 елей). Света, МАФов и покрытий на балансе нет</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 1</t>
         </is>
@@ -3068,36 +3228,40 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A5,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D5" s="36" t="n">
+      <c r="D5" s="38" t="n">
         <v>2.5</v>
       </c>
-      <c r="E5" s="36" t="n">
+      <c r="E5" s="38" t="n">
         <v>32.11</v>
       </c>
-      <c r="F5" s="36" t="n">
+      <c r="F5" s="38" t="n">
         <v>2.23</v>
       </c>
-      <c r="G5" s="36" t="n">
+      <c r="G5" s="38" t="n">
         <v>5.23</v>
       </c>
-      <c r="H5" s="36" t="n">
+      <c r="H5" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="36" t="n">
+      <c r="I5" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="37">
+      <c r="J5" s="39">
         <f>SUM(D5:I5)</f>
         <v/>
       </c>
-      <c r="K5" s="38" t="inlineStr">
+      <c r="K5" s="40">
+        <f>IFERROR(J5/C5*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="41" t="inlineStr">
         <is>
           <t>брусчатка 279 м², 1 647 кустарников + 515 многолетников + 49 деревьев, 10 скамеек, 20 светильников, гирлянда 300 м</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 2</t>
         </is>
@@ -3110,36 +3274,40 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A6,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="38" t="n">
         <v>2.07</v>
       </c>
-      <c r="E6" s="36" t="n">
+      <c r="E6" s="38" t="n">
         <v>20.68</v>
       </c>
-      <c r="F6" s="36" t="n">
+      <c r="F6" s="38" t="n">
         <v>1.47</v>
       </c>
-      <c r="G6" s="36" t="n">
+      <c r="G6" s="38" t="n">
         <v>5.85</v>
       </c>
-      <c r="H6" s="36" t="n">
+      <c r="H6" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="36" t="n">
+      <c r="I6" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="37">
+      <c r="J6" s="39">
         <f>SUM(D6:I6)</f>
         <v/>
       </c>
-      <c r="K6" s="38" t="inlineStr">
+      <c r="K6" s="40">
+        <f>IFERROR(J6/C6*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="41" t="inlineStr">
         <is>
           <t>брусчатка 226 м², 1 087 кустарников + 34 дерева, 8 скамеек, 20 светильников, гирлянда 480 м</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
@@ -3152,29 +3320,33 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A7,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D7" s="39" t="n">
+      <c r="D7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="E7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="39" t="n">
+      <c r="F7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="39" t="n">
+      <c r="G7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="39" t="n">
+      <c r="H7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="39" t="n">
+      <c r="I7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="37">
+      <c r="J7" s="39">
         <f>SUM(D7:I7)</f>
         <v/>
       </c>
-      <c r="K7" s="38" t="inlineStr">
+      <c r="K7" s="40">
+        <f>IFERROR(J7/C7*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="41" t="inlineStr">
         <is>
           <t>СПРАВКА ЗАПРОШЕНА у застройщика — внести после нулевого спринта (жёлтые ячейки)</t>
         </is>
@@ -3194,29 +3366,33 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A8,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="38" t="n">
         <v>14.97</v>
       </c>
-      <c r="E8" s="36" t="n">
+      <c r="E8" s="38" t="n">
         <v>38.65</v>
       </c>
-      <c r="F8" s="36" t="n">
+      <c r="F8" s="38" t="n">
         <v>2.38</v>
       </c>
-      <c r="G8" s="36" t="n">
+      <c r="G8" s="38" t="n">
         <v>4.26</v>
       </c>
-      <c r="H8" s="36" t="n">
+      <c r="H8" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="36" t="n">
+      <c r="I8" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="37">
+      <c r="J8" s="39">
         <f>SUM(D8:I8)</f>
         <v/>
       </c>
-      <c r="K8" s="38" t="inlineStr">
+      <c r="K8" s="40">
+        <f>IFERROR(J8/C8*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="41" t="inlineStr">
         <is>
           <t>брусчатка 2 000 м², 2 226 кустарников + 42 дерева, 11 скамеек, 14 светильников 3,5 м, гирлянда 250 м</t>
         </is>
@@ -3236,29 +3412,33 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A9,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D9" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="36" t="n">
+      <c r="E9" s="38" t="n">
         <v>21.89</v>
       </c>
-      <c r="F9" s="36" t="n">
+      <c r="F9" s="38" t="n">
         <v>53.75</v>
       </c>
-      <c r="G9" s="36" t="n">
+      <c r="G9" s="38" t="n">
         <v>1.3</v>
       </c>
-      <c r="H9" s="36" t="n">
+      <c r="H9" s="38" t="n">
         <v>1.34</v>
       </c>
-      <c r="I9" s="36" t="n">
+      <c r="I9" s="38" t="n">
         <v>57.09</v>
       </c>
-      <c r="J9" s="37">
+      <c r="J9" s="39">
         <f>SUM(D9:I9)</f>
         <v/>
       </c>
-      <c r="K9" s="38" t="inlineStr">
+      <c r="K9" s="40">
+        <f>IFERROR(J9/C9*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="41" t="inlineStr">
         <is>
           <t>детское ядро: две горки (26,2 и 14,5 млн), карусель, батут, качели, тренажёр; автополив Hunter/Grundfos; земля 0,37 га</t>
         </is>
@@ -3278,29 +3458,33 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A10,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="D10" s="38" t="n">
         <v>43.81</v>
       </c>
-      <c r="E10" s="36" t="n">
+      <c r="E10" s="38" t="n">
         <v>46.89</v>
       </c>
-      <c r="F10" s="36" t="n">
+      <c r="F10" s="38" t="n">
         <v>29.55</v>
       </c>
-      <c r="G10" s="36" t="n">
+      <c r="G10" s="38" t="n">
         <v>8.81</v>
       </c>
-      <c r="H10" s="36" t="n">
+      <c r="H10" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="36" t="n">
+      <c r="I10" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="37">
+      <c r="J10" s="39">
         <f>SUM(D10:I10)</f>
         <v/>
       </c>
-      <c r="K10" s="38" t="inlineStr">
+      <c r="K10" s="40">
+        <f>IFERROR(J10/C10*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="41" t="inlineStr">
         <is>
           <t>спецификация: покрытия ~5 200 м², 10 игровых комплексов, 27 скамеек, 21 урна, 23 опоры света (материалы, без НДС)</t>
         </is>
@@ -3320,29 +3504,33 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A11,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="E11" s="38" t="n">
         <v>6.83</v>
       </c>
-      <c r="F11" s="36" t="n">
+      <c r="F11" s="38" t="n">
         <v>23</v>
       </c>
-      <c r="G11" s="36" t="n">
+      <c r="G11" s="38" t="n">
         <v>1.26</v>
       </c>
-      <c r="H11" s="36" t="n">
+      <c r="H11" s="38" t="n">
         <v>0.7</v>
       </c>
-      <c r="I11" s="36" t="n">
+      <c r="I11" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="37">
+      <c r="J11" s="39">
         <f>SUM(D11:I11)</f>
         <v/>
       </c>
-      <c r="K11" s="38" t="inlineStr">
+      <c r="K11" s="40">
+        <f>IFERROR(J11/C11*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="41" t="inlineStr">
         <is>
           <t>спортядро: огороженное поле 312 м² искусственной травы (борт 5 м), баскетбол, воркаут-серия, 4 вида качелей, канатный лаз</t>
         </is>
@@ -3362,29 +3550,33 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A12,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D12" s="36" t="n">
+      <c r="D12" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="36" t="n">
+      <c r="E12" s="38" t="n">
         <v>16.52</v>
       </c>
-      <c r="F12" s="36" t="n">
+      <c r="F12" s="38" t="n">
         <v>52.11</v>
       </c>
-      <c r="G12" s="36" t="n">
+      <c r="G12" s="38" t="n">
         <v>4.08</v>
       </c>
-      <c r="H12" s="36" t="n">
+      <c r="H12" s="38" t="n">
         <v>0.72</v>
       </c>
-      <c r="I12" s="36" t="n">
+      <c r="I12" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="37">
+      <c r="J12" s="39">
         <f>SUM(D12:I12)</f>
         <v/>
       </c>
-      <c r="K12" s="38" t="inlineStr">
+      <c r="K12" s="40">
+        <f>IFERROR(J12/C12*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="41" t="inlineStr">
         <is>
           <t>игровой комплекс 42 млн (тартан, скалодром, тоннели), воркаут, теннисный стол, 54 светильника, автополив</t>
         </is>
@@ -3404,80 +3596,88 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A13,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D13" s="36" t="n">
+      <c r="D13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="36" t="n">
+      <c r="E13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="36" t="n">
+      <c r="F13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="36" t="n">
+      <c r="G13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="36" t="n">
+      <c r="H13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="36" t="n">
+      <c r="I13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="37">
+      <c r="J13" s="39">
         <f>SUM(D13:I13)</f>
         <v/>
       </c>
-      <c r="K13" s="38" t="inlineStr">
+      <c r="K13" s="40">
+        <f>IFERROR(J13/C13*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="41" t="inlineStr">
         <is>
           <t>справка без стоимостей: 47 деревьев (сосна, осина, клён) — вне шорт-листа</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="40" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>Итого шорт-лист (9 объектов)</t>
         </is>
       </c>
-      <c r="B15" s="41">
+      <c r="B15" s="44">
         <f>SUM(B4:B12)</f>
         <v/>
       </c>
-      <c r="C15" s="41">
+      <c r="C15" s="44">
         <f>SUM(C4:C12)</f>
         <v/>
       </c>
-      <c r="D15" s="42">
+      <c r="D15" s="45">
         <f>SUM(D4:D12)</f>
         <v/>
       </c>
-      <c r="E15" s="42">
+      <c r="E15" s="45">
         <f>SUM(E4:E12)</f>
         <v/>
       </c>
-      <c r="F15" s="42">
+      <c r="F15" s="45">
         <f>SUM(F4:F12)</f>
         <v/>
       </c>
-      <c r="G15" s="42">
+      <c r="G15" s="45">
         <f>SUM(G4:G12)</f>
         <v/>
       </c>
-      <c r="H15" s="42">
+      <c r="H15" s="45">
         <f>SUM(H4:H12)</f>
         <v/>
       </c>
-      <c r="I15" s="42">
+      <c r="I15" s="45">
         <f>SUM(I4:I12)</f>
         <v/>
       </c>
-      <c r="J15" s="42">
+      <c r="J15" s="45">
         <f>SUM(J4:J12)</f>
         <v/>
       </c>
-      <c r="K15" s="43" t="n"/>
+      <c r="K15" s="45">
+        <f>IFERROR(J15/C15*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="46" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
@@ -3490,35 +3690,39 @@
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A16,Объекты!$B$4:$B$36,0)),"")</f>
         <v/>
       </c>
-      <c r="D16" s="44">
+      <c r="D16" s="40">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E16" s="44">
+      <c r="E16" s="40">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F16" s="44">
+      <c r="F16" s="40">
         <f>F5+F6</f>
         <v/>
       </c>
-      <c r="G16" s="44">
+      <c r="G16" s="40">
         <f>G5+G6</f>
         <v/>
       </c>
-      <c r="H16" s="44">
+      <c r="H16" s="40">
         <f>H5+H6</f>
         <v/>
       </c>
-      <c r="I16" s="44">
+      <c r="I16" s="40">
         <f>I5+I6</f>
         <v/>
       </c>
-      <c r="J16" s="45">
+      <c r="J16" s="47">
         <f>SUM(D16:I16)</f>
         <v/>
       </c>
-      <c r="K16" s="46" t="inlineStr">
+      <c r="K16" s="40">
+        <f>IFERROR(J16/C16*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="48" t="inlineStr">
         <is>
           <t>строка для выпадающего списка Т1: сумма двух Flora</t>
         </is>
@@ -3526,8 +3730,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3549,49 +3753,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="47" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>Финмодель Т1 · Транзитная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="48" t="inlineStr">
+      <c r="A3" s="50" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="49" t="inlineStr">
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
       </c>
-      <c r="C3" s="50" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="51">
+      <c r="D3" s="53">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="52">
+      <c r="B4" s="54">
         <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
         <v/>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="53">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -3619,14 +3823,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
+      <c r="B7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3634,15 +3838,15 @@
           <t>Вендинг, 1 автомат</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>аренда точки 25–45 тыс тг/мес</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
+      <c r="C8" s="35" t="n">
         <v>0.3</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="35" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -3652,15 +3856,15 @@
           <t>Спонсорство «Усынови клумбу»</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>3–5 спонсоров по 80–150 тыс тг/год</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C9" s="35" t="n">
         <v>0.2</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="35" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -3670,43 +3874,43 @@
           <t>Реклама на навигации</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>при подходящем юрстатусе земли</t>
         </is>
       </c>
-      <c r="C10" s="33" t="n">
+      <c r="C10" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="35" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="54" t="inlineStr">
+      <c r="A11" s="56" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B11" s="43" t="n"/>
-      <c r="C11" s="55">
+      <c r="B11" s="46" t="n"/>
+      <c r="C11" s="57">
         <f>SUM(C8:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="55">
+      <c r="D11" s="57">
         <f>SUM(D8:D10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="53" t="inlineStr">
+      <c r="A12" s="55" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B12" s="31" t="n"/>
-      <c r="C12" s="31" t="n"/>
-      <c r="D12" s="31" t="n"/>
+      <c r="B12" s="33" t="n"/>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -3714,16 +3918,16 @@
           <t>Уборка и снегоуборка</t>
         </is>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C13" s="56">
+      <c r="C13" s="58">
         <f>$D$4*Нормативы!C5*12/1000000</f>
         <v/>
       </c>
-      <c r="D13" s="56">
+      <c r="D13" s="58">
         <f>$D$4*Нормативы!D5*12/1000000</f>
         <v/>
       </c>
@@ -3734,16 +3938,16 @@
           <t>Озеленение и полив</t>
         </is>
       </c>
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C14" s="56">
+      <c r="C14" s="58">
         <f>$D$3*Нормативы!C6*7/1000000</f>
         <v/>
       </c>
-      <c r="D14" s="56">
+      <c r="D14" s="58">
         <f>$D$3*Нормативы!D6*7/1000000</f>
         <v/>
       </c>
@@ -3754,16 +3958,16 @@
           <t>Свет, электро, digital</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C15" s="56">
+      <c r="C15" s="58">
         <f>$D$4*Нормативы!C7/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="56">
+      <c r="D15" s="58">
         <f>$D$4*Нормативы!D7/1000000</f>
         <v/>
       </c>
@@ -3774,16 +3978,16 @@
           <t>Координатор кластера</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="56">
+      <c r="C16" s="58">
         <f>Нормативы!$C$15*Нормативы!C8*12/1000</f>
         <v/>
       </c>
-      <c r="D16" s="56">
+      <c r="D16" s="58">
         <f>Нормативы!$D$15*Нормативы!D8*12/1000</f>
         <v/>
       </c>
@@ -3794,45 +3998,45 @@
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="58">
         <f>Нормативы!$C$17*($B$4+Нормативы!C12)</f>
         <v/>
       </c>
-      <c r="D17" s="56">
+      <c r="D17" s="58">
         <f>Нормативы!$D$17*($B$4+Нормативы!D12)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="57" t="inlineStr">
+      <c r="A18" s="59" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B18" s="43" t="n"/>
-      <c r="C18" s="58">
+      <c r="B18" s="46" t="n"/>
+      <c r="C18" s="60">
         <f>SUM(C13:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="58">
+      <c r="D18" s="60">
         <f>SUM(D13:D17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="53" t="inlineStr">
+      <c r="A20" s="55" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B20" s="31" t="n"/>
-      <c r="C20" s="31" t="n"/>
-      <c r="D20" s="31" t="n"/>
+      <c r="B20" s="33" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -3840,16 +4044,16 @@
           <t>Консервативный сценарий</t>
         </is>
       </c>
-      <c r="B21" s="26" t="inlineStr">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C21" s="59">
+      <c r="C21" s="61">
         <f>IFERROR(C11/D18,0)</f>
         <v/>
       </c>
-      <c r="D21" s="31" t="n"/>
+      <c r="D21" s="33" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -3857,16 +4061,16 @@
           <t>По середине вилок</t>
         </is>
       </c>
-      <c r="B22" s="26" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C22" s="59">
+      <c r="C22" s="61">
         <f>IFERROR(AVERAGE(C11:D11)/AVERAGE(C18:D18),0)</f>
         <v/>
       </c>
-      <c r="D22" s="31" t="n"/>
+      <c r="D22" s="33" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -3874,57 +4078,57 @@
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B23" s="26" t="inlineStr">
+      <c r="B23" s="28" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C23" s="59">
+      <c r="C23" s="61">
         <f>IFERROR(D11/C18,0)</f>
         <v/>
       </c>
-      <c r="D23" s="31" t="n"/>
+      <c r="D23" s="33" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="60" t="inlineStr">
+      <c r="A24" s="62" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B24" s="31" t="n"/>
-      <c r="C24" s="61" t="inlineStr">
+      <c r="B24" s="33" t="n"/>
+      <c r="C24" s="63" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
       </c>
-      <c r="D24" s="31" t="n"/>
+      <c r="D24" s="33" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="53" t="inlineStr">
+      <c r="A26" s="55" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B26" s="31" t="n"/>
-      <c r="C26" s="31" t="n"/>
-      <c r="D26" s="31" t="n"/>
+      <c r="B26" s="33" t="n"/>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="33" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="62" t="inlineStr">
+      <c r="A27" s="64" t="inlineStr">
         <is>
           <t>• Кластер: общий координатор и бригада, не своя</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="62" t="inlineStr">
+      <c r="A28" s="64" t="inlineStr">
         <is>
           <t>• Спонсоры продлеваются на второй год</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr">
+      <c r="A29" s="64" t="inlineStr">
         <is>
           <t>• Юрстатус пропускает рекламу на стелах</t>
         </is>
@@ -3975,49 +4179,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="47" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>Финмодель Т2 · Активная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="48" t="inlineStr">
+      <c r="A3" s="50" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="49" t="inlineStr">
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
       </c>
-      <c r="C3" s="50" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="51">
+      <c r="D3" s="53">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="52">
+      <c r="B4" s="54">
         <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
         <v/>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="53">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -4045,14 +4249,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
+      <c r="B7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -4060,15 +4264,15 @@
           <t>НТО-якорь: кофе-павильон</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
+      <c r="C8" s="35" t="n">
         <v>1.8</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="35" t="n">
         <v>3.6</v>
       </c>
     </row>
@@ -4078,15 +4282,15 @@
           <t>Ярмарка выходного дня</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C9" s="35" t="n">
         <v>0.7</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="35" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -4096,15 +4300,15 @@
           <t>Секции и кикшеринг</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>слоты тренерам + rev-share операторов</t>
         </is>
       </c>
-      <c r="C10" s="33" t="n">
+      <c r="C10" s="35" t="n">
         <v>0.6</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="35" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -4114,15 +4318,15 @@
           <t>Digital-экран и реклама</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>при подходящем юрстатусе земли</t>
         </is>
       </c>
-      <c r="C11" s="33" t="n">
+      <c r="C11" s="35" t="n">
         <v>0.8</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="35" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4132,43 +4336,43 @@
           <t>Спонсорство объектов</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>воркаут, клумбы, скамейки</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n">
+      <c r="C12" s="35" t="n">
         <v>0.5</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="35" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="54" t="inlineStr">
+      <c r="A13" s="56" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B13" s="43" t="n"/>
-      <c r="C13" s="55">
+      <c r="B13" s="46" t="n"/>
+      <c r="C13" s="57">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="55">
+      <c r="D13" s="57">
         <f>SUM(D8:D12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
+      <c r="B14" s="33" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -4176,16 +4380,16 @@
           <t>Уборка и снегоуборка</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C15" s="56">
+      <c r="C15" s="58">
         <f>$D$4*Нормативы!E5*12/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="56">
+      <c r="D15" s="58">
         <f>$D$4*Нормативы!F5*12/1000000</f>
         <v/>
       </c>
@@ -4196,16 +4400,16 @@
           <t>Озеленение и полив</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C16" s="56">
+      <c r="C16" s="58">
         <f>$D$3*Нормативы!E6*7/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="56">
+      <c r="D16" s="58">
         <f>$D$3*Нормативы!F6*7/1000000</f>
         <v/>
       </c>
@@ -4216,16 +4420,16 @@
           <t>Свет, электро, digital</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="58">
         <f>$D$4*Нормативы!E7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="56">
+      <c r="D17" s="58">
         <f>$D$4*Нормативы!F7/1000000</f>
         <v/>
       </c>
@@ -4236,16 +4440,16 @@
           <t>Программа и маркетинг</t>
         </is>
       </c>
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="58">
         <f>Нормативы!E9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D18" s="56">
+      <c r="D18" s="58">
         <f>Нормативы!F9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -4256,16 +4460,16 @@
           <t>Координатор кластера</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="58">
         <f>Нормативы!$C$15*Нормативы!E8*12/1000</f>
         <v/>
       </c>
-      <c r="D19" s="56">
+      <c r="D19" s="58">
         <f>Нормативы!$D$15*Нормативы!F8*12/1000</f>
         <v/>
       </c>
@@ -4276,45 +4480,45 @@
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C20" s="56">
+      <c r="C20" s="58">
         <f>Нормативы!$C$17*($B$4+Нормативы!E12)</f>
         <v/>
       </c>
-      <c r="D20" s="56">
+      <c r="D20" s="58">
         <f>Нормативы!$D$17*($B$4+Нормативы!F12)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="57" t="inlineStr">
+      <c r="A21" s="59" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B21" s="43" t="n"/>
-      <c r="C21" s="58">
+      <c r="B21" s="46" t="n"/>
+      <c r="C21" s="60">
         <f>SUM(C15:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="58">
+      <c r="D21" s="60">
         <f>SUM(D15:D20)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="53" t="inlineStr">
+      <c r="A23" s="55" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="31" t="n"/>
-      <c r="D23" s="31" t="n"/>
+      <c r="B23" s="33" t="n"/>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -4322,16 +4526,16 @@
           <t>Консервативный сценарий</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C24" s="59">
+      <c r="C24" s="61">
         <f>IFERROR(C13/D21,0)</f>
         <v/>
       </c>
-      <c r="D24" s="31" t="n"/>
+      <c r="D24" s="33" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -4339,16 +4543,16 @@
           <t>По середине вилок</t>
         </is>
       </c>
-      <c r="B25" s="26" t="inlineStr">
+      <c r="B25" s="28" t="inlineStr">
         <is>
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C25" s="59">
+      <c r="C25" s="61">
         <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
         <v/>
       </c>
-      <c r="D25" s="31" t="n"/>
+      <c r="D25" s="33" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -4356,64 +4560,64 @@
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B26" s="26" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C26" s="59">
+      <c r="C26" s="61">
         <f>IFERROR(D13/C21,0)</f>
         <v/>
       </c>
-      <c r="D26" s="31" t="n"/>
+      <c r="D26" s="33" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="60" t="inlineStr">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B27" s="31" t="n"/>
-      <c r="C27" s="61" t="inlineStr">
+      <c r="B27" s="33" t="n"/>
+      <c r="C27" s="63" t="inlineStr">
         <is>
           <t>40–70%</t>
         </is>
       </c>
-      <c r="D27" s="31" t="n"/>
+      <c r="D27" s="33" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="53" t="inlineStr">
+      <c r="A29" s="55" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B29" s="31" t="n"/>
-      <c r="C29" s="31" t="n"/>
-      <c r="D29" s="31" t="n"/>
+      <c r="B29" s="33" t="n"/>
+      <c r="C29" s="33" t="n"/>
+      <c r="D29" s="33" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="62" t="inlineStr">
+      <c r="A30" s="64" t="inlineStr">
         <is>
           <t>• Справка по активам Хедлайнера получена, суммы внесены в лист «Активы»</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="62" t="inlineStr">
+      <c r="A31" s="64" t="inlineStr">
         <is>
           <t>• Якорь-павильон заполнен с мая по сентябрь</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr">
+      <c r="A32" s="64" t="inlineStr">
         <is>
           <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr">
+      <c r="A33" s="64" t="inlineStr">
         <is>
           <t>• Вечерние слоты секций выкуплены</t>
         </is>
@@ -4465,49 +4669,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="47" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>Финмодель Т3 · Сквер / плейхаб</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="48" t="inlineStr">
+      <c r="A3" s="50" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="49" t="inlineStr">
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
       </c>
-      <c r="C3" s="50" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="51">
+      <c r="D3" s="53">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="52">
+      <c r="B4" s="54">
         <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
         <v/>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="53">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -4535,14 +4739,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
+      <c r="B7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -4550,15 +4754,15 @@
           <t>Две НТО-точки</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>кофе и выпечка: аренда + % оборота</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
+      <c r="C8" s="35" t="n">
         <v>2.4</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="35" t="n">
         <v>4.8</v>
       </c>
     </row>
@@ -4568,15 +4772,15 @@
           <t>Каток: прокат и билеты</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>компактный контур, 120–160 дней</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C9" s="35" t="n">
         <v>1.5</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="35" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -4586,15 +4790,15 @@
           <t>Событийная аренда</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>10–18 частных и корпоративных событий</t>
         </is>
       </c>
-      <c r="C10" s="33" t="n">
+      <c r="C10" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="35" t="n">
         <v>2.8</v>
       </c>
     </row>
@@ -4604,15 +4808,15 @@
           <t>Ярмарки, маркеты, секции</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>круглогодичный календарь</t>
         </is>
       </c>
-      <c r="C11" s="33" t="n">
+      <c r="C11" s="35" t="n">
         <v>1.3</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="35" t="n">
         <v>2.6</v>
       </c>
     </row>
@@ -4622,43 +4826,43 @@
           <t>Спонсор года и реклама</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>один якорный партнёр + экран</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n">
+      <c r="C12" s="35" t="n">
         <v>1.5</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="35" t="n">
         <v>3.7</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="54" t="inlineStr">
+      <c r="A13" s="56" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B13" s="43" t="n"/>
-      <c r="C13" s="55">
+      <c r="B13" s="46" t="n"/>
+      <c r="C13" s="57">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="55">
+      <c r="D13" s="57">
         <f>SUM(D8:D12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
+      <c r="B14" s="33" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -4666,16 +4870,16 @@
           <t>Уборка и снегоуборка</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C15" s="56">
+      <c r="C15" s="58">
         <f>$D$4*Нормативы!G5*12/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="56">
+      <c r="D15" s="58">
         <f>$D$4*Нормативы!H5*12/1000000</f>
         <v/>
       </c>
@@ -4686,16 +4890,16 @@
           <t>Озеленение и полив</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C16" s="56">
+      <c r="C16" s="58">
         <f>$D$3*Нормативы!G6*7/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="56">
+      <c r="D16" s="58">
         <f>$D$3*Нормативы!H6*7/1000000</f>
         <v/>
       </c>
@@ -4706,16 +4910,16 @@
           <t>Свет, электро, digital</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="58">
         <f>$D$4*Нормативы!G7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="56">
+      <c r="D17" s="58">
         <f>$D$4*Нормативы!H7/1000000</f>
         <v/>
       </c>
@@ -4726,16 +4930,16 @@
           <t>Зимний пакет</t>
         </is>
       </c>
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="58">
         <f>Нормативы!G10</f>
         <v/>
       </c>
-      <c r="D18" s="56">
+      <c r="D18" s="58">
         <f>Нормативы!H10</f>
         <v/>
       </c>
@@ -4746,16 +4950,16 @@
           <t>Программа и маркетинг</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="58">
         <f>Нормативы!G9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D19" s="56">
+      <c r="D19" s="58">
         <f>Нормативы!H9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -4766,16 +4970,16 @@
           <t>Координатор кластера</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C20" s="56">
+      <c r="C20" s="58">
         <f>Нормативы!$C$15*Нормативы!G8*12/1000</f>
         <v/>
       </c>
-      <c r="D20" s="56">
+      <c r="D20" s="58">
         <f>Нормативы!$D$15*Нормативы!H8*12/1000</f>
         <v/>
       </c>
@@ -4786,45 +4990,45 @@
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B21" s="26" t="inlineStr">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C21" s="56">
+      <c r="C21" s="58">
         <f>Нормативы!$C$17*($B$4+Нормативы!G12)</f>
         <v/>
       </c>
-      <c r="D21" s="56">
+      <c r="D21" s="58">
         <f>Нормативы!$D$17*($B$4+Нормативы!H12)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="57" t="inlineStr">
+      <c r="A22" s="59" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B22" s="43" t="n"/>
-      <c r="C22" s="58">
+      <c r="B22" s="46" t="n"/>
+      <c r="C22" s="60">
         <f>SUM(C15:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="58">
+      <c r="D22" s="60">
         <f>SUM(D15:D21)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="53" t="inlineStr">
+      <c r="A24" s="55" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B24" s="31" t="n"/>
-      <c r="C24" s="31" t="n"/>
-      <c r="D24" s="31" t="n"/>
+      <c r="B24" s="33" t="n"/>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -4832,16 +5036,16 @@
           <t>Консервативный сценарий</t>
         </is>
       </c>
-      <c r="B25" s="26" t="inlineStr">
+      <c r="B25" s="28" t="inlineStr">
         <is>
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C25" s="59">
+      <c r="C25" s="61">
         <f>IFERROR(C13/D22,0)</f>
         <v/>
       </c>
-      <c r="D25" s="31" t="n"/>
+      <c r="D25" s="33" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -4849,16 +5053,16 @@
           <t>По середине вилок</t>
         </is>
       </c>
-      <c r="B26" s="26" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
         <is>
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C26" s="59">
+      <c r="C26" s="61">
         <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C22:D22),0)</f>
         <v/>
       </c>
-      <c r="D26" s="31" t="n"/>
+      <c r="D26" s="33" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -4866,57 +5070,57 @@
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B27" s="26" t="inlineStr">
+      <c r="B27" s="28" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C27" s="59">
+      <c r="C27" s="61">
         <f>IFERROR(D13/C22,0)</f>
         <v/>
       </c>
-      <c r="D27" s="31" t="n"/>
+      <c r="D27" s="33" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="60" t="inlineStr">
+      <c r="A28" s="62" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B28" s="31" t="n"/>
-      <c r="C28" s="61" t="inlineStr">
+      <c r="B28" s="33" t="n"/>
+      <c r="C28" s="63" t="inlineStr">
         <is>
           <t>70–100%</t>
         </is>
       </c>
-      <c r="D28" s="31" t="n"/>
+      <c r="D28" s="33" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="53" t="inlineStr">
+      <c r="A30" s="55" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B30" s="31" t="n"/>
-      <c r="C30" s="31" t="n"/>
-      <c r="D30" s="31" t="n"/>
+      <c r="B30" s="33" t="n"/>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="33" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="62" t="inlineStr">
+      <c r="A31" s="64" t="inlineStr">
         <is>
           <t>• Каток отработал первую зиму без простоев</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr">
+      <c r="A32" s="64" t="inlineStr">
         <is>
           <t>• Заявок на события больше, чем слотов</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr">
+      <c r="A33" s="64" t="inlineStr">
         <is>
           <t>• Спонсор года подписан до старта сезона</t>
         </is>
@@ -4967,49 +5171,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="47" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>Финмодель Т4 · Парк по ГЧП (BTO)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="48" t="inlineStr">
+      <c r="A3" s="50" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="49" t="inlineStr">
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>Sphere Park</t>
         </is>
       </c>
-      <c r="C3" s="50" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="51">
+      <c r="D3" s="53">
         <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="52">
+      <c r="B4" s="54">
         <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
         <v/>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="53">
         <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
         <v/>
       </c>
@@ -5037,14 +5241,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
+      <c r="B7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -5052,15 +5256,15 @@
           <t>Компенсация эксплуатации (акимат)</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>структура BTO: ~0,33 млрд тг за 5 лет</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
+      <c r="C8" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="35" t="n">
         <v>70</v>
       </c>
     </row>
@@ -5070,15 +5274,15 @@
           <t>НТО-точки, 3–5 шт</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>кофе, стритфуд, прокат</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C9" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="35" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5088,15 +5292,15 @@
           <t>Каток и зимний прокат</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>большой контур, 120–160 дней</t>
         </is>
       </c>
-      <c r="C10" s="33" t="n">
+      <c r="C10" s="35" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="35" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5106,15 +5310,15 @@
           <t>Событийная аренда и фестивали</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>городской масштаб</t>
         </is>
       </c>
-      <c r="C11" s="33" t="n">
+      <c r="C11" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="35" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5124,15 +5328,15 @@
           <t>Ярмарки и маркеты</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>круглогодично</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n">
+      <c r="C12" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="35" t="n">
         <v>4</v>
       </c>
     </row>
@@ -5142,43 +5346,43 @@
           <t>Спонсоры и реклама</t>
         </is>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>якорные партнёры</t>
         </is>
       </c>
-      <c r="C13" s="33" t="n">
+      <c r="C13" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="33" t="n">
+      <c r="D13" s="35" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="54" t="inlineStr">
+      <c r="A14" s="56" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
-      <c r="B14" s="43" t="n"/>
-      <c r="C14" s="55">
+      <c r="B14" s="46" t="n"/>
+      <c r="C14" s="57">
         <f>SUM(C8:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="55">
+      <c r="D14" s="57">
         <f>SUM(D8:D13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="53" t="inlineStr">
+      <c r="A15" s="55" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
       </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="31" t="n"/>
+      <c r="B15" s="33" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="33" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -5186,16 +5390,16 @@
           <t>Уборка и снегоуборка</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="56">
+      <c r="C16" s="58">
         <f>$D$4*Нормативы!I5*12/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="56">
+      <c r="D16" s="58">
         <f>$D$4*Нормативы!J5*12/1000000</f>
         <v/>
       </c>
@@ -5206,16 +5410,16 @@
           <t>Озеленение и полив</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="58">
         <f>$D$3*Нормативы!I6*7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="56">
+      <c r="D17" s="58">
         <f>$D$3*Нормативы!J6*7/1000000</f>
         <v/>
       </c>
@@ -5226,16 +5430,16 @@
           <t>Свет, электро, digital</t>
         </is>
       </c>
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="58">
         <f>$D$4*Нормативы!I7/1000000</f>
         <v/>
       </c>
-      <c r="D18" s="56">
+      <c r="D18" s="58">
         <f>$D$4*Нормативы!J7/1000000</f>
         <v/>
       </c>
@@ -5246,16 +5450,16 @@
           <t>Зимний пакет</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="58">
         <f>Нормативы!I10</f>
         <v/>
       </c>
-      <c r="D19" s="56">
+      <c r="D19" s="58">
         <f>Нормативы!J10</f>
         <v/>
       </c>
@@ -5266,16 +5470,16 @@
           <t>Программа и маркетинг</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C20" s="56">
+      <c r="C20" s="58">
         <f>Нормативы!I9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D20" s="56">
+      <c r="D20" s="58">
         <f>Нормативы!J9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -5286,16 +5490,16 @@
           <t>Персонал парка</t>
         </is>
       </c>
-      <c r="B21" s="26" t="inlineStr">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C21" s="56">
+      <c r="C21" s="58">
         <f>Нормативы!I11</f>
         <v/>
       </c>
-      <c r="D21" s="56">
+      <c r="D21" s="58">
         <f>Нормативы!J11</f>
         <v/>
       </c>
@@ -5306,45 +5510,45 @@
           <t>Ремфонд</t>
         </is>
       </c>
-      <c r="B22" s="26" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C22" s="56">
+      <c r="C22" s="58">
         <f>Нормативы!$C$17*($B$4+Нормативы!I12)</f>
         <v/>
       </c>
-      <c r="D22" s="56">
+      <c r="D22" s="58">
         <f>Нормативы!$D$17*($B$4+Нормативы!J12)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="57" t="inlineStr">
+      <c r="A23" s="59" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
-      <c r="B23" s="43" t="n"/>
-      <c r="C23" s="58">
+      <c r="B23" s="46" t="n"/>
+      <c r="C23" s="60">
         <f>SUM(C16:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="58">
+      <c r="D23" s="60">
         <f>SUM(D16:D22)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="53" t="inlineStr">
+      <c r="A25" s="55" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
       </c>
-      <c r="B25" s="31" t="n"/>
-      <c r="C25" s="31" t="n"/>
-      <c r="D25" s="31" t="n"/>
+      <c r="B25" s="33" t="n"/>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="33" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -5352,16 +5556,16 @@
           <t>Консервативный сценарий</t>
         </is>
       </c>
-      <c r="B26" s="26" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
         <is>
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C26" s="59">
+      <c r="C26" s="61">
         <f>IFERROR(C14/D23,0)</f>
         <v/>
       </c>
-      <c r="D26" s="31" t="n"/>
+      <c r="D26" s="33" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -5369,16 +5573,16 @@
           <t>По середине вилок</t>
         </is>
       </c>
-      <c r="B27" s="26" t="inlineStr">
+      <c r="B27" s="28" t="inlineStr">
         <is>
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C27" s="59">
+      <c r="C27" s="61">
         <f>IFERROR(AVERAGE(C14:D14)/AVERAGE(C23:D23),0)</f>
         <v/>
       </c>
-      <c r="D27" s="31" t="n"/>
+      <c r="D27" s="33" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -5386,71 +5590,71 @@
           <t>Оптимистичный сценарий</t>
         </is>
       </c>
-      <c r="B28" s="26" t="inlineStr">
+      <c r="B28" s="28" t="inlineStr">
         <is>
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C28" s="59">
+      <c r="C28" s="61">
         <f>IFERROR(D14/C23,0)</f>
         <v/>
       </c>
-      <c r="D28" s="31" t="n"/>
+      <c r="D28" s="33" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="60" t="inlineStr">
+      <c r="A29" s="62" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
-      <c r="B29" s="31" t="n"/>
-      <c r="C29" s="61" t="inlineStr">
+      <c r="B29" s="33" t="n"/>
+      <c r="C29" s="63" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
       </c>
-      <c r="D29" s="31" t="n"/>
+      <c r="D29" s="33" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="53" t="inlineStr">
+      <c r="A31" s="55" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
       </c>
-      <c r="B31" s="31" t="n"/>
-      <c r="C31" s="31" t="n"/>
-      <c r="D31" s="31" t="n"/>
+      <c r="B31" s="33" t="n"/>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="33" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr">
+      <c r="A32" s="64" t="inlineStr">
         <is>
           <t>• Ремфонд и капремонт сидят в компенсации эксплуатации (BTO), в OPEX не дублируются</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr">
+      <c r="A33" s="64" t="inlineStr">
         <is>
           <t>• ГЧП-договор подписан, компенсация в бюджете МИО</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="62" t="inlineStr">
+      <c r="A34" s="64" t="inlineStr">
         <is>
           <t>• Каток и события дотягивают покрытие до 100%+</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="62" t="inlineStr">
+      <c r="A35" s="64" t="inlineStr">
         <is>
           <t>• Стандарт содержания выше городского бенчмарка</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="62" t="inlineStr">
+      <c r="A36" s="64" t="inlineStr">
         <is>
           <t>• CAPEX ~2,2 млрд тг компенсируется бюджетом МИО отдельно (2026–2031) — в операционную модель не входит</t>
         </is>

</xml_diff>

<commit_message>
Rework pilot perimeter: Grand Turan + four-alley cluster, budget sheet
Deck (33 slides): pilot set changed after the site visit — Grand Turan
as a standalone contour plus a cluster of Headliner Exclusive, Flora 1,
Flora 2 and Aura; Avenue 5 moved to reserve. New maintenance budget
slide (18-29M KZT/yr) and next-steps slide (legal audit, budget
approval, winter operators); satellite slide now shows the new
perimeter.

Workbook v6: four-alley cluster object in the registry and Assets
sheet, T2 model defaults to the cluster, new Pilot Budget sheet with
per-object maintenance formulas and cluster coordinator at 0.93 FTE.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014o1yT6nCgffZ5H25q7THst
</commit_message>
<xml_diff>
--- a/docs/research/BIG-Life-finmodels-T1-T4.xlsx
+++ b/docs/research/BIG-Life-finmodels-T1-T4.xlsx
@@ -11,10 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нормативы" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Активы" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т1 Транзитная" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т2 Активная" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т3 Сквер" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т4 Sphere Park" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бюджет пилота" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т1 Транзитная" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т2 Активная" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т3 Сквер" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Т4 Sphere Park" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,18 +71,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001E7A45"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001B2A6E"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001E7A45"/>
       <sz val="9.5"/>
     </font>
     <font>
@@ -141,6 +142,23 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="008A93A6"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="008A93A6"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001B2A6E"/>
       <sz val="14"/>
     </font>
@@ -183,12 +201,6 @@
       <b val="1"/>
       <color rgb="001B2A6E"/>
       <sz val="10.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="008A93A6"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -267,10 +279,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -281,22 +293,22 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -315,10 +327,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -357,7 +369,7 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -381,35 +393,56 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="27" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="28" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -805,7 +838,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая — фактический обмер Google Earth для группы A (для незамеренных: озеленение × коэффициент). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Жёлтые ячейки — редактируемые ставки.</t>
+          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая — фактический обмер Google Earth для группы A (для незамеренных: озеленение × коэффициент). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Лист «Бюджет пилота» — годовое содержание выбранного периметра: Гранд Туран + кластер из четырёх. Жёлтые ячейки — редактируемые ставки.</t>
         </is>
       </c>
     </row>
@@ -825,7 +858,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Т2 · Хедлайнер Экс.</t>
+          <t>Т2 · Пилотный кластер</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1144,7 +1177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1263,7 +1296,7 @@
       <c r="A5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
@@ -1284,9 +1317,9 @@
       <c r="F5" s="17" t="n">
         <v>3114</v>
       </c>
-      <c r="G5" s="22" t="inlineStr">
-        <is>
-          <t>Пилот</t>
+      <c r="G5" s="21" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
@@ -1362,7 +1395,7 @@
       <c r="F7" s="17" t="n">
         <v>10805</v>
       </c>
-      <c r="G7" s="23" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1380,7 +1413,7 @@
       <c r="A8" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Аура Аллея</t>
         </is>
@@ -1403,7 +1436,7 @@
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Пилот</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
@@ -1419,7 +1452,7 @@
       <c r="A9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
@@ -1440,7 +1473,7 @@
       <c r="F9" s="17" t="n">
         <v>4100</v>
       </c>
-      <c r="G9" s="22" t="inlineStr">
+      <c r="G9" s="23" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1458,7 +1491,7 @@
       <c r="A10" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Аллея Гранд Туран Комфорт</t>
         </is>
@@ -1481,7 +1514,7 @@
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Пилот</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
@@ -1497,7 +1530,7 @@
       <c r="A11" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 1</t>
         </is>
@@ -1518,7 +1551,7 @@
       <c r="F11" s="17" t="n">
         <v>1512</v>
       </c>
-      <c r="G11" s="22" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1536,7 +1569,7 @@
       <c r="A12" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 2</t>
         </is>
@@ -1557,7 +1590,7 @@
       <c r="F12" s="17" t="n">
         <v>1210</v>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
@@ -1596,7 +1629,7 @@
       <c r="F13" s="17" t="n">
         <v>2843</v>
       </c>
-      <c r="G13" s="23" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1929,7 +1962,7 @@
       <c r="F21" s="26" t="n">
         <v>4200</v>
       </c>
-      <c r="G21" s="23" t="inlineStr">
+      <c r="G21" s="21" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -2536,7 +2569,7 @@
       <c r="A36" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="21" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
@@ -2558,17 +2591,57 @@
         <f>F11+F12</f>
         <v/>
       </c>
-      <c r="G36" s="22" t="inlineStr">
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>вспомогательная строка: две Flora вместе</t>
+        </is>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>Пилотный кластер: Хедлайнер + Flora + Аура</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Т2</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="n">
+        <v>5476</v>
+      </c>
+      <c r="F37" s="18">
+        <f>F8+F9+F11+F12</f>
+        <v/>
+      </c>
+      <c r="G37" s="23" t="inlineStr">
         <is>
           <t>Пилот</t>
         </is>
       </c>
-      <c r="H36" s="16" t="inlineStr">
-        <is>
-          <t>пилот Т1: два объекта под одной командой</t>
-        </is>
-      </c>
-      <c r="I36" s="20" t="n">
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>пилот: 4 аллеи одной командой — Хедлайнер Эксклюзив, Flora 1, Flora 2, Аура</t>
+        </is>
+      </c>
+      <c r="I37" s="20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3075,7 +3148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3169,17 +3242,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Сквер Авеню 5</t>
         </is>
       </c>
       <c r="B4" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A4,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A4,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C4" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A4,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A4,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D4" s="38" t="n">
@@ -3215,17 +3288,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 1</t>
         </is>
       </c>
       <c r="B5" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A5,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A5,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C5" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A5,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A5,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D5" s="38" t="n">
@@ -3261,17 +3334,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 2</t>
         </is>
       </c>
       <c r="B6" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A6,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A6,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C6" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A6,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A6,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D6" s="38" t="n">
@@ -3307,17 +3380,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
       </c>
       <c r="B7" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A7,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A7,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C7" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A7,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A7,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D7" s="42" t="n">
@@ -3359,11 +3432,11 @@
         </is>
       </c>
       <c r="B8" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A8,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A8,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A8,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A8,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D8" s="38" t="n">
@@ -3405,11 +3478,11 @@
         </is>
       </c>
       <c r="B9" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A9,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A9,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A9,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A9,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D9" s="38" t="n">
@@ -3451,11 +3524,11 @@
         </is>
       </c>
       <c r="B10" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A10,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A10,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A10,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A10,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D10" s="38" t="n">
@@ -3497,11 +3570,11 @@
         </is>
       </c>
       <c r="B11" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A11,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A11,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A11,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A11,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D11" s="38" t="n">
@@ -3543,11 +3616,11 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A12,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A12,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C12" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A12,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A12,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D12" s="38" t="n">
@@ -3589,11 +3662,11 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A13,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A13,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C13" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A13,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A13,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D13" s="38" t="n">
@@ -3677,17 +3750,17 @@
       <c r="L15" s="46" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
       </c>
       <c r="B16" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($A16,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A16,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="C16" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($A16,Объекты!$B$4:$B$36,0)),"")</f>
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A16,Объекты!$B$4:$B$37,0)),"")</f>
         <v/>
       </c>
       <c r="D16" s="40">
@@ -3725,6 +3798,58 @@
       <c r="L16" s="48" t="inlineStr">
         <is>
           <t>строка для выпадающего списка Т1: сумма двух Flora</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Пилотный кластер: Хедлайнер + Flora + Аура</t>
+        </is>
+      </c>
+      <c r="B17" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A17,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A17,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D17" s="40">
+        <f>D7+D5+D6+D8</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>E7+E5+E6+E8</f>
+        <v/>
+      </c>
+      <c r="F17" s="40">
+        <f>F7+F5+F6+F8</f>
+        <v/>
+      </c>
+      <c r="G17" s="40">
+        <f>G7+G5+G6+G8</f>
+        <v/>
+      </c>
+      <c r="H17" s="40">
+        <f>H7+H5+H6+H8</f>
+        <v/>
+      </c>
+      <c r="I17" s="40">
+        <f>I7+I5+I6+I8</f>
+        <v/>
+      </c>
+      <c r="J17" s="47">
+        <f>SUM(D17:I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="40">
+        <f>IFERROR(J17/C17*1000,"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="48" t="inlineStr">
+        <is>
+          <t>пилот: сумма четырёх аллей; активы Хедлайнера войдут после справки</t>
         </is>
       </c>
     </row>
@@ -3743,6 +3868,606 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8.5" customWidth="1" min="5" max="5"/>
+    <col width="8.5" customWidth="1" min="6" max="6"/>
+    <col width="8.5" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="8" max="8"/>
+    <col width="8.5" customWidth="1" min="9" max="9"/>
+    <col width="8.5" customWidth="1" min="10" max="10"/>
+    <col width="8.5" customWidth="1" min="11" max="11"/>
+    <col width="8.5" customWidth="1" min="12" max="12"/>
+    <col width="9.5" customWidth="1" min="13" max="13"/>
+    <col width="9.5" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Годовой бюджет содержания пилотного периметра</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Содержание as-is: уборка и свет от общей площади (обмер), озеленение от зелёной, ремфонд от активов на балансе, координация по долям ставок. Все ставки — лист «Нормативы». Программа активации — справочно, отдельной строкой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="49" t="inlineStr">
+        <is>
+          <t>Объект</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="C4" s="50" t="inlineStr">
+        <is>
+          <t>Озеленение, м²</t>
+        </is>
+      </c>
+      <c r="D4" s="50" t="inlineStr">
+        <is>
+          <t>Общая, м²</t>
+        </is>
+      </c>
+      <c r="E4" s="50" t="inlineStr">
+        <is>
+          <t>Уборка мин</t>
+        </is>
+      </c>
+      <c r="F4" s="50" t="inlineStr">
+        <is>
+          <t>Уборка макс</t>
+        </is>
+      </c>
+      <c r="G4" s="50" t="inlineStr">
+        <is>
+          <t>Озелен. мин</t>
+        </is>
+      </c>
+      <c r="H4" s="50" t="inlineStr">
+        <is>
+          <t>Озелен. макс</t>
+        </is>
+      </c>
+      <c r="I4" s="50" t="inlineStr">
+        <is>
+          <t>Свет мин</t>
+        </is>
+      </c>
+      <c r="J4" s="50" t="inlineStr">
+        <is>
+          <t>Свет макс</t>
+        </is>
+      </c>
+      <c r="K4" s="50" t="inlineStr">
+        <is>
+          <t>Ремфонд мин</t>
+        </is>
+      </c>
+      <c r="L4" s="50" t="inlineStr">
+        <is>
+          <t>Ремфонд макс</t>
+        </is>
+      </c>
+      <c r="M4" s="50" t="inlineStr">
+        <is>
+          <t>Итого мин</t>
+        </is>
+      </c>
+      <c r="N4" s="50" t="inlineStr">
+        <is>
+          <t>Итого макс</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Аллея Гранд Туран Комфорт</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Т2</t>
+        </is>
+      </c>
+      <c r="C5" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A5,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A5,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E5" s="51">
+        <f>$D5*Нормативы!E5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="F5" s="51">
+        <f>$D5*Нормативы!F5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="G5" s="51">
+        <f>$C5*Нормативы!E6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="H5" s="51">
+        <f>$C5*Нормативы!F6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="I5" s="51">
+        <f>$D5*Нормативы!E7/1000000</f>
+        <v/>
+      </c>
+      <c r="J5" s="51">
+        <f>$D5*Нормативы!F7/1000000</f>
+        <v/>
+      </c>
+      <c r="K5" s="51">
+        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A5,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="L5" s="51">
+        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A5,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="M5" s="39">
+        <f>E5+G5+I5+K5</f>
+        <v/>
+      </c>
+      <c r="N5" s="39">
+        <f>F5+H5+J5+L5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Аллея Хедлайнер Эксклюзив</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Т2</t>
+        </is>
+      </c>
+      <c r="C6" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A6,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D6" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A6,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E6" s="51">
+        <f>$D6*Нормативы!E5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="F6" s="51">
+        <f>$D6*Нормативы!F5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="G6" s="51">
+        <f>$C6*Нормативы!E6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="H6" s="51">
+        <f>$C6*Нормативы!F6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="I6" s="51">
+        <f>$D6*Нормативы!E7/1000000</f>
+        <v/>
+      </c>
+      <c r="J6" s="51">
+        <f>$D6*Нормативы!F7/1000000</f>
+        <v/>
+      </c>
+      <c r="K6" s="51">
+        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A6,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="L6" s="51">
+        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A6,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="M6" s="39">
+        <f>E6+G6+I6+K6</f>
+        <v/>
+      </c>
+      <c r="N6" s="39">
+        <f>F6+H6+J6+L6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Аллея ЖК Flora 1</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Т1</t>
+        </is>
+      </c>
+      <c r="C7" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A7,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D7" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A7,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E7" s="51">
+        <f>$D7*Нормативы!C5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="F7" s="51">
+        <f>$D7*Нормативы!D5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="G7" s="51">
+        <f>$C7*Нормативы!C6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="H7" s="51">
+        <f>$C7*Нормативы!D6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="I7" s="51">
+        <f>$D7*Нормативы!C7/1000000</f>
+        <v/>
+      </c>
+      <c r="J7" s="51">
+        <f>$D7*Нормативы!D7/1000000</f>
+        <v/>
+      </c>
+      <c r="K7" s="51">
+        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A7,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="L7" s="51">
+        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A7,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="M7" s="39">
+        <f>E7+G7+I7+K7</f>
+        <v/>
+      </c>
+      <c r="N7" s="39">
+        <f>F7+H7+J7+L7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Аллея ЖК Flora 2</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Т1</t>
+        </is>
+      </c>
+      <c r="C8" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A8,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A8,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="51">
+        <f>$D8*Нормативы!C5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="F8" s="51">
+        <f>$D8*Нормативы!D5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="G8" s="51">
+        <f>$C8*Нормативы!C6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="H8" s="51">
+        <f>$C8*Нормативы!D6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="I8" s="51">
+        <f>$D8*Нормативы!C7/1000000</f>
+        <v/>
+      </c>
+      <c r="J8" s="51">
+        <f>$D8*Нормативы!D7/1000000</f>
+        <v/>
+      </c>
+      <c r="K8" s="51">
+        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A8,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="L8" s="51">
+        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A8,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="M8" s="39">
+        <f>E8+G8+I8+K8</f>
+        <v/>
+      </c>
+      <c r="N8" s="39">
+        <f>F8+H8+J8+L8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Аура Аллея</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Т1</t>
+        </is>
+      </c>
+      <c r="C9" s="18">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A9,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A9,Объекты!$B$4:$B$37,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E9" s="51">
+        <f>$D9*Нормативы!C5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="F9" s="51">
+        <f>$D9*Нормативы!D5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="G9" s="51">
+        <f>$C9*Нормативы!C6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="H9" s="51">
+        <f>$C9*Нормативы!D6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="I9" s="51">
+        <f>$D9*Нормативы!C7/1000000</f>
+        <v/>
+      </c>
+      <c r="J9" s="51">
+        <f>$D9*Нормативы!D7/1000000</f>
+        <v/>
+      </c>
+      <c r="K9" s="51">
+        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A9,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="L9" s="51">
+        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A9,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="M9" s="39">
+        <f>E9+G9+I9+K9</f>
+        <v/>
+      </c>
+      <c r="N9" s="39">
+        <f>F9+H9+J9+L9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>Координатор кластера (сумма долей: Т2 + 3 × Т1)</t>
+        </is>
+      </c>
+      <c r="B10" s="53" t="inlineStr">
+        <is>
+          <t>один координатор на четыре аллеи: 0,33 + 3 × 0,20 = 0,93 ставки</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="33" t="n"/>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="33" t="n"/>
+      <c r="I10" s="33" t="n"/>
+      <c r="J10" s="33" t="n"/>
+      <c r="K10" s="33" t="n"/>
+      <c r="L10" s="33" t="n"/>
+      <c r="M10" s="38">
+        <f>(Нормативы!E8+3*Нормативы!C8)*Нормативы!$C$15*12/1000</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>(Нормативы!F8+3*Нормативы!D8)*Нормативы!$D$15*12/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>Координатор Гранд Турана (доля Т2)</t>
+        </is>
+      </c>
+      <c r="B11" s="53" t="inlineStr">
+        <is>
+          <t>0,33 ставки; при расширении Управления 4 станет кластерным</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="33" t="n"/>
+      <c r="F11" s="33" t="n"/>
+      <c r="G11" s="33" t="n"/>
+      <c r="H11" s="33" t="n"/>
+      <c r="I11" s="33" t="n"/>
+      <c r="J11" s="33" t="n"/>
+      <c r="K11" s="33" t="n"/>
+      <c r="L11" s="33" t="n"/>
+      <c r="M11" s="38">
+        <f>Нормативы!E8*Нормативы!$C$15*12/1000</f>
+        <v/>
+      </c>
+      <c r="N11" s="38">
+        <f>Нормативы!F8*Нормативы!$D$15*12/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="54" t="inlineStr">
+        <is>
+          <t>Кластер (Хедлайнер + Flora 1, 2 + Аура), итого</t>
+        </is>
+      </c>
+      <c r="B13" s="46" t="n"/>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="33" t="n"/>
+      <c r="F13" s="33" t="n"/>
+      <c r="G13" s="33" t="n"/>
+      <c r="H13" s="33" t="n"/>
+      <c r="I13" s="33" t="n"/>
+      <c r="J13" s="33" t="n"/>
+      <c r="K13" s="33" t="n"/>
+      <c r="L13" s="33" t="n"/>
+      <c r="M13" s="55">
+        <f>M6+M7+M8+M9+M10</f>
+        <v/>
+      </c>
+      <c r="N13" s="55">
+        <f>N6+N7+N8+N9+N10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>Гранд Туран, итого</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
+      <c r="E14" s="33" t="n"/>
+      <c r="F14" s="33" t="n"/>
+      <c r="G14" s="33" t="n"/>
+      <c r="H14" s="33" t="n"/>
+      <c r="I14" s="33" t="n"/>
+      <c r="J14" s="33" t="n"/>
+      <c r="K14" s="33" t="n"/>
+      <c r="L14" s="33" t="n"/>
+      <c r="M14" s="55">
+        <f>M5+M11</f>
+        <v/>
+      </c>
+      <c r="N14" s="55">
+        <f>N5+N11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="56" t="inlineStr">
+        <is>
+          <t>ПИЛОТ: СОДЕРЖАНИЕ, ИТОГО</t>
+        </is>
+      </c>
+      <c r="B15" s="46" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="33" t="n"/>
+      <c r="E15" s="33" t="n"/>
+      <c r="F15" s="33" t="n"/>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="33" t="n"/>
+      <c r="I15" s="33" t="n"/>
+      <c r="J15" s="33" t="n"/>
+      <c r="K15" s="33" t="n"/>
+      <c r="L15" s="33" t="n"/>
+      <c r="M15" s="57">
+        <f>M13+M14</f>
+        <v/>
+      </c>
+      <c r="N15" s="57">
+        <f>N13+N14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="52" t="inlineStr">
+        <is>
+          <t>Программа активации (справочно, два контура)</t>
+        </is>
+      </c>
+      <c r="B17" s="53" t="inlineStr">
+        <is>
+          <t>события по нормативу Т2 на каждый контур; это активация, в содержание не входит</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n"/>
+      <c r="D17" s="33" t="n"/>
+      <c r="E17" s="33" t="n"/>
+      <c r="F17" s="33" t="n"/>
+      <c r="G17" s="33" t="n"/>
+      <c r="H17" s="33" t="n"/>
+      <c r="I17" s="33" t="n"/>
+      <c r="J17" s="33" t="n"/>
+      <c r="K17" s="33" t="n"/>
+      <c r="L17" s="33" t="n"/>
+      <c r="M17" s="38">
+        <f>2*Нормативы!E9*Нормативы!$C$16/1000</f>
+        <v/>
+      </c>
+      <c r="N17" s="38">
+        <f>2*Нормативы!F9*Нормативы!$D$16/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Ремфонд Хедлайнера сейчас 0: справка о балансовой стоимости запрошена — суммы добавятся в лист «Активы» и бюджет пересчитается. Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="A19:N20"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3753,50 +4478,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Финмодель Т1 · Транзитная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="51" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>Аллеи ЖК Flora 1 + 2 (кластер)</t>
         </is>
       </c>
-      <c r="C3" s="52" t="inlineStr">
+      <c r="C3" s="61" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="53">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+      <c r="D3" s="62">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="59" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="54">
-        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
+      <c r="B4" s="63">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($B$3,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="53">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+      <c r="D4" s="62">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -3823,7 +4548,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="55" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -3887,23 +4612,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="56" t="inlineStr">
+      <c r="A11" s="65" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
       <c r="B11" s="46" t="n"/>
-      <c r="C11" s="57">
+      <c r="C11" s="66">
         <f>SUM(C8:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="57">
+      <c r="D11" s="66">
         <f>SUM(D8:D10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="55" t="inlineStr">
+      <c r="A12" s="64" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -3923,11 +4648,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C13" s="58">
+      <c r="C13" s="67">
         <f>$D$4*Нормативы!C5*12/1000000</f>
         <v/>
       </c>
-      <c r="D13" s="58">
+      <c r="D13" s="67">
         <f>$D$4*Нормативы!D5*12/1000000</f>
         <v/>
       </c>
@@ -3943,11 +4668,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C14" s="58">
+      <c r="C14" s="67">
         <f>$D$3*Нормативы!C6*7/1000000</f>
         <v/>
       </c>
-      <c r="D14" s="58">
+      <c r="D14" s="67">
         <f>$D$3*Нормативы!D6*7/1000000</f>
         <v/>
       </c>
@@ -3963,11 +4688,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C15" s="58">
+      <c r="C15" s="67">
         <f>$D$4*Нормативы!C7/1000000</f>
         <v/>
       </c>
-      <c r="D15" s="58">
+      <c r="D15" s="67">
         <f>$D$4*Нормативы!D7/1000000</f>
         <v/>
       </c>
@@ -3983,11 +4708,11 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="58">
+      <c r="C16" s="67">
         <f>Нормативы!$C$15*Нормативы!C8*12/1000</f>
         <v/>
       </c>
-      <c r="D16" s="58">
+      <c r="D16" s="67">
         <f>Нормативы!$D$15*Нормативы!D8*12/1000</f>
         <v/>
       </c>
@@ -4003,33 +4728,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C17" s="58">
+      <c r="C17" s="67">
         <f>Нормативы!$C$17*($B$4+Нормативы!C12)</f>
         <v/>
       </c>
-      <c r="D17" s="58">
+      <c r="D17" s="67">
         <f>Нормативы!$D$17*($B$4+Нормативы!D12)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="68" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
       <c r="B18" s="46" t="n"/>
-      <c r="C18" s="60">
+      <c r="C18" s="69">
         <f>SUM(C13:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="60">
+      <c r="D18" s="69">
         <f>SUM(D13:D17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="55" t="inlineStr">
+      <c r="A20" s="64" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -4049,7 +4774,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C21" s="61">
+      <c r="C21" s="70">
         <f>IFERROR(C11/D18,0)</f>
         <v/>
       </c>
@@ -4066,7 +4791,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C22" s="61">
+      <c r="C22" s="70">
         <f>IFERROR(AVERAGE(C11:D11)/AVERAGE(C18:D18),0)</f>
         <v/>
       </c>
@@ -4083,20 +4808,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C23" s="61">
+      <c r="C23" s="70">
         <f>IFERROR(D11/C18,0)</f>
         <v/>
       </c>
       <c r="D23" s="33" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="62" t="inlineStr">
+      <c r="A24" s="71" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B24" s="33" t="n"/>
-      <c r="C24" s="63" t="inlineStr">
+      <c r="C24" s="72" t="inlineStr">
         <is>
           <t>10–30%</t>
         </is>
@@ -4104,7 +4829,7 @@
       <c r="D24" s="33" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="55" t="inlineStr">
+      <c r="A26" s="64" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -4114,21 +4839,21 @@
       <c r="D26" s="33" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="64" t="inlineStr">
+      <c r="A27" s="73" t="inlineStr">
         <is>
           <t>• Кластер: общий координатор и бригада, не своя</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="64" t="inlineStr">
+      <c r="A28" s="73" t="inlineStr">
         <is>
           <t>• Спонсоры продлеваются на второй год</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="64" t="inlineStr">
+      <c r="A29" s="73" t="inlineStr">
         <is>
           <t>• Юрстатус пропускает рекламу на стелах</t>
         </is>
@@ -4156,497 +4881,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$36</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="49" t="inlineStr">
-        <is>
-          <t>Финмодель Т2 · Активная аллея</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="50" t="inlineStr">
-        <is>
-          <t>Объект (выберите из списка):</t>
-        </is>
-      </c>
-      <c r="B3" s="51" t="inlineStr">
-        <is>
-          <t>Аллея Хедлайнер Эксклюзив</t>
-        </is>
-      </c>
-      <c r="C3" s="52" t="inlineStr">
-        <is>
-          <t>Озеленение, м²:</t>
-        </is>
-      </c>
-      <c r="D3" s="53">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="50" t="inlineStr">
-        <is>
-          <t>Активы на балансе, млн тг:</t>
-        </is>
-      </c>
-      <c r="B4" s="54">
-        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
-        <is>
-          <t>Общая площадь, м²:</t>
-        </is>
-      </c>
-      <c r="D4" s="53">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Как считаем / привязка</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Мин, млн тг/год</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Макс, млн тг/год</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="55" t="inlineStr">
-        <is>
-          <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
-        </is>
-      </c>
-      <c r="B7" s="33" t="n"/>
-      <c r="C7" s="33" t="n"/>
-      <c r="D7" s="33" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>НТО-якорь: кофе-павильон</t>
-        </is>
-      </c>
-      <c r="B8" s="28" t="inlineStr">
-        <is>
-          <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
-        </is>
-      </c>
-      <c r="C8" s="35" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="D8" s="35" t="n">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Ярмарка выходного дня</t>
-        </is>
-      </c>
-      <c r="B9" s="28" t="inlineStr">
-        <is>
-          <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
-        </is>
-      </c>
-      <c r="C9" s="35" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D9" s="35" t="n">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Секции и кикшеринг</t>
-        </is>
-      </c>
-      <c r="B10" s="28" t="inlineStr">
-        <is>
-          <t>слоты тренерам + rev-share операторов</t>
-        </is>
-      </c>
-      <c r="C10" s="35" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D10" s="35" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Digital-экран и реклама</t>
-        </is>
-      </c>
-      <c r="B11" s="28" t="inlineStr">
-        <is>
-          <t>при подходящем юрстатусе земли</t>
-        </is>
-      </c>
-      <c r="C11" s="35" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D11" s="35" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Спонсорство объектов</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t>воркаут, клумбы, скамейки</t>
-        </is>
-      </c>
-      <c r="C12" s="35" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D12" s="35" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="56" t="inlineStr">
-        <is>
-          <t>Доходы, итого</t>
-        </is>
-      </c>
-      <c r="B13" s="46" t="n"/>
-      <c r="C13" s="57">
-        <f>SUM(C8:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="57">
-        <f>SUM(D8:D12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="55" t="inlineStr">
-        <is>
-          <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="n"/>
-      <c r="C14" s="33" t="n"/>
-      <c r="D14" s="33" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Уборка и снегоуборка</t>
-        </is>
-      </c>
-      <c r="B15" s="28" t="inlineStr">
-        <is>
-          <t>общая площадь × норматив × 12 мес</t>
-        </is>
-      </c>
-      <c r="C15" s="58">
-        <f>$D$4*Нормативы!E5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="58">
-        <f>$D$4*Нормативы!F5*12/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Озеленение и полив</t>
-        </is>
-      </c>
-      <c r="B16" s="28" t="inlineStr">
-        <is>
-          <t>озеленение × норматив × 7 мес (апр–окт)</t>
-        </is>
-      </c>
-      <c r="C16" s="58">
-        <f>$D$3*Нормативы!E6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="58">
-        <f>$D$3*Нормативы!F6*7/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Свет, электро, digital</t>
-        </is>
-      </c>
-      <c r="B17" s="28" t="inlineStr">
-        <is>
-          <t>общая площадь × годовой норматив</t>
-        </is>
-      </c>
-      <c r="C17" s="58">
-        <f>$D$4*Нормативы!E7/1000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="58">
-        <f>$D$4*Нормативы!F7/1000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Программа и маркетинг</t>
-        </is>
-      </c>
-      <c r="B18" s="28" t="inlineStr">
-        <is>
-          <t>число событий × цена события</t>
-        </is>
-      </c>
-      <c r="C18" s="58">
-        <f>Нормативы!E9*Нормативы!$C$16/1000</f>
-        <v/>
-      </c>
-      <c r="D18" s="58">
-        <f>Нормативы!F9*Нормативы!$D$16/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Координатор кластера</t>
-        </is>
-      </c>
-      <c r="B19" s="28" t="inlineStr">
-        <is>
-          <t>ставка × доля × 12 мес</t>
-        </is>
-      </c>
-      <c r="C19" s="58">
-        <f>Нормативы!$C$15*Нормативы!E8*12/1000</f>
-        <v/>
-      </c>
-      <c r="D19" s="58">
-        <f>Нормативы!$D$15*Нормативы!F8*12/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Ремфонд</t>
-        </is>
-      </c>
-      <c r="B20" s="28" t="inlineStr">
-        <is>
-          <t>% в год от активов на балансе + CAPEX активации</t>
-        </is>
-      </c>
-      <c r="C20" s="58">
-        <f>Нормативы!$C$17*($B$4+Нормативы!E12)</f>
-        <v/>
-      </c>
-      <c r="D20" s="58">
-        <f>Нормативы!$D$17*($B$4+Нормативы!F12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="59" t="inlineStr">
-        <is>
-          <t>OPEX, итого</t>
-        </is>
-      </c>
-      <c r="B21" s="46" t="n"/>
-      <c r="C21" s="60">
-        <f>SUM(C15:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="60">
-        <f>SUM(D15:D20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="55" t="inlineStr">
-        <is>
-          <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
-        </is>
-      </c>
-      <c r="B23" s="33" t="n"/>
-      <c r="C23" s="33" t="n"/>
-      <c r="D23" s="33" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Консервативный сценарий</t>
-        </is>
-      </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>низ доходов / верх расходов</t>
-        </is>
-      </c>
-      <c r="C24" s="61">
-        <f>IFERROR(C13/D21,0)</f>
-        <v/>
-      </c>
-      <c r="D24" s="33" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>По середине вилок</t>
-        </is>
-      </c>
-      <c r="B25" s="28" t="inlineStr">
-        <is>
-          <t>средние значения обеих вилок</t>
-        </is>
-      </c>
-      <c r="C25" s="61">
-        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
-        <v/>
-      </c>
-      <c r="D25" s="33" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Оптимистичный сценарий</t>
-        </is>
-      </c>
-      <c r="B26" s="28" t="inlineStr">
-        <is>
-          <t>верх доходов / низ расходов</t>
-        </is>
-      </c>
-      <c r="C26" s="61">
-        <f>IFERROR(D13/C21,0)</f>
-        <v/>
-      </c>
-      <c r="D26" s="33" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="62" t="inlineStr">
-        <is>
-          <t>Целевой коридор пилота</t>
-        </is>
-      </c>
-      <c r="B27" s="33" t="n"/>
-      <c r="C27" s="63" t="inlineStr">
-        <is>
-          <t>40–70%</t>
-        </is>
-      </c>
-      <c r="D27" s="33" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="55" t="inlineStr">
-        <is>
-          <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
-        </is>
-      </c>
-      <c r="B29" s="33" t="n"/>
-      <c r="C29" s="33" t="n"/>
-      <c r="D29" s="33" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="64" t="inlineStr">
-        <is>
-          <t>• Справка по активам Хедлайнера получена, суммы внесены в лист «Активы»</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="64" t="inlineStr">
-        <is>
-          <t>• Якорь-павильон заполнен с мая по сентябрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="64" t="inlineStr">
-        <is>
-          <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="64" t="inlineStr">
-        <is>
-          <t>• Вечерние слоты секций выкуплены</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36"/>
-  </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A35:D36"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A14:D14"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$36</formula1>
+      <formula1>=Объекты!$B$4:$B$37</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4669,50 +4904,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="49" t="inlineStr">
-        <is>
-          <t>Финмодель Т3 · Сквер / плейхаб</t>
+      <c r="A1" s="58" t="inlineStr">
+        <is>
+          <t>Финмодель Т2 · Активная аллея</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="51" t="inlineStr">
-        <is>
-          <t>Сквер Авеню 5</t>
-        </is>
-      </c>
-      <c r="C3" s="52" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>Пилотный кластер: Хедлайнер + Flora + Аура</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="53">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+      <c r="D3" s="62">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="59" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="54">
-        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
+      <c r="B4" s="63">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($B$3,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="53">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+      <c r="D4" s="62">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -4739,7 +4974,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="55" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -4751,111 +4986,111 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Две НТО-точки</t>
+          <t>НТО-якорь: кофе-павильон</t>
         </is>
       </c>
       <c r="B8" s="28" t="inlineStr">
         <is>
-          <t>кофе и выпечка: аренда + % оборота</t>
+          <t>аренда 120–250 тыс тг/мес + 2–5% оборота</t>
         </is>
       </c>
       <c r="C8" s="35" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="D8" s="35" t="n">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Каток: прокат и билеты</t>
+          <t>Ярмарка выходного дня</t>
         </is>
       </c>
       <c r="B9" s="28" t="inlineStr">
         <is>
-          <t>компактный контур, 120–160 дней</t>
+          <t>12–16 ярмарок, 15–25 мест по 3–5 тыс тг</t>
         </is>
       </c>
       <c r="C9" s="35" t="n">
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="D9" s="35" t="n">
-        <v>3.5</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Событийная аренда</t>
+          <t>Секции и кикшеринг</t>
         </is>
       </c>
       <c r="B10" s="28" t="inlineStr">
         <is>
-          <t>10–18 частных и корпоративных событий</t>
+          <t>слоты тренерам + rev-share операторов</t>
         </is>
       </c>
       <c r="C10" s="35" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="D10" s="35" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Ярмарки, маркеты, секции</t>
+          <t>Digital-экран и реклама</t>
         </is>
       </c>
       <c r="B11" s="28" t="inlineStr">
         <is>
-          <t>круглогодичный календарь</t>
+          <t>при подходящем юрстатусе земли</t>
         </is>
       </c>
       <c r="C11" s="35" t="n">
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Спонсор года и реклама</t>
+          <t>Спонсорство объектов</t>
         </is>
       </c>
       <c r="B12" s="28" t="inlineStr">
         <is>
-          <t>один якорный партнёр + экран</t>
+          <t>воркаут, клумбы, скамейки</t>
         </is>
       </c>
       <c r="C12" s="35" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>3.7</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="56" t="inlineStr">
+      <c r="A13" s="65" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
       <c r="B13" s="46" t="n"/>
-      <c r="C13" s="57">
+      <c r="C13" s="66">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="66">
         <f>SUM(D8:D12)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="55" t="inlineStr">
+      <c r="A14" s="64" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -4875,12 +5110,12 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C15" s="58">
-        <f>$D$4*Нормативы!G5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="58">
-        <f>$D$4*Нормативы!H5*12/1000000</f>
+      <c r="C15" s="67">
+        <f>$D$4*Нормативы!E5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="67">
+        <f>$D$4*Нормативы!F5*12/1000000</f>
         <v/>
       </c>
     </row>
@@ -4895,12 +5130,12 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C16" s="58">
-        <f>$D$3*Нормативы!G6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="58">
-        <f>$D$3*Нормативы!H6*7/1000000</f>
+      <c r="C16" s="67">
+        <f>$D$3*Нормативы!E6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="67">
+        <f>$D$3*Нормативы!F6*7/1000000</f>
         <v/>
       </c>
     </row>
@@ -4915,58 +5150,548 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C17" s="58">
-        <f>$D$4*Нормативы!G7/1000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="58">
-        <f>$D$4*Нормативы!H7/1000000</f>
+      <c r="C17" s="67">
+        <f>$D$4*Нормативы!E7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="67">
+        <f>$D$4*Нормативы!F7/1000000</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Зимний пакет</t>
+          <t>Программа и маркетинг</t>
         </is>
       </c>
       <c r="B18" s="28" t="inlineStr">
         <is>
-          <t>норматив, млн тг/год</t>
-        </is>
-      </c>
-      <c r="C18" s="58">
-        <f>Нормативы!G10</f>
-        <v/>
-      </c>
-      <c r="D18" s="58">
-        <f>Нормативы!H10</f>
+          <t>число событий × цена события</t>
+        </is>
+      </c>
+      <c r="C18" s="67">
+        <f>Нормативы!E9*Нормативы!$C$16/1000</f>
+        <v/>
+      </c>
+      <c r="D18" s="67">
+        <f>Нормативы!F9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Программа и маркетинг</t>
+          <t>Координатор кластера</t>
         </is>
       </c>
       <c r="B19" s="28" t="inlineStr">
         <is>
-          <t>число событий × цена события</t>
-        </is>
-      </c>
-      <c r="C19" s="58">
-        <f>Нормативы!G9*Нормативы!$C$16/1000</f>
-        <v/>
-      </c>
-      <c r="D19" s="58">
-        <f>Нормативы!H9*Нормативы!$D$16/1000</f>
+          <t>ставка × доля × 12 мес</t>
+        </is>
+      </c>
+      <c r="C19" s="67">
+        <f>Нормативы!$C$15*Нормативы!E8*12/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="67">
+        <f>Нормативы!$D$15*Нормативы!F8*12/1000</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>Ремфонд</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>% в год от активов на балансе + CAPEX активации</t>
+        </is>
+      </c>
+      <c r="C20" s="67">
+        <f>Нормативы!$C$17*($B$4+Нормативы!E12)</f>
+        <v/>
+      </c>
+      <c r="D20" s="67">
+        <f>Нормативы!$D$17*($B$4+Нормативы!F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="68" t="inlineStr">
+        <is>
+          <t>OPEX, итого</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="n"/>
+      <c r="C21" s="69">
+        <f>SUM(C15:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="69">
+        <f>SUM(D15:D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="64" t="inlineStr">
+        <is>
+          <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="n"/>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Консервативный сценарий</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>низ доходов / верх расходов</t>
+        </is>
+      </c>
+      <c r="C24" s="70">
+        <f>IFERROR(C13/D21,0)</f>
+        <v/>
+      </c>
+      <c r="D24" s="33" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>По середине вилок</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>средние значения обеих вилок</t>
+        </is>
+      </c>
+      <c r="C25" s="70">
+        <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C21:D21),0)</f>
+        <v/>
+      </c>
+      <c r="D25" s="33" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Оптимистичный сценарий</t>
+        </is>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>верх доходов / низ расходов</t>
+        </is>
+      </c>
+      <c r="C26" s="70">
+        <f>IFERROR(D13/C21,0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="33" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="71" t="inlineStr">
+        <is>
+          <t>Целевой коридор пилота</t>
+        </is>
+      </c>
+      <c r="B27" s="33" t="n"/>
+      <c r="C27" s="72" t="inlineStr">
+        <is>
+          <t>40–70%</t>
+        </is>
+      </c>
+      <c r="D27" s="33" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="64" t="inlineStr">
+        <is>
+          <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
+        </is>
+      </c>
+      <c r="B29" s="33" t="n"/>
+      <c r="C29" s="33" t="n"/>
+      <c r="D29" s="33" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="73" t="inlineStr">
+        <is>
+          <t>• Справка по активам Хедлайнера получена, суммы внесены в лист «Активы»</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="73" t="inlineStr">
+        <is>
+          <t>• Якорь-павильон заполнен с мая по сентябрь</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="73" t="inlineStr">
+        <is>
+          <t>• Ярмарка стала привычкой района: 12+ за сезон</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="73" t="inlineStr">
+        <is>
+          <t>• Вечерние слоты секций выкуплены</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A35:D36"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=Объекты!$B$4:$B$37</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="58" t="inlineStr">
+        <is>
+          <t>Финмодель Т3 · Сквер / плейхаб</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="59" t="inlineStr">
+        <is>
+          <t>Объект (выберите из списка):</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>Сквер Авеню 5</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>Озеленение, м²:</t>
+        </is>
+      </c>
+      <c r="D3" s="62">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>Активы на балансе, млн тг:</t>
+        </is>
+      </c>
+      <c r="B4" s="63">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($B$3,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
+        <is>
+          <t>Общая площадь, м²:</t>
+        </is>
+      </c>
+      <c r="D4" s="62">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Как считаем / привязка</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Мин, млн тг/год</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Макс, млн тг/год</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
+        <is>
+          <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Две НТО-точки</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>кофе и выпечка: аренда + % оборота</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D8" s="35" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Каток: прокат и билеты</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>компактный контур, 120–160 дней</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Событийная аренда</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>10–18 частных и корпоративных событий</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Ярмарки, маркеты, секции</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>круглогодичный календарь</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D11" s="35" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Спонсор года и реклама</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>один якорный партнёр + экран</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="65" t="inlineStr">
+        <is>
+          <t>Доходы, итого</t>
+        </is>
+      </c>
+      <c r="B13" s="46" t="n"/>
+      <c r="C13" s="66">
+        <f>SUM(C8:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="66">
+        <f>SUM(D8:D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="64" t="inlineStr">
+        <is>
+          <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Уборка и снегоуборка</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>общая площадь × норматив × 12 мес</t>
+        </is>
+      </c>
+      <c r="C15" s="67">
+        <f>$D$4*Нормативы!G5*12/1000000</f>
+        <v/>
+      </c>
+      <c r="D15" s="67">
+        <f>$D$4*Нормативы!H5*12/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Озеленение и полив</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>озеленение × норматив × 7 мес (апр–окт)</t>
+        </is>
+      </c>
+      <c r="C16" s="67">
+        <f>$D$3*Нормативы!G6*7/1000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="67">
+        <f>$D$3*Нормативы!H6*7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Свет, электро, digital</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>общая площадь × годовой норматив</t>
+        </is>
+      </c>
+      <c r="C17" s="67">
+        <f>$D$4*Нормативы!G7/1000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="67">
+        <f>$D$4*Нормативы!H7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Зимний пакет</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>норматив, млн тг/год</t>
+        </is>
+      </c>
+      <c r="C18" s="67">
+        <f>Нормативы!G10</f>
+        <v/>
+      </c>
+      <c r="D18" s="67">
+        <f>Нормативы!H10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Программа и маркетинг</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>число событий × цена события</t>
+        </is>
+      </c>
+      <c r="C19" s="67">
+        <f>Нормативы!G9*Нормативы!$C$16/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="67">
+        <f>Нормативы!H9*Нормативы!$D$16/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t>Координатор кластера</t>
         </is>
       </c>
@@ -4975,11 +5700,11 @@
           <t>ставка × доля × 12 мес</t>
         </is>
       </c>
-      <c r="C20" s="58">
+      <c r="C20" s="67">
         <f>Нормативы!$C$15*Нормативы!G8*12/1000</f>
         <v/>
       </c>
-      <c r="D20" s="58">
+      <c r="D20" s="67">
         <f>Нормативы!$D$15*Нормативы!H8*12/1000</f>
         <v/>
       </c>
@@ -4995,33 +5720,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C21" s="58">
+      <c r="C21" s="67">
         <f>Нормативы!$C$17*($B$4+Нормативы!G12)</f>
         <v/>
       </c>
-      <c r="D21" s="58">
+      <c r="D21" s="67">
         <f>Нормативы!$D$17*($B$4+Нормативы!H12)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="59" t="inlineStr">
+      <c r="A22" s="68" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
       <c r="B22" s="46" t="n"/>
-      <c r="C22" s="60">
+      <c r="C22" s="69">
         <f>SUM(C15:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="60">
+      <c r="D22" s="69">
         <f>SUM(D15:D21)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="55" t="inlineStr">
+      <c r="A24" s="64" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -5041,7 +5766,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C25" s="61">
+      <c r="C25" s="70">
         <f>IFERROR(C13/D22,0)</f>
         <v/>
       </c>
@@ -5058,7 +5783,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C26" s="61">
+      <c r="C26" s="70">
         <f>IFERROR(AVERAGE(C13:D13)/AVERAGE(C22:D22),0)</f>
         <v/>
       </c>
@@ -5075,20 +5800,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C27" s="61">
+      <c r="C27" s="70">
         <f>IFERROR(D13/C22,0)</f>
         <v/>
       </c>
       <c r="D27" s="33" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="62" t="inlineStr">
+      <c r="A28" s="71" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B28" s="33" t="n"/>
-      <c r="C28" s="63" t="inlineStr">
+      <c r="C28" s="72" t="inlineStr">
         <is>
           <t>70–100%</t>
         </is>
@@ -5096,7 +5821,7 @@
       <c r="D28" s="33" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="55" t="inlineStr">
+      <c r="A30" s="64" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -5106,21 +5831,21 @@
       <c r="D30" s="33" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="64" t="inlineStr">
+      <c r="A31" s="73" t="inlineStr">
         <is>
           <t>• Каток отработал первую зиму без простоев</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="64" t="inlineStr">
+      <c r="A32" s="73" t="inlineStr">
         <is>
           <t>• Заявок на события больше, чем слотов</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="64" t="inlineStr">
+      <c r="A33" s="73" t="inlineStr">
         <is>
           <t>• Спонсор года подписан до старта сезона</t>
         </is>
@@ -5148,14 +5873,14 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$36</formula1>
+      <formula1>=Объекты!$B$4:$B$37</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5171,50 +5896,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Финмодель Т4 · Парк по ГЧП (BTO)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>Объект (выберите из списка):</t>
         </is>
       </c>
-      <c r="B3" s="51" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>Sphere Park</t>
         </is>
       </c>
-      <c r="C3" s="52" t="inlineStr">
+      <c r="C3" s="61" t="inlineStr">
         <is>
           <t>Озеленение, м²:</t>
         </is>
       </c>
-      <c r="D3" s="53">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+      <c r="D3" s="62">
+        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="59" t="inlineStr">
         <is>
           <t>Активы на балансе, млн тг:</t>
         </is>
       </c>
-      <c r="B4" s="54">
-        <f>IFERROR(INDEX(Активы!$J$4:$J$16,MATCH($B$3,Активы!$A$4:$A$16,0)),0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
+      <c r="B4" s="63">
+        <f>IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($B$3,Активы!$A$4:$A$17,0)),0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>Общая площадь, м²:</t>
         </is>
       </c>
-      <c r="D4" s="53">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$36,MATCH($B$3,Объекты!$B$4:$B$36,0)),0)</f>
+      <c r="D4" s="62">
+        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($B$3,Объекты!$B$4:$B$37,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -5241,7 +5966,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="55" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>ДОХОДЫ (вилки: зависят от программы, не от площади)</t>
         </is>
@@ -5359,23 +6084,23 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="56" t="inlineStr">
+      <c r="A14" s="65" t="inlineStr">
         <is>
           <t>Доходы, итого</t>
         </is>
       </c>
       <c r="B14" s="46" t="n"/>
-      <c r="C14" s="57">
+      <c r="C14" s="66">
         <f>SUM(C8:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="57">
+      <c r="D14" s="66">
         <f>SUM(D8:D13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="55" t="inlineStr">
+      <c r="A15" s="64" t="inlineStr">
         <is>
           <t>РАСХОДЫ (OPEX): формулы «площадь × нормативы»</t>
         </is>
@@ -5395,11 +6120,11 @@
           <t>общая площадь × норматив × 12 мес</t>
         </is>
       </c>
-      <c r="C16" s="58">
+      <c r="C16" s="67">
         <f>$D$4*Нормативы!I5*12/1000000</f>
         <v/>
       </c>
-      <c r="D16" s="58">
+      <c r="D16" s="67">
         <f>$D$4*Нормативы!J5*12/1000000</f>
         <v/>
       </c>
@@ -5415,11 +6140,11 @@
           <t>озеленение × норматив × 7 мес (апр–окт)</t>
         </is>
       </c>
-      <c r="C17" s="58">
+      <c r="C17" s="67">
         <f>$D$3*Нормативы!I6*7/1000000</f>
         <v/>
       </c>
-      <c r="D17" s="58">
+      <c r="D17" s="67">
         <f>$D$3*Нормативы!J6*7/1000000</f>
         <v/>
       </c>
@@ -5435,11 +6160,11 @@
           <t>общая площадь × годовой норматив</t>
         </is>
       </c>
-      <c r="C18" s="58">
+      <c r="C18" s="67">
         <f>$D$4*Нормативы!I7/1000000</f>
         <v/>
       </c>
-      <c r="D18" s="58">
+      <c r="D18" s="67">
         <f>$D$4*Нормативы!J7/1000000</f>
         <v/>
       </c>
@@ -5455,11 +6180,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C19" s="58">
+      <c r="C19" s="67">
         <f>Нормативы!I10</f>
         <v/>
       </c>
-      <c r="D19" s="58">
+      <c r="D19" s="67">
         <f>Нормативы!J10</f>
         <v/>
       </c>
@@ -5475,11 +6200,11 @@
           <t>число событий × цена события</t>
         </is>
       </c>
-      <c r="C20" s="58">
+      <c r="C20" s="67">
         <f>Нормативы!I9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="D20" s="58">
+      <c r="D20" s="67">
         <f>Нормативы!J9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
@@ -5495,11 +6220,11 @@
           <t>норматив, млн тг/год</t>
         </is>
       </c>
-      <c r="C21" s="58">
+      <c r="C21" s="67">
         <f>Нормативы!I11</f>
         <v/>
       </c>
-      <c r="D21" s="58">
+      <c r="D21" s="67">
         <f>Нормативы!J11</f>
         <v/>
       </c>
@@ -5515,33 +6240,33 @@
           <t>% в год от активов на балансе + CAPEX активации</t>
         </is>
       </c>
-      <c r="C22" s="58">
+      <c r="C22" s="67">
         <f>Нормативы!$C$17*($B$4+Нормативы!I12)</f>
         <v/>
       </c>
-      <c r="D22" s="58">
+      <c r="D22" s="67">
         <f>Нормативы!$D$17*($B$4+Нормативы!J12)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="59" t="inlineStr">
+      <c r="A23" s="68" t="inlineStr">
         <is>
           <t>OPEX, итого</t>
         </is>
       </c>
       <c r="B23" s="46" t="n"/>
-      <c r="C23" s="60">
+      <c r="C23" s="69">
         <f>SUM(C16:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="60">
+      <c r="D23" s="69">
         <f>SUM(D16:D22)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="55" t="inlineStr">
+      <c r="A25" s="64" t="inlineStr">
         <is>
           <t>ПОКРЫТИЕ OPEX ДОХОДАМИ</t>
         </is>
@@ -5561,7 +6286,7 @@
           <t>низ доходов / верх расходов</t>
         </is>
       </c>
-      <c r="C26" s="61">
+      <c r="C26" s="70">
         <f>IFERROR(C14/D23,0)</f>
         <v/>
       </c>
@@ -5578,7 +6303,7 @@
           <t>средние значения обеих вилок</t>
         </is>
       </c>
-      <c r="C27" s="61">
+      <c r="C27" s="70">
         <f>IFERROR(AVERAGE(C14:D14)/AVERAGE(C23:D23),0)</f>
         <v/>
       </c>
@@ -5595,20 +6320,20 @@
           <t>верх доходов / низ расходов</t>
         </is>
       </c>
-      <c r="C28" s="61">
+      <c r="C28" s="70">
         <f>IFERROR(D14/C23,0)</f>
         <v/>
       </c>
       <c r="D28" s="33" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr">
+      <c r="A29" s="71" t="inlineStr">
         <is>
           <t>Целевой коридор пилота</t>
         </is>
       </c>
       <c r="B29" s="33" t="n"/>
-      <c r="C29" s="63" t="inlineStr">
+      <c r="C29" s="72" t="inlineStr">
         <is>
           <t>80–110%</t>
         </is>
@@ -5616,7 +6341,7 @@
       <c r="D29" s="33" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="55" t="inlineStr">
+      <c r="A31" s="64" t="inlineStr">
         <is>
           <t>ЧТО ДОЛЖНО СОЙТИСЬ</t>
         </is>
@@ -5626,35 +6351,35 @@
       <c r="D31" s="33" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="64" t="inlineStr">
+      <c r="A32" s="73" t="inlineStr">
         <is>
           <t>• Ремфонд и капремонт сидят в компенсации эксплуатации (BTO), в OPEX не дублируются</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="64" t="inlineStr">
+      <c r="A33" s="73" t="inlineStr">
         <is>
           <t>• ГЧП-договор подписан, компенсация в бюджете МИО</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="64" t="inlineStr">
+      <c r="A34" s="73" t="inlineStr">
         <is>
           <t>• Каток и события дотягивают покрытие до 100%+</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="64" t="inlineStr">
+      <c r="A35" s="73" t="inlineStr">
         <is>
           <t>• Стандарт содержания выше городского бенчмарка</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="64" t="inlineStr">
+      <c r="A36" s="73" t="inlineStr">
         <is>
           <t>• CAPEX ~2,2 млрд тг компенсируется бюджетом МИО отдельно (2026–2031) — в операционную модель не входит</t>
         </is>
@@ -5684,7 +6409,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Объекты!$B$4:$B$36</formula1>
+      <formula1>=Объекты!$B$4:$B$37</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Set pilot pair to Grand Turan and Nexpo Union
Deck: rebased on the client-edited 20-slide version. Shortlist,
perimeter, assets and roadmap slides now carry the two-pilot set;
cluster cards and their satellite crops replaced by a wide Grand Turan
contour and a Nexpo Union card noting the survey is still pending.

Workbook v7: pilot roles in the registry, Pilot Budget sheet rebuilt
for the two alleys with separate coordinator shares (10.5-17.4M KZT
per year), T2 sheet defaults to Grand Turan.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014o1yT6nCgffZ5H25q7THst
</commit_message>
<xml_diff>
--- a/docs/research/BIG-Life-finmodels-T1-T4.xlsx
+++ b/docs/research/BIG-Life-finmodels-T1-T4.xlsx
@@ -838,7 +838,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая — фактический обмер Google Earth для группы A (для незамеренных: озеленение × коэффициент). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Лист «Бюджет пилота» — годовое содержание выбранного периметра: Гранд Туран + кластер из четырёх. Жёлтые ячейки — редактируемые ставки.</t>
+          <t>Как пользоваться. На листах моделей выберите объект из выпадающего списка (лист «Объекты», 32 территории, шорт-лист отмечен «Да») — обе площади подтянутся сами: озеленение из реестра, общая — фактический обмер Google Earth для группы A (для незамеренных: озеленение × коэффициент). Уборка и свет считаются от общей площади, озеленение и полив — от зелёной. Лист «Активы» — балансовая стоимость по справкам застройщиков; ремфонд = 1–1,5% в год от активов и планового CAPEX активации. Лист «Бюджет пилота» — годовое содержание пилота: Гранд Туран и Nexpo Юнион. Жёлтые ячейки — редактируемые ставки.</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Т2 · Пилотный кластер</t>
+          <t>Т2 · Гранд Туран</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1413,7 +1413,7 @@
       <c r="A8" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Аура Аллея</t>
         </is>
@@ -1434,9 +1434,9 @@
       <c r="F8" s="17" t="n">
         <v>1415</v>
       </c>
-      <c r="G8" s="23" t="inlineStr">
-        <is>
-          <t>Пилот</t>
+      <c r="G8" s="21" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
@@ -1452,7 +1452,7 @@
       <c r="A9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Аллея Хедлайнер Эксклюзив</t>
         </is>
@@ -1473,9 +1473,9 @@
       <c r="F9" s="17" t="n">
         <v>4100</v>
       </c>
-      <c r="G9" s="23" t="inlineStr">
-        <is>
-          <t>Пилот</t>
+      <c r="G9" s="21" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
@@ -1530,7 +1530,7 @@
       <c r="A11" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 1</t>
         </is>
@@ -1551,9 +1551,9 @@
       <c r="F11" s="17" t="n">
         <v>1512</v>
       </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>Пилот</t>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
@@ -1569,7 +1569,7 @@
       <c r="A12" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>Аллея ЖК Flora 2</t>
         </is>
@@ -1590,9 +1590,9 @@
       <c r="F12" s="17" t="n">
         <v>1210</v>
       </c>
-      <c r="G12" s="23" t="inlineStr">
-        <is>
-          <t>Пилот</t>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
@@ -1941,7 +1941,7 @@
       <c r="A21" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>Аллея Nexpo Юнион</t>
         </is>
@@ -1962,9 +1962,9 @@
       <c r="F21" s="26" t="n">
         <v>4200</v>
       </c>
-      <c r="G21" s="21" t="inlineStr">
-        <is>
-          <t>Да</t>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>Пилот</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">
@@ -2609,7 +2609,7 @@
       <c r="A37" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Пилотный кластер: Хедлайнер + Flora + Аура</t>
         </is>
@@ -2631,9 +2631,9 @@
         <f>F8+F9+F11+F12</f>
         <v/>
       </c>
-      <c r="G37" s="23" t="inlineStr">
-        <is>
-          <t>Пилот</t>
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" s="16" t="inlineStr">
@@ -3868,7 +3868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3897,7 +3897,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Содержание as-is: уборка и свет от общей площади (обмер), озеленение от зелёной, ремфонд от активов на балансе, координация по долям ставок. Все ставки — лист «Нормативы». Программа активации — справочно, отдельной строкой.</t>
+          <t>Пилотный периметр: Гранд Туран и Nexpo Юнион. Уборка и свет от общей площади, озеленение от зелёной, ремфонд от активов на балансе, координация по долям ставок. Все ставки — лист «Нормативы». Программа активации — справочно, отдельной строкой.</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4036,7 @@
     <row r="6">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>Аллея Хедлайнер Эксклюзив</t>
+          <t>Аллея Nexpo Юнион</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
@@ -4094,196 +4094,72 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>Аллея ЖК Flora 1</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Т1</t>
-        </is>
-      </c>
-      <c r="C7" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A7,Объекты!$B$4:$B$37,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D7" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A7,Объекты!$B$4:$B$37,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E7" s="51">
-        <f>$D7*Нормативы!C5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="F7" s="51">
-        <f>$D7*Нормативы!D5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="G7" s="51">
-        <f>$C7*Нормативы!C6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="H7" s="51">
-        <f>$C7*Нормативы!D6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="I7" s="51">
-        <f>$D7*Нормативы!C7/1000000</f>
-        <v/>
-      </c>
-      <c r="J7" s="51">
-        <f>$D7*Нормативы!D7/1000000</f>
-        <v/>
-      </c>
-      <c r="K7" s="51">
-        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A7,Активы!$A$4:$A$17,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="51">
-        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A7,Активы!$A$4:$A$17,0)),0)</f>
-        <v/>
-      </c>
-      <c r="M7" s="39">
-        <f>E7+G7+I7+K7</f>
-        <v/>
-      </c>
-      <c r="N7" s="39">
-        <f>F7+H7+J7+L7</f>
+      <c r="A7" s="52" t="inlineStr">
+        <is>
+          <t>Координатор Гранд Турана (доля Т2)</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="inlineStr">
+        <is>
+          <t>0,33 ставки на объект</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="33" t="n"/>
+      <c r="F7" s="33" t="n"/>
+      <c r="G7" s="33" t="n"/>
+      <c r="H7" s="33" t="n"/>
+      <c r="I7" s="33" t="n"/>
+      <c r="J7" s="33" t="n"/>
+      <c r="K7" s="33" t="n"/>
+      <c r="L7" s="33" t="n"/>
+      <c r="M7" s="38">
+        <f>Нормативы!E8*Нормативы!$C$15*12/1000</f>
+        <v/>
+      </c>
+      <c r="N7" s="38">
+        <f>Нормативы!F8*Нормативы!$D$15*12/1000</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
-        <is>
-          <t>Аллея ЖК Flora 2</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>Т1</t>
-        </is>
-      </c>
-      <c r="C8" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A8,Объекты!$B$4:$B$37,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A8,Объекты!$B$4:$B$37,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E8" s="51">
-        <f>$D8*Нормативы!C5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="F8" s="51">
-        <f>$D8*Нормативы!D5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="G8" s="51">
-        <f>$C8*Нормативы!C6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="H8" s="51">
-        <f>$C8*Нормативы!D6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="I8" s="51">
-        <f>$D8*Нормативы!C7/1000000</f>
-        <v/>
-      </c>
-      <c r="J8" s="51">
-        <f>$D8*Нормативы!D7/1000000</f>
-        <v/>
-      </c>
-      <c r="K8" s="51">
-        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A8,Активы!$A$4:$A$17,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="51">
-        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A8,Активы!$A$4:$A$17,0)),0)</f>
-        <v/>
-      </c>
-      <c r="M8" s="39">
-        <f>E8+G8+I8+K8</f>
-        <v/>
-      </c>
-      <c r="N8" s="39">
-        <f>F8+H8+J8+L8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="22" t="inlineStr">
-        <is>
-          <t>Аура Аллея</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>Т1</t>
-        </is>
-      </c>
-      <c r="C9" s="18">
-        <f>IFERROR(INDEX(Объекты!$E$4:$E$37,MATCH($A9,Объекты!$B$4:$B$37,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>IFERROR(INDEX(Объекты!$F$4:$F$37,MATCH($A9,Объекты!$B$4:$B$37,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E9" s="51">
-        <f>$D9*Нормативы!C5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="F9" s="51">
-        <f>$D9*Нормативы!D5*12/1000000</f>
-        <v/>
-      </c>
-      <c r="G9" s="51">
-        <f>$C9*Нормативы!C6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="H9" s="51">
-        <f>$C9*Нормативы!D6*7/1000000</f>
-        <v/>
-      </c>
-      <c r="I9" s="51">
-        <f>$D9*Нормативы!C7/1000000</f>
-        <v/>
-      </c>
-      <c r="J9" s="51">
-        <f>$D9*Нормативы!D7/1000000</f>
-        <v/>
-      </c>
-      <c r="K9" s="51">
-        <f>Нормативы!$C$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A9,Активы!$A$4:$A$17,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="51">
-        <f>Нормативы!$D$17*IFERROR(INDEX(Активы!$J$4:$J$17,MATCH($A9,Активы!$A$4:$A$17,0)),0)</f>
-        <v/>
-      </c>
-      <c r="M9" s="39">
-        <f>E9+G9+I9+K9</f>
-        <v/>
-      </c>
-      <c r="N9" s="39">
-        <f>F9+H9+J9+L9</f>
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>Координатор Nexpo Юниона (доля Т2)</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>0,33 ставки; при общем координаторе на два контура ставка складывается</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="33" t="n"/>
+      <c r="G8" s="33" t="n"/>
+      <c r="H8" s="33" t="n"/>
+      <c r="I8" s="33" t="n"/>
+      <c r="J8" s="33" t="n"/>
+      <c r="K8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
+      <c r="M8" s="38">
+        <f>Нормативы!E8*Нормативы!$C$15*12/1000</f>
+        <v/>
+      </c>
+      <c r="N8" s="38">
+        <f>Нормативы!F8*Нормативы!$D$15*12/1000</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="52" t="inlineStr">
-        <is>
-          <t>Координатор кластера (сумма долей: Т2 + 3 × Т1)</t>
-        </is>
-      </c>
-      <c r="B10" s="53" t="inlineStr">
-        <is>
-          <t>один координатор на четыре аллеи: 0,33 + 3 × 0,20 = 0,93 ставки</t>
-        </is>
-      </c>
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Гранд Туран, итого</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="n"/>
       <c r="C10" s="33" t="n"/>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n"/>
@@ -4294,26 +4170,22 @@
       <c r="J10" s="33" t="n"/>
       <c r="K10" s="33" t="n"/>
       <c r="L10" s="33" t="n"/>
-      <c r="M10" s="38">
-        <f>(Нормативы!E8+3*Нормативы!C8)*Нормативы!$C$15*12/1000</f>
-        <v/>
-      </c>
-      <c r="N10" s="38">
-        <f>(Нормативы!F8+3*Нормативы!D8)*Нормативы!$D$15*12/1000</f>
+      <c r="M10" s="55">
+        <f>M5+M7</f>
+        <v/>
+      </c>
+      <c r="N10" s="55">
+        <f>N5+N7</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="52" t="inlineStr">
-        <is>
-          <t>Координатор Гранд Турана (доля Т2)</t>
-        </is>
-      </c>
-      <c r="B11" s="53" t="inlineStr">
-        <is>
-          <t>0,33 ставки; при расширении Управления 4 станет кластерным</t>
-        </is>
-      </c>
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t>Nexpo Юнион, итого</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="n"/>
       <c r="C11" s="33" t="n"/>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n"/>
@@ -4324,48 +4196,52 @@
       <c r="J11" s="33" t="n"/>
       <c r="K11" s="33" t="n"/>
       <c r="L11" s="33" t="n"/>
-      <c r="M11" s="38">
-        <f>Нормативы!E8*Нормативы!$C$15*12/1000</f>
-        <v/>
-      </c>
-      <c r="N11" s="38">
-        <f>Нормативы!F8*Нормативы!$D$15*12/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="54" t="inlineStr">
-        <is>
-          <t>Кластер (Хедлайнер + Flora 1, 2 + Аура), итого</t>
-        </is>
-      </c>
-      <c r="B13" s="46" t="n"/>
-      <c r="C13" s="33" t="n"/>
-      <c r="D13" s="33" t="n"/>
-      <c r="E13" s="33" t="n"/>
-      <c r="F13" s="33" t="n"/>
-      <c r="G13" s="33" t="n"/>
-      <c r="H13" s="33" t="n"/>
-      <c r="I13" s="33" t="n"/>
-      <c r="J13" s="33" t="n"/>
-      <c r="K13" s="33" t="n"/>
-      <c r="L13" s="33" t="n"/>
-      <c r="M13" s="55">
-        <f>M6+M7+M8+M9+M10</f>
-        <v/>
-      </c>
-      <c r="N13" s="55">
-        <f>N6+N7+N8+N9+N10</f>
+      <c r="M11" s="55">
+        <f>M6+M8</f>
+        <v/>
+      </c>
+      <c r="N11" s="55">
+        <f>N6+N8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>ПИЛОТ: СОДЕРЖАНИЕ, ИТОГО</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="n"/>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="33" t="n"/>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="33" t="n"/>
+      <c r="I12" s="33" t="n"/>
+      <c r="J12" s="33" t="n"/>
+      <c r="K12" s="33" t="n"/>
+      <c r="L12" s="33" t="n"/>
+      <c r="M12" s="57">
+        <f>M10+M11</f>
+        <v/>
+      </c>
+      <c r="N12" s="57">
+        <f>N10+N11</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="54" t="inlineStr">
-        <is>
-          <t>Гранд Туран, итого</t>
-        </is>
-      </c>
-      <c r="B14" s="46" t="n"/>
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>Программа активации (справочно, два контура)</t>
+        </is>
+      </c>
+      <c r="B14" s="53" t="inlineStr">
+        <is>
+          <t>события по нормативу Т2 на каждый контур; это активация, в содержание не входит</t>
+        </is>
+      </c>
       <c r="C14" s="33" t="n"/>
       <c r="D14" s="33" t="n"/>
       <c r="E14" s="33" t="n"/>
@@ -4376,87 +4252,31 @@
       <c r="J14" s="33" t="n"/>
       <c r="K14" s="33" t="n"/>
       <c r="L14" s="33" t="n"/>
-      <c r="M14" s="55">
-        <f>M5+M11</f>
-        <v/>
-      </c>
-      <c r="N14" s="55">
-        <f>N5+N11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="56" t="inlineStr">
-        <is>
-          <t>ПИЛОТ: СОДЕРЖАНИЕ, ИТОГО</t>
-        </is>
-      </c>
-      <c r="B15" s="46" t="n"/>
-      <c r="C15" s="33" t="n"/>
-      <c r="D15" s="33" t="n"/>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="33" t="n"/>
-      <c r="G15" s="33" t="n"/>
-      <c r="H15" s="33" t="n"/>
-      <c r="I15" s="33" t="n"/>
-      <c r="J15" s="33" t="n"/>
-      <c r="K15" s="33" t="n"/>
-      <c r="L15" s="33" t="n"/>
-      <c r="M15" s="57">
-        <f>M13+M14</f>
-        <v/>
-      </c>
-      <c r="N15" s="57">
-        <f>N13+N14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="52" t="inlineStr">
-        <is>
-          <t>Программа активации (справочно, два контура)</t>
-        </is>
-      </c>
-      <c r="B17" s="53" t="inlineStr">
-        <is>
-          <t>события по нормативу Т2 на каждый контур; это активация, в содержание не входит</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="n"/>
-      <c r="D17" s="33" t="n"/>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="33" t="n"/>
-      <c r="G17" s="33" t="n"/>
-      <c r="H17" s="33" t="n"/>
-      <c r="I17" s="33" t="n"/>
-      <c r="J17" s="33" t="n"/>
-      <c r="K17" s="33" t="n"/>
-      <c r="L17" s="33" t="n"/>
-      <c r="M17" s="38">
+      <c r="M14" s="38">
         <f>2*Нормативы!E9*Нормативы!$C$16/1000</f>
         <v/>
       </c>
-      <c r="N17" s="38">
+      <c r="N14" s="38">
         <f>2*Нормативы!F9*Нормативы!$D$16/1000</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Ремфонд Хедлайнера сейчас 0: справка о балансовой стоимости запрошена — суммы добавятся в лист «Активы» и бюджет пересчитается. Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Nexpo Юнион не передан и сейчас не обслуживается: его содержание — новые деньги, а не перераспределение. Общая площадь оценочная, замер уточнит уборку и свет. Вилки планировочные, для защиты подхода. Точные ставки дадут факт BI Green и нулевой спринт (сентябрь–октябрь 2026); полная модель с помесячной сезонностью собирается на них в ноябре 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B7:L7"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="B10:L10"/>
-    <mergeCell ref="A19:N20"/>
-    <mergeCell ref="B17:L17"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A16:N17"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4918,7 +4738,7 @@
       </c>
       <c r="B3" s="60" t="inlineStr">
         <is>
-          <t>Пилотный кластер: Хедлайнер + Flora + Аура</t>
+          <t>Аллея Гранд Туран Комфорт</t>
         </is>
       </c>
       <c r="C3" s="61" t="inlineStr">

</xml_diff>